<commit_message>
- Added biokerosene inventory - Added new market for kerosene - Updated scenario file with new data for kerosene and mobility
</commit_message>
<xml_diff>
--- a/inventories/lci-Tr2050.xlsx
+++ b/inventories/lci-Tr2050.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engie-my.sharepoint.com/personal/db6421_engie_com/Documents/Documents/GitHub/ADEME_scenarios_premise_gas/inventories/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engie-my.sharepoint.com/personal/db6421_engie_com/Documents/Documents/Local_repo/ADEME_scenarios_premise_gas/inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1812" documentId="13_ncr:1_{6A9A1C53-53B4-4DAF-B82F-70FF83AECA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5960DED-332F-4C3B-BA33-6F8DDDE6C464}"/>
+  <xr:revisionPtr revIDLastSave="2075" documentId="13_ncr:1_{6A9A1C53-53B4-4DAF-B82F-70FF83AECA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9248497-8342-4C26-BFBB-B93D2B6376E2}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="lci" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4115" uniqueCount="484">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4446" uniqueCount="516">
   <si>
     <t>Database</t>
   </si>
@@ -1488,6 +1488,102 @@
   </si>
   <si>
     <t>refused derived fuels</t>
+  </si>
+  <si>
+    <t>WCO pretreatment</t>
+  </si>
+  <si>
+    <t>Pretreated oils</t>
+  </si>
+  <si>
+    <t>Pretreated waste cooking oils. Source: "Uncovering the environmental performances of emerging candidates for Sustainable Aviation" (https://doi.org/10.48531/JBRU.CALMIP/D0PWA8)</t>
+  </si>
+  <si>
+    <t>heat and power co-generation, natural gas, conventional power plant, 100MW electrical</t>
+  </si>
+  <si>
+    <t>heat, district or industrial, natural gas</t>
+  </si>
+  <si>
+    <t>market for wastewater from vegetable oil refinery</t>
+  </si>
+  <si>
+    <t>wastewater from vegetable oil refinery</t>
+  </si>
+  <si>
+    <t>market for used vegetable cooking oil</t>
+  </si>
+  <si>
+    <t>used vegetable cooking oil</t>
+  </si>
+  <si>
+    <t>market for transport, freight, lorry &gt;32 metric ton, EURO5</t>
+  </si>
+  <si>
+    <t>transport, freight, lorry &gt;32 metric ton, EURO5</t>
+  </si>
+  <si>
+    <t>WCO purification</t>
+  </si>
+  <si>
+    <t>Purified oils</t>
+  </si>
+  <si>
+    <t>phosphoric acid, industrial grade, without water, in 85% solution state</t>
+  </si>
+  <si>
+    <t>market for phosphoric acid, industrial grade, without water, in 85% solution state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Purified waste cooking oils. Source: "Uncovering the environmental performances of emerging candidates for Sustainable Aviation" (https://doi.org/10.48531/JBRU.CALMIP/D0PWA8). The phospholipid produced in the activity is considered as a waste in this system model </t>
+  </si>
+  <si>
+    <t>treatment of wastewater, average, wastewater treatment</t>
+  </si>
+  <si>
+    <t>wastewater, average</t>
+  </si>
+  <si>
+    <t>WCO hydrogeoxygenation</t>
+  </si>
+  <si>
+    <t>Paraffin (hydrocarbon)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Uncovering the environmental performances of emerging candidates for Sustainable Aviation" (https://doi.org/10.48531/JBRU.CALMIP/D0PWA8). The phospholipid produced in the activity is considered as a waste in this system model </t>
+  </si>
+  <si>
+    <t>Hydrogen</t>
+  </si>
+  <si>
+    <t>Platinum-gamma alumina catalyst</t>
+  </si>
+  <si>
+    <t>market for platinum</t>
+  </si>
+  <si>
+    <t>platinum</t>
+  </si>
+  <si>
+    <t>nitric acid production, product in 50% solution state</t>
+  </si>
+  <si>
+    <t>nitric acid, without water, in 50% solution state</t>
+  </si>
+  <si>
+    <t>RER w/o RU</t>
+  </si>
+  <si>
+    <t>WCO hydrocracking</t>
+  </si>
+  <si>
+    <t>Biokerosene (HVO)</t>
+  </si>
+  <si>
+    <t>The original LCI is scaled to 1 kg based on the reported LHV of HEFA (44.46 MJ/kg)</t>
+  </si>
+  <si>
+    <t>IAI Area, EU27 &amp; EFTA</t>
   </si>
 </sst>
 </file>
@@ -1644,7 +1740,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -1727,6 +1823,9 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2011,7 +2110,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AH960"/>
+  <dimension ref="A1:AH1053"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="73.140625" customWidth="1"/>
@@ -26011,6 +26110,1461 @@
         <v>470</v>
       </c>
     </row>
+    <row r="961" spans="1:10">
+      <c r="A961" s="49"/>
+      <c r="B961" s="50"/>
+      <c r="C961" s="49"/>
+      <c r="D961" s="49"/>
+      <c r="E961" s="49"/>
+      <c r="F961" s="49"/>
+      <c r="G961" s="49"/>
+      <c r="H961" s="49"/>
+      <c r="I961" s="49"/>
+    </row>
+    <row r="962" spans="1:10" ht="15.75">
+      <c r="A962" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B962" s="43" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="963" spans="1:10">
+      <c r="A963" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B963" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="H963" s="55"/>
+    </row>
+    <row r="964" spans="1:10">
+      <c r="A964" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B964">
+        <v>1</v>
+      </c>
+      <c r="F964" s="13"/>
+      <c r="H964" s="13"/>
+    </row>
+    <row r="965" spans="1:10">
+      <c r="A965" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B965" t="s">
+        <v>485</v>
+      </c>
+      <c r="F965" s="13"/>
+      <c r="J965" s="56"/>
+    </row>
+    <row r="966" spans="1:10">
+      <c r="A966" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B966" t="s">
+        <v>59</v>
+      </c>
+      <c r="F966" s="20"/>
+    </row>
+    <row r="967" spans="1:10">
+      <c r="A967" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="B967" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="968" spans="1:10">
+      <c r="A968" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="B968" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="969" spans="1:10" ht="15.75">
+      <c r="A969" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B969" s="26"/>
+      <c r="C969" s="25"/>
+      <c r="D969" s="26"/>
+      <c r="E969" s="26"/>
+      <c r="F969" s="26"/>
+      <c r="G969" s="26"/>
+      <c r="H969" s="26"/>
+      <c r="I969" s="26"/>
+    </row>
+    <row r="970" spans="1:10">
+      <c r="A970" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B970" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="C970" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D970" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E970" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="F970" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="G970" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="H970" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="I970" s="24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="971" spans="1:10">
+      <c r="A971" s="31" t="s">
+        <v>484</v>
+      </c>
+      <c r="B971" s="31" t="s">
+        <v>485</v>
+      </c>
+      <c r="C971" s="26">
+        <v>1</v>
+      </c>
+      <c r="D971" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="F971" s="24"/>
+      <c r="G971" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H971" t="s">
+        <v>18</v>
+      </c>
+      <c r="I971" s="24"/>
+    </row>
+    <row r="972" spans="1:10">
+      <c r="A972" s="26" t="s">
+        <v>491</v>
+      </c>
+      <c r="B972" s="13" t="s">
+        <v>492</v>
+      </c>
+      <c r="C972" s="41">
+        <v>1.7509999999999999</v>
+      </c>
+      <c r="D972" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="G972" t="s">
+        <v>96</v>
+      </c>
+      <c r="H972" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="973" spans="1:10">
+      <c r="A973" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B973" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="C973">
+        <v>4.779502986996028E-2</v>
+      </c>
+      <c r="D973" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="G973" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="H973" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="974" spans="1:10">
+      <c r="A974" s="31" t="s">
+        <v>493</v>
+      </c>
+      <c r="B974" s="31" t="s">
+        <v>494</v>
+      </c>
+      <c r="C974">
+        <v>0.17513974577662458</v>
+      </c>
+      <c r="D974" s="26" t="s">
+        <v>158</v>
+      </c>
+      <c r="G974" t="s">
+        <v>36</v>
+      </c>
+      <c r="H974" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="975" spans="1:10">
+      <c r="A975" s="31" t="s">
+        <v>34</v>
+      </c>
+      <c r="B975" s="31" t="s">
+        <v>33</v>
+      </c>
+      <c r="C975">
+        <v>2.29E-2</v>
+      </c>
+      <c r="D975" t="s">
+        <v>19</v>
+      </c>
+      <c r="G975" t="s">
+        <v>28</v>
+      </c>
+      <c r="H975" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="976" spans="1:10">
+      <c r="A976" s="58" t="s">
+        <v>487</v>
+      </c>
+      <c r="B976" s="13" t="s">
+        <v>488</v>
+      </c>
+      <c r="C976">
+        <v>2E-3</v>
+      </c>
+      <c r="D976" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="G976" t="s">
+        <v>28</v>
+      </c>
+      <c r="H976" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="977" spans="1:10">
+      <c r="A977" t="s">
+        <v>489</v>
+      </c>
+      <c r="B977" s="13" t="s">
+        <v>490</v>
+      </c>
+      <c r="C977">
+        <v>-4.7795029869960301E-2</v>
+      </c>
+      <c r="D977" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="G977" t="s">
+        <v>96</v>
+      </c>
+      <c r="H977" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="978" spans="1:10">
+      <c r="A978" t="s">
+        <v>93</v>
+      </c>
+      <c r="C978" s="13">
+        <v>0.75139745776624589</v>
+      </c>
+      <c r="D978" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="E978" t="s">
+        <v>83</v>
+      </c>
+      <c r="F978" t="s">
+        <v>25</v>
+      </c>
+      <c r="G978" s="13"/>
+      <c r="H978" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="979" spans="1:10">
+      <c r="A979" s="49"/>
+      <c r="B979" s="50"/>
+      <c r="C979" s="49"/>
+      <c r="D979" s="49"/>
+      <c r="E979" s="49"/>
+      <c r="F979" s="49"/>
+      <c r="G979" s="49"/>
+      <c r="H979" s="49"/>
+      <c r="I979" s="49"/>
+    </row>
+    <row r="980" spans="1:10" ht="15.75">
+      <c r="A980" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B980" s="43" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="981" spans="1:10">
+      <c r="A981" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B981" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="H981" s="55"/>
+    </row>
+    <row r="982" spans="1:10">
+      <c r="A982" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B982">
+        <v>1</v>
+      </c>
+      <c r="F982" s="13"/>
+      <c r="H982" s="13"/>
+    </row>
+    <row r="983" spans="1:10">
+      <c r="A983" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B983" t="s">
+        <v>496</v>
+      </c>
+      <c r="F983" s="13"/>
+      <c r="J983" s="56"/>
+    </row>
+    <row r="984" spans="1:10">
+      <c r="A984" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B984" t="s">
+        <v>59</v>
+      </c>
+      <c r="F984" s="20"/>
+    </row>
+    <row r="985" spans="1:10">
+      <c r="A985" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="B985" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="986" spans="1:10">
+      <c r="A986" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="B986" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="987" spans="1:10" ht="15.75">
+      <c r="A987" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B987" s="26"/>
+      <c r="C987" s="25"/>
+      <c r="D987" s="26"/>
+      <c r="E987" s="26"/>
+      <c r="F987" s="26"/>
+      <c r="G987" s="26"/>
+      <c r="H987" s="26"/>
+      <c r="I987" s="26"/>
+    </row>
+    <row r="988" spans="1:10">
+      <c r="A988" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B988" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="C988" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D988" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E988" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="F988" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="G988" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="H988" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="I988" s="24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="989" spans="1:10">
+      <c r="A989" s="31" t="s">
+        <v>495</v>
+      </c>
+      <c r="B989" s="31" t="s">
+        <v>496</v>
+      </c>
+      <c r="C989" s="26">
+        <v>1</v>
+      </c>
+      <c r="D989" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="F989" s="24"/>
+      <c r="G989" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H989" t="s">
+        <v>18</v>
+      </c>
+      <c r="I989" s="24"/>
+    </row>
+    <row r="990" spans="1:10">
+      <c r="A990" s="31" t="s">
+        <v>484</v>
+      </c>
+      <c r="B990" s="31" t="s">
+        <v>485</v>
+      </c>
+      <c r="C990" s="41">
+        <v>1.02</v>
+      </c>
+      <c r="D990" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="G990" t="s">
+        <v>28</v>
+      </c>
+      <c r="H990" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="991" spans="1:10">
+      <c r="A991" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B991" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="C991">
+        <v>0.02</v>
+      </c>
+      <c r="D991" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="G991" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="H991" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="992" spans="1:10">
+      <c r="A992" s="31" t="s">
+        <v>498</v>
+      </c>
+      <c r="B992" s="31" t="s">
+        <v>497</v>
+      </c>
+      <c r="C992">
+        <v>7.6485543677358989E-4</v>
+      </c>
+      <c r="D992" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="G992" t="s">
+        <v>96</v>
+      </c>
+      <c r="H992" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="993" spans="1:10">
+      <c r="A993" s="31" t="s">
+        <v>233</v>
+      </c>
+      <c r="B993" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="C993">
+        <v>1.4532253298698207E-3</v>
+      </c>
+      <c r="D993" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="G993" t="s">
+        <v>96</v>
+      </c>
+      <c r="H993" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="994" spans="1:10">
+      <c r="A994" s="31" t="s">
+        <v>34</v>
+      </c>
+      <c r="B994" s="31" t="s">
+        <v>33</v>
+      </c>
+      <c r="C994">
+        <v>0.01</v>
+      </c>
+      <c r="D994" t="s">
+        <v>19</v>
+      </c>
+      <c r="G994" t="s">
+        <v>28</v>
+      </c>
+      <c r="H994" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="995" spans="1:10">
+      <c r="A995" t="s">
+        <v>500</v>
+      </c>
+      <c r="B995" s="13" t="s">
+        <v>501</v>
+      </c>
+      <c r="C995">
+        <v>-0.02</v>
+      </c>
+      <c r="D995" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="G995" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="H995" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="996" spans="1:10">
+      <c r="A996" s="49"/>
+      <c r="B996" s="50"/>
+      <c r="C996" s="49"/>
+      <c r="D996" s="49"/>
+      <c r="E996" s="49"/>
+      <c r="F996" s="49"/>
+      <c r="G996" s="49"/>
+      <c r="H996" s="49"/>
+      <c r="I996" s="49"/>
+    </row>
+    <row r="997" spans="1:10" ht="15.75">
+      <c r="A997" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B997" s="43" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="998" spans="1:10">
+      <c r="A998" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B998" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="H998" s="55"/>
+    </row>
+    <row r="999" spans="1:10">
+      <c r="A999" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B999">
+        <v>1</v>
+      </c>
+      <c r="F999" s="13"/>
+      <c r="H999" s="13"/>
+    </row>
+    <row r="1000" spans="1:10">
+      <c r="A1000" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1000" s="43" t="s">
+        <v>506</v>
+      </c>
+      <c r="F1000" s="13"/>
+      <c r="J1000" s="56"/>
+    </row>
+    <row r="1001" spans="1:10">
+      <c r="A1001" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1001" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1001" s="20"/>
+    </row>
+    <row r="1002" spans="1:10">
+      <c r="A1002" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1002" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="1003" spans="1:10">
+      <c r="A1003" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1003" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="1004" spans="1:10" ht="15.75">
+      <c r="A1004" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1004" s="26"/>
+      <c r="C1004" s="25"/>
+      <c r="D1004" s="26"/>
+      <c r="E1004" s="26"/>
+      <c r="F1004" s="26"/>
+      <c r="G1004" s="26"/>
+      <c r="H1004" s="26"/>
+      <c r="I1004" s="26"/>
+    </row>
+    <row r="1005" spans="1:10">
+      <c r="A1005" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1005" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1005" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1005" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1005" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="F1005" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1005" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1005" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1005" s="24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1006" spans="1:10">
+      <c r="A1006" s="31" t="s">
+        <v>506</v>
+      </c>
+      <c r="B1006" s="31" t="s">
+        <v>506</v>
+      </c>
+      <c r="C1006" s="26">
+        <v>1</v>
+      </c>
+      <c r="D1006" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1006" s="24"/>
+      <c r="G1006" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1006" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1006" s="24"/>
+    </row>
+    <row r="1007" spans="1:10">
+      <c r="A1007" s="31" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1007" s="31" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1007" s="13">
+        <v>2.2599999999999999E-2</v>
+      </c>
+      <c r="D1007" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1007" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1007" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1008" spans="1:10">
+      <c r="A1008" s="58" t="s">
+        <v>487</v>
+      </c>
+      <c r="B1008" s="13" t="s">
+        <v>488</v>
+      </c>
+      <c r="C1008">
+        <v>5.8150000000000004</v>
+      </c>
+      <c r="D1008" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1008" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1008" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1009" spans="1:10">
+      <c r="A1009" t="s">
+        <v>507</v>
+      </c>
+      <c r="B1009" s="13" t="s">
+        <v>508</v>
+      </c>
+      <c r="C1009" s="13">
+        <v>1.2333333333333333E-2</v>
+      </c>
+      <c r="D1009" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1009" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1009" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1010" spans="1:10">
+      <c r="A1010" t="s">
+        <v>473</v>
+      </c>
+      <c r="B1010" s="13" t="s">
+        <v>472</v>
+      </c>
+      <c r="C1010" s="13">
+        <v>0.98766666666666669</v>
+      </c>
+      <c r="D1010" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1010" s="13" t="s">
+        <v>515</v>
+      </c>
+      <c r="H1010" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1011" spans="1:10">
+      <c r="A1011" s="31" t="s">
+        <v>509</v>
+      </c>
+      <c r="B1011" s="13" t="s">
+        <v>510</v>
+      </c>
+      <c r="C1011" s="13">
+        <v>0.04</v>
+      </c>
+      <c r="D1011" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1011" s="13" t="s">
+        <v>511</v>
+      </c>
+      <c r="H1011" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1012" spans="1:10">
+      <c r="A1012" s="31" t="s">
+        <v>233</v>
+      </c>
+      <c r="B1012" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="C1012" s="13">
+        <v>8.3000000000000004E-2</v>
+      </c>
+      <c r="D1012" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1012" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1012" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1013" spans="1:10">
+      <c r="A1013" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1013" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1013" s="13">
+        <v>0.45424999999999999</v>
+      </c>
+      <c r="D1013" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1013" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1013" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1014" spans="1:10">
+      <c r="A1014" s="49"/>
+      <c r="B1014" s="50"/>
+      <c r="C1014" s="49"/>
+      <c r="D1014" s="49"/>
+      <c r="E1014" s="49"/>
+      <c r="F1014" s="49"/>
+      <c r="G1014" s="49"/>
+      <c r="H1014" s="49"/>
+      <c r="I1014" s="49"/>
+    </row>
+    <row r="1015" spans="1:10" ht="15.75">
+      <c r="A1015" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1015" s="43" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="1016" spans="1:10">
+      <c r="A1016" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1016" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1016" s="55"/>
+    </row>
+    <row r="1017" spans="1:10">
+      <c r="A1017" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1017">
+        <v>1</v>
+      </c>
+      <c r="F1017" s="13"/>
+      <c r="H1017" s="13"/>
+    </row>
+    <row r="1018" spans="1:10">
+      <c r="A1018" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1018" t="s">
+        <v>503</v>
+      </c>
+      <c r="F1018" s="13"/>
+      <c r="J1018" s="56"/>
+    </row>
+    <row r="1019" spans="1:10">
+      <c r="A1019" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1019" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1019" s="20"/>
+    </row>
+    <row r="1020" spans="1:10">
+      <c r="A1020" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1020" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="1021" spans="1:10">
+      <c r="A1021" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1021" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="1022" spans="1:10" ht="15.75">
+      <c r="A1022" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1022" s="26"/>
+      <c r="C1022" s="25"/>
+      <c r="D1022" s="26"/>
+      <c r="E1022" s="26"/>
+      <c r="F1022" s="26"/>
+      <c r="G1022" s="26"/>
+      <c r="H1022" s="26"/>
+      <c r="I1022" s="26"/>
+    </row>
+    <row r="1023" spans="1:10">
+      <c r="A1023" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1023" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1023" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1023" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1023" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="F1023" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1023" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1023" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1023" s="24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1024" spans="1:10">
+      <c r="A1024" s="31" t="s">
+        <v>502</v>
+      </c>
+      <c r="B1024" s="31" t="s">
+        <v>503</v>
+      </c>
+      <c r="C1024" s="26">
+        <v>1</v>
+      </c>
+      <c r="D1024" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1024" s="24"/>
+      <c r="G1024" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1024" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1024" s="24"/>
+    </row>
+    <row r="1025" spans="1:10">
+      <c r="A1025" s="31" t="s">
+        <v>495</v>
+      </c>
+      <c r="B1025" s="31" t="s">
+        <v>496</v>
+      </c>
+      <c r="C1025" s="41">
+        <v>1.35</v>
+      </c>
+      <c r="D1025" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1025" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1025" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1026" spans="1:10">
+      <c r="A1026" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1026" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1026">
+        <v>0.02</v>
+      </c>
+      <c r="D1026" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1026" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1026" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1027" spans="1:10">
+      <c r="A1027" s="31" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1027" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1027">
+        <v>3.8444917129434458E-2</v>
+      </c>
+      <c r="D1027" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1027" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1027" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1028" spans="1:10">
+      <c r="A1028" s="31" t="s">
+        <v>506</v>
+      </c>
+      <c r="B1028" s="31" t="s">
+        <v>506</v>
+      </c>
+      <c r="C1028">
+        <v>2.966014848457161E-5</v>
+      </c>
+      <c r="D1028" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1028" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1028" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1029" spans="1:10">
+      <c r="A1029" s="31" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1029" s="31" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1029">
+        <v>0.08</v>
+      </c>
+      <c r="D1029" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1029" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1029" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1030" spans="1:10">
+      <c r="A1030" s="58" t="s">
+        <v>487</v>
+      </c>
+      <c r="B1030" s="13" t="s">
+        <v>488</v>
+      </c>
+      <c r="C1030">
+        <v>4.17</v>
+      </c>
+      <c r="D1030" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1030" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1030" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1031" spans="1:10">
+      <c r="A1031" t="s">
+        <v>138</v>
+      </c>
+      <c r="C1031" s="13">
+        <v>0.16600000000000001</v>
+      </c>
+      <c r="D1031" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1031" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1031" t="s">
+        <v>109</v>
+      </c>
+      <c r="G1031" s="13"/>
+      <c r="H1031" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1032" spans="1:10">
+      <c r="A1032" s="31" t="s">
+        <v>140</v>
+      </c>
+      <c r="C1032" s="13">
+        <v>2.3E-2</v>
+      </c>
+      <c r="D1032" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1032" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1032" t="s">
+        <v>109</v>
+      </c>
+      <c r="G1032" s="13"/>
+      <c r="H1032" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1033" spans="1:10">
+      <c r="A1033" t="s">
+        <v>93</v>
+      </c>
+      <c r="C1033" s="13">
+        <v>0.13200000000000001</v>
+      </c>
+      <c r="D1033" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="E1033" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1033" t="s">
+        <v>25</v>
+      </c>
+      <c r="G1033" s="13"/>
+      <c r="H1033" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1034" spans="1:10">
+      <c r="A1034" t="s">
+        <v>505</v>
+      </c>
+      <c r="C1034" s="13">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="D1034" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1034" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1034" t="s">
+        <v>25</v>
+      </c>
+      <c r="G1034" s="13"/>
+      <c r="H1034" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1035" spans="1:10">
+      <c r="A1035" s="49"/>
+      <c r="B1035" s="50"/>
+      <c r="C1035" s="49"/>
+      <c r="D1035" s="49"/>
+      <c r="E1035" s="49"/>
+      <c r="F1035" s="49"/>
+      <c r="G1035" s="49"/>
+      <c r="H1035" s="49"/>
+      <c r="I1035" s="49"/>
+    </row>
+    <row r="1036" spans="1:10" ht="15.75">
+      <c r="A1036" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1036" s="43" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="1037" spans="1:10">
+      <c r="A1037" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1037" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1037" s="55"/>
+    </row>
+    <row r="1038" spans="1:10">
+      <c r="A1038" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1038">
+        <v>1</v>
+      </c>
+      <c r="F1038" s="13"/>
+      <c r="H1038" s="13"/>
+    </row>
+    <row r="1039" spans="1:10">
+      <c r="A1039" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1039" t="s">
+        <v>513</v>
+      </c>
+      <c r="F1039" s="13"/>
+      <c r="J1039" s="56"/>
+    </row>
+    <row r="1040" spans="1:10">
+      <c r="A1040" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1040" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1040" s="20"/>
+    </row>
+    <row r="1041" spans="1:9">
+      <c r="A1041" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1041" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="1042" spans="1:9">
+      <c r="A1042" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1042" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="1043" spans="1:9" ht="15.75">
+      <c r="A1043" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1043" s="26"/>
+      <c r="C1043" s="25"/>
+      <c r="D1043" s="26"/>
+      <c r="E1043" s="26"/>
+      <c r="F1043" s="26"/>
+      <c r="G1043" s="26"/>
+      <c r="H1043" s="26"/>
+      <c r="I1043" s="26"/>
+    </row>
+    <row r="1044" spans="1:9">
+      <c r="A1044" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1044" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1044" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1044" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1044" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="F1044" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1044" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1044" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1044" s="24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1045" spans="1:9">
+      <c r="A1045" s="31" t="s">
+        <v>512</v>
+      </c>
+      <c r="B1045" t="s">
+        <v>513</v>
+      </c>
+      <c r="C1045" s="26">
+        <v>1</v>
+      </c>
+      <c r="D1045" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1045" s="24"/>
+      <c r="G1045" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1045" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1045" s="26" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="1046" spans="1:9">
+      <c r="A1046" s="31" t="s">
+        <v>502</v>
+      </c>
+      <c r="B1046" s="31" t="s">
+        <v>503</v>
+      </c>
+      <c r="C1046" s="41">
+        <v>1.9251563934282565</v>
+      </c>
+      <c r="D1046" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1046" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1046" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1047" spans="1:9">
+      <c r="A1047" s="31" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1047" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1047">
+        <v>1.2513516557283666E-2</v>
+      </c>
+      <c r="D1047" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1047" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1047" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1048" spans="1:9">
+      <c r="A1048" s="31" t="s">
+        <v>506</v>
+      </c>
+      <c r="B1048" s="31" t="s">
+        <v>506</v>
+      </c>
+      <c r="C1048">
+        <v>4.2272109117479624E-5</v>
+      </c>
+      <c r="D1048" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1048" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1048" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1049" spans="1:9">
+      <c r="A1049" s="31" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1049" s="31" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1049">
+        <v>9.7719999999999987E-2</v>
+      </c>
+      <c r="D1049" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1049" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1049" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1050" spans="1:9">
+      <c r="A1050" s="58" t="s">
+        <v>487</v>
+      </c>
+      <c r="B1050" s="13" t="s">
+        <v>488</v>
+      </c>
+      <c r="C1050">
+        <v>8.0279021605958292</v>
+      </c>
+      <c r="D1050" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1050" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1050" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1051" spans="1:9">
+      <c r="A1051" t="s">
+        <v>138</v>
+      </c>
+      <c r="C1051" s="13">
+        <v>3.7649468801674725E-2</v>
+      </c>
+      <c r="D1051" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1051" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1051" t="s">
+        <v>109</v>
+      </c>
+      <c r="G1051" s="13"/>
+      <c r="H1051" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1052" spans="1:9">
+      <c r="A1052" s="31" t="s">
+        <v>140</v>
+      </c>
+      <c r="C1052" s="13">
+        <v>1.3022194842719922E-3</v>
+      </c>
+      <c r="D1052" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1052" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1052" t="s">
+        <v>109</v>
+      </c>
+      <c r="G1052" s="13"/>
+      <c r="H1052" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1053" spans="1:9">
+      <c r="A1053" t="s">
+        <v>93</v>
+      </c>
+      <c r="C1053" s="13">
+        <v>2.9173775990772428E-2</v>
+      </c>
+      <c r="D1053" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="E1053" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1053" t="s">
+        <v>25</v>
+      </c>
+      <c r="G1053" s="13"/>
+      <c r="H1053" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="14" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added LCI for mobility by plane
</commit_message>
<xml_diff>
--- a/inventories/lci-Tr2050.xlsx
+++ b/inventories/lci-Tr2050.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engie-my.sharepoint.com/personal/db6421_engie_com/Documents/Documents/Local_repo/ADEME_scenarios_premise_gas/inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2075" documentId="13_ncr:1_{6A9A1C53-53B4-4DAF-B82F-70FF83AECA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9248497-8342-4C26-BFBB-B93D2B6376E2}"/>
+  <xr:revisionPtr revIDLastSave="2150" documentId="13_ncr:1_{6A9A1C53-53B4-4DAF-B82F-70FF83AECA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F45A5959-8A16-4CAE-B5EB-9FAA9A681AAB}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4446" uniqueCount="516">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4519" uniqueCount="528">
   <si>
     <t>Database</t>
   </si>
@@ -1584,6 +1584,42 @@
   </si>
   <si>
     <t>IAI Area, EU27 &amp; EFTA</t>
+  </si>
+  <si>
+    <t>kerosene</t>
+  </si>
+  <si>
+    <t>market for kerosene</t>
+  </si>
+  <si>
+    <t>Carbon monoxide, fossil</t>
+  </si>
+  <si>
+    <t>Sulfur oxides</t>
+  </si>
+  <si>
+    <t>aircraft, passenger, medium haul</t>
+  </si>
+  <si>
+    <t>market for aircraft, passenger, medium haul</t>
+  </si>
+  <si>
+    <t>airport</t>
+  </si>
+  <si>
+    <t>market for airport</t>
+  </si>
+  <si>
+    <t>Scaled to 1 pkm from "GENESIS_2030_conventional_Base" (Thonemann et al., 2024) considering kerosene consumption in ecoinvent 391</t>
+  </si>
+  <si>
+    <t>transport, passenger aircraft</t>
+  </si>
+  <si>
+    <t>transport, passenger aircraft, medium haul</t>
+  </si>
+  <si>
+    <t>person kilometer</t>
   </si>
 </sst>
 </file>
@@ -2110,7 +2146,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AH1053"/>
+  <dimension ref="A1:AH1073"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="73.140625" customWidth="1"/>
@@ -27565,6 +27601,321 @@
         <v>15</v>
       </c>
     </row>
+    <row r="1054" spans="1:9">
+      <c r="A1054" s="49"/>
+      <c r="B1054" s="50"/>
+      <c r="C1054" s="49"/>
+      <c r="D1054" s="49"/>
+      <c r="E1054" s="49"/>
+      <c r="F1054" s="49"/>
+      <c r="G1054" s="49"/>
+      <c r="H1054" s="49"/>
+      <c r="I1054" s="49"/>
+    </row>
+    <row r="1055" spans="1:9" ht="15.75">
+      <c r="A1055" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1055" s="24" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="1056" spans="1:9">
+      <c r="A1056" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1056" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1056" s="55"/>
+    </row>
+    <row r="1057" spans="1:10">
+      <c r="A1057" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1057">
+        <v>1</v>
+      </c>
+      <c r="F1057" s="13"/>
+      <c r="H1057" s="13"/>
+    </row>
+    <row r="1058" spans="1:10">
+      <c r="A1058" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1058" s="26" t="s">
+        <v>526</v>
+      </c>
+      <c r="F1058" s="13"/>
+      <c r="J1058" s="56"/>
+    </row>
+    <row r="1059" spans="1:10">
+      <c r="A1059" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1059" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1059" s="20"/>
+    </row>
+    <row r="1060" spans="1:10">
+      <c r="A1060" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1060" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="1061" spans="1:10">
+      <c r="A1061" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1061" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="1062" spans="1:10" ht="15.75">
+      <c r="A1062" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1062" s="26"/>
+      <c r="C1062" s="25"/>
+      <c r="D1062" s="26"/>
+      <c r="E1062" s="26"/>
+      <c r="F1062" s="26"/>
+      <c r="G1062" s="26"/>
+      <c r="H1062" s="26"/>
+      <c r="I1062" s="26"/>
+    </row>
+    <row r="1063" spans="1:10">
+      <c r="A1063" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1063" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1063" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1063" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1063" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="F1063" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1063" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1063" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1063" s="24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1064" spans="1:10">
+      <c r="A1064" s="26" t="s">
+        <v>525</v>
+      </c>
+      <c r="B1064" s="26" t="s">
+        <v>526</v>
+      </c>
+      <c r="C1064">
+        <v>1</v>
+      </c>
+      <c r="D1064" t="s">
+        <v>527</v>
+      </c>
+      <c r="G1064" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1064" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="1065" spans="1:10">
+      <c r="A1065" t="s">
+        <v>521</v>
+      </c>
+      <c r="B1065" s="13" t="s">
+        <v>520</v>
+      </c>
+      <c r="C1065">
+        <v>6.1215814640472162E-10</v>
+      </c>
+      <c r="D1065" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1065" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1065" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1066" spans="1:10">
+      <c r="A1066" t="s">
+        <v>523</v>
+      </c>
+      <c r="B1066" s="13" t="s">
+        <v>522</v>
+      </c>
+      <c r="C1066">
+        <v>4.742138768774307E-10</v>
+      </c>
+      <c r="D1066" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1066" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1066" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1067" spans="1:10">
+      <c r="A1067" t="s">
+        <v>517</v>
+      </c>
+      <c r="B1067" s="13" t="s">
+        <v>516</v>
+      </c>
+      <c r="C1067">
+        <v>2.6426999999999999E-2</v>
+      </c>
+      <c r="D1067" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1067" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1067" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1068" spans="1:10">
+      <c r="A1068" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1068">
+        <v>3.0319294841785747E-4</v>
+      </c>
+      <c r="D1068" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1068" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1068" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1068" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1069" spans="1:10">
+      <c r="A1069" t="s">
+        <v>518</v>
+      </c>
+      <c r="C1069">
+        <v>1.0312926008611849E-4</v>
+      </c>
+      <c r="D1069" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1069" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1069" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1069" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1070" spans="1:10">
+      <c r="A1070" t="s">
+        <v>431</v>
+      </c>
+      <c r="C1070">
+        <v>9.6919104678861535E-6</v>
+      </c>
+      <c r="D1070" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1070" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1070" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1070" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1071" spans="1:10">
+      <c r="A1071" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1071">
+        <v>8.3218361203244121E-2</v>
+      </c>
+      <c r="D1071" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1071" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1071" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1071" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1072" spans="1:10">
+      <c r="A1072" t="s">
+        <v>93</v>
+      </c>
+      <c r="C1072">
+        <v>3.2505107742137262E-5</v>
+      </c>
+      <c r="D1072" t="s">
+        <v>91</v>
+      </c>
+      <c r="E1072" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1072" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1072" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1073" spans="1:8">
+      <c r="A1073" t="s">
+        <v>519</v>
+      </c>
+      <c r="C1073">
+        <v>2.219861016536204E-5</v>
+      </c>
+      <c r="D1073" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1073" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1073" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1073" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="14" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
- Added activities and market structure for space heating and cooling in residential buildings
</commit_message>
<xml_diff>
--- a/inventories/lci-Tr2050.xlsx
+++ b/inventories/lci-Tr2050.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engie-my.sharepoint.com/personal/db6421_engie_com/Documents/Documents/Local_repo/ADEME_scenarios_premise_gas/inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2150" documentId="13_ncr:1_{6A9A1C53-53B4-4DAF-B82F-70FF83AECA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F45A5959-8A16-4CAE-B5EB-9FAA9A681AAB}"/>
+  <xr:revisionPtr revIDLastSave="2165" documentId="13_ncr:1_{6A9A1C53-53B4-4DAF-B82F-70FF83AECA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7DD2D845-EE12-4BE8-A9A0-F260AE1981B4}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="lci" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4519" uniqueCount="528">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4551" uniqueCount="530">
   <si>
     <t>Database</t>
   </si>
@@ -1620,6 +1620,12 @@
   </si>
   <si>
     <t>person kilometer</t>
+  </si>
+  <si>
+    <t>heat, electric boiler</t>
+  </si>
+  <si>
+    <t>heat</t>
   </si>
 </sst>
 </file>
@@ -2146,7 +2152,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AH1073"/>
+  <dimension ref="A1:AH1085"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="73.140625" customWidth="1"/>
@@ -27896,7 +27902,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="1073" spans="1:8">
+    <row r="1073" spans="1:10">
       <c r="A1073" t="s">
         <v>519</v>
       </c>
@@ -27914,6 +27920,159 @@
       </c>
       <c r="H1073" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="1074" spans="1:10">
+      <c r="A1074" s="49"/>
+      <c r="B1074" s="50"/>
+      <c r="C1074" s="49"/>
+      <c r="D1074" s="49"/>
+      <c r="E1074" s="49"/>
+      <c r="F1074" s="49"/>
+      <c r="G1074" s="49"/>
+      <c r="H1074" s="49"/>
+      <c r="I1074" s="49"/>
+    </row>
+    <row r="1075" spans="1:10" ht="15.75">
+      <c r="A1075" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1075" s="24" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="1076" spans="1:10">
+      <c r="A1076" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1076" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1076" s="55"/>
+    </row>
+    <row r="1077" spans="1:10">
+      <c r="A1077" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1077">
+        <v>1</v>
+      </c>
+      <c r="F1077" s="13"/>
+      <c r="H1077" s="13"/>
+    </row>
+    <row r="1078" spans="1:10">
+      <c r="A1078" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1078" s="26" t="s">
+        <v>529</v>
+      </c>
+      <c r="F1078" s="13"/>
+      <c r="J1078" s="56"/>
+    </row>
+    <row r="1079" spans="1:10">
+      <c r="A1079" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1079" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1079" s="20"/>
+    </row>
+    <row r="1080" spans="1:10">
+      <c r="A1080" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1080" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="1081" spans="1:10">
+      <c r="A1081" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1081"/>
+    </row>
+    <row r="1082" spans="1:10" ht="15.75">
+      <c r="A1082" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1082" s="26"/>
+      <c r="C1082" s="25"/>
+      <c r="D1082" s="26"/>
+      <c r="E1082" s="26"/>
+      <c r="F1082" s="26"/>
+      <c r="G1082" s="26"/>
+      <c r="H1082" s="26"/>
+      <c r="I1082" s="26"/>
+    </row>
+    <row r="1083" spans="1:10">
+      <c r="A1083" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1083" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1083" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1083" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1083" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="F1083" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1083" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1083" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1083" s="24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1084" spans="1:10">
+      <c r="A1084" s="26" t="s">
+        <v>528</v>
+      </c>
+      <c r="B1084" s="26" t="s">
+        <v>529</v>
+      </c>
+      <c r="C1084">
+        <v>1</v>
+      </c>
+      <c r="D1084" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1084" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1084" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="1085" spans="1:10">
+      <c r="A1085" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1085" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1085">
+        <v>0.27777777777777779</v>
+      </c>
+      <c r="D1085" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1085" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1085" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
- Updated petrola nd diesel production pathways - Added new market for LPG and light fuel oil - Added new market for district heat - Updated district heat production pathways for buildings
</commit_message>
<xml_diff>
--- a/inventories/lci-Tr2050.xlsx
+++ b/inventories/lci-Tr2050.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engie-my.sharepoint.com/personal/db6421_engie_com/Documents/Documents/Local_repo/ADEME_scenarios_premise_gas/inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2165" documentId="13_ncr:1_{6A9A1C53-53B4-4DAF-B82F-70FF83AECA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7DD2D845-EE12-4BE8-A9A0-F260AE1981B4}"/>
+  <xr:revisionPtr revIDLastSave="2223" documentId="13_ncr:1_{6A9A1C53-53B4-4DAF-B82F-70FF83AECA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A01ECB3-D384-4DA9-A7D0-747CFC982C57}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4551" uniqueCount="530">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4604" uniqueCount="538">
   <si>
     <t>Database</t>
   </si>
@@ -1626,6 +1626,30 @@
   </si>
   <si>
     <t>heat</t>
+  </si>
+  <si>
+    <t>ethanol production from whey</t>
+  </si>
+  <si>
+    <t>ethanol production from grass</t>
+  </si>
+  <si>
+    <t>ethanol production from sugar beet</t>
+  </si>
+  <si>
+    <t>ethanol, without water, in 95% solution state, from fermentation</t>
+  </si>
+  <si>
+    <t>Adapted from the Swiss process in ecoinvent, considering equal distribution among feedstocks</t>
+  </si>
+  <si>
+    <t>dewatering of ethanol from biomass, from 95% to 99.7%</t>
+  </si>
+  <si>
+    <t>ethanol, from fermentation, 99.7%</t>
+  </si>
+  <si>
+    <t>heat production, natural gas, at boiler condensing modulating &gt;100kW</t>
   </si>
 </sst>
 </file>
@@ -2152,7 +2176,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AH1085"/>
+  <dimension ref="A1:AH1101"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="73.140625" customWidth="1"/>
@@ -28075,6 +28099,241 @@
         <v>12</v>
       </c>
     </row>
+    <row r="1086" spans="1:10">
+      <c r="A1086" s="49"/>
+      <c r="B1086" s="50"/>
+      <c r="C1086" s="49"/>
+      <c r="D1086" s="49"/>
+      <c r="E1086" s="49"/>
+      <c r="F1086" s="49"/>
+      <c r="G1086" s="49"/>
+      <c r="H1086" s="49"/>
+      <c r="I1086" s="49"/>
+    </row>
+    <row r="1087" spans="1:10" ht="15.75">
+      <c r="A1087" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1087" s="24" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="1088" spans="1:10">
+      <c r="A1088" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1088" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1088" s="55"/>
+    </row>
+    <row r="1089" spans="1:10">
+      <c r="A1089" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1089">
+        <v>1</v>
+      </c>
+      <c r="F1089" s="13"/>
+      <c r="H1089" s="13"/>
+    </row>
+    <row r="1090" spans="1:10">
+      <c r="A1090" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1090" s="26" t="s">
+        <v>536</v>
+      </c>
+      <c r="F1090" s="13"/>
+      <c r="J1090" s="56"/>
+    </row>
+    <row r="1091" spans="1:10">
+      <c r="A1091" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1091" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1091" s="20"/>
+    </row>
+    <row r="1092" spans="1:10">
+      <c r="A1092" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1092" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="1093" spans="1:10">
+      <c r="A1093" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1093" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="1094" spans="1:10" ht="15.75">
+      <c r="A1094" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1094" s="26"/>
+      <c r="C1094" s="25"/>
+      <c r="D1094" s="26"/>
+      <c r="E1094" s="26"/>
+      <c r="F1094" s="26"/>
+      <c r="G1094" s="26"/>
+      <c r="H1094" s="26"/>
+      <c r="I1094" s="26"/>
+    </row>
+    <row r="1095" spans="1:10">
+      <c r="A1095" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1095" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1095" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1095" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1095" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="F1095" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1095" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1095" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1095" s="24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1096" spans="1:10">
+      <c r="A1096" s="26" t="s">
+        <v>535</v>
+      </c>
+      <c r="B1096" s="26" t="s">
+        <v>536</v>
+      </c>
+      <c r="C1096">
+        <v>1</v>
+      </c>
+      <c r="D1096" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1096" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1096" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="1097" spans="1:10">
+      <c r="A1097" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1097" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1097" s="13">
+        <v>8.3599999999999999E-5</v>
+      </c>
+      <c r="D1097" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1097" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1097" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1098" spans="1:10">
+      <c r="A1098" t="s">
+        <v>537</v>
+      </c>
+      <c r="B1098" s="13" t="s">
+        <v>488</v>
+      </c>
+      <c r="C1098">
+        <v>6.25E-2</v>
+      </c>
+      <c r="D1098" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1098" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1098" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1099" spans="1:10">
+      <c r="A1099" t="s">
+        <v>530</v>
+      </c>
+      <c r="B1099" s="13" t="s">
+        <v>533</v>
+      </c>
+      <c r="C1099" s="41">
+        <v>0.33329999999999999</v>
+      </c>
+      <c r="D1099" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1099" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1099" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1100" spans="1:10">
+      <c r="A1100" t="s">
+        <v>531</v>
+      </c>
+      <c r="B1100" s="13" t="s">
+        <v>533</v>
+      </c>
+      <c r="C1100" s="41">
+        <v>0.33329999999999999</v>
+      </c>
+      <c r="D1100" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1100" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1100" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1101" spans="1:10">
+      <c r="A1101" t="s">
+        <v>532</v>
+      </c>
+      <c r="B1101" s="13" t="s">
+        <v>533</v>
+      </c>
+      <c r="C1101" s="41">
+        <v>0.33329999999999999</v>
+      </c>
+      <c r="D1101" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1101" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1101" t="s">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="14" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated bioethanol production to avoid unlinked exchanges message
</commit_message>
<xml_diff>
--- a/inventories/lci-Tr2050.xlsx
+++ b/inventories/lci-Tr2050.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engie-my.sharepoint.com/personal/db6421_engie_com/Documents/Documents/Local_repo/ADEME_scenarios_premise_gas/inventories/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DB6421\OneDrive - ENGIE\Documents\Local_repo\ADEME_scenarios_premise_gas\inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2223" documentId="13_ncr:1_{6A9A1C53-53B4-4DAF-B82F-70FF83AECA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A01ECB3-D384-4DA9-A7D0-747CFC982C57}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0F9393E-493D-4D41-96B2-57E4008F0D51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="lci" sheetId="1" r:id="rId1"/>
@@ -2177,17 +2177,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AH1101"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="73.140625" customWidth="1"/>
-    <col min="2" max="2" width="18.5703125" style="13" customWidth="1"/>
-    <col min="3" max="3" width="17.140625" customWidth="1"/>
-    <col min="4" max="4" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.42578125" customWidth="1"/>
-    <col min="6" max="6" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="109.7109375" customWidth="1"/>
+    <col min="1" max="1" width="73.109375" customWidth="1"/>
+    <col min="2" max="2" width="18.5546875" style="13" customWidth="1"/>
+    <col min="3" max="3" width="17.109375" customWidth="1"/>
+    <col min="4" max="4" width="24.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.44140625" customWidth="1"/>
+    <col min="6" max="6" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="109.6640625" customWidth="1"/>
     <col min="10" max="10" width="31" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2239,7 +2239,7 @@
       <c r="I4" s="6"/>
       <c r="K4" s="5"/>
     </row>
-    <row r="5" spans="1:14" ht="15.75">
+    <row r="5" spans="1:14" ht="15.6">
       <c r="A5" s="18" t="s">
         <v>1</v>
       </c>
@@ -2321,7 +2321,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="15.75">
+    <row r="13" spans="1:14" ht="15.6">
       <c r="A13" s="18" t="s">
         <v>7</v>
       </c>
@@ -2330,7 +2330,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="15.75">
+    <row r="14" spans="1:14" ht="15.6">
       <c r="A14" s="18" t="s">
         <v>8</v>
       </c>
@@ -3043,7 +3043,7 @@
       <c r="AG47" s="47"/>
       <c r="AH47" s="47"/>
     </row>
-    <row r="48" spans="1:34" s="15" customFormat="1" ht="15.75">
+    <row r="48" spans="1:34" s="15" customFormat="1" ht="15.6">
       <c r="A48" s="2" t="s">
         <v>1</v>
       </c>
@@ -3063,7 +3063,7 @@
       <c r="O48" s="16"/>
       <c r="P48" s="16"/>
     </row>
-    <row r="49" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="49" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A49" s="2" t="s">
         <v>3</v>
       </c>
@@ -3083,7 +3083,7 @@
       <c r="O49" s="16"/>
       <c r="P49" s="16"/>
     </row>
-    <row r="50" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="50" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A50" s="2" t="s">
         <v>11</v>
       </c>
@@ -3103,7 +3103,7 @@
       <c r="O50" s="16"/>
       <c r="P50" s="16"/>
     </row>
-    <row r="51" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="51" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A51" s="2" t="s">
         <v>4</v>
       </c>
@@ -3123,7 +3123,7 @@
       <c r="O51" s="16"/>
       <c r="P51" s="16"/>
     </row>
-    <row r="52" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="52" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A52" s="2" t="s">
         <v>2</v>
       </c>
@@ -3143,7 +3143,7 @@
       <c r="O52" s="16"/>
       <c r="P52" s="16"/>
     </row>
-    <row r="53" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="53" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A53" s="2" t="s">
         <v>6</v>
       </c>
@@ -3165,7 +3165,7 @@
       <c r="O53" s="16"/>
       <c r="P53" s="16"/>
     </row>
-    <row r="54" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="54" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A54" s="2" t="s">
         <v>7</v>
       </c>
@@ -3185,7 +3185,7 @@
       <c r="O54" s="16"/>
       <c r="P54" s="16"/>
     </row>
-    <row r="55" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="55" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A55" s="2" t="s">
         <v>8</v>
       </c>
@@ -3223,7 +3223,7 @@
       <c r="S55" s="17"/>
       <c r="T55" s="18"/>
     </row>
-    <row r="56" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="56" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A56" t="s">
         <v>54</v>
       </c>
@@ -3255,7 +3255,7 @@
       <c r="P56" s="16"/>
       <c r="T56"/>
     </row>
-    <row r="57" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="57" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A57" t="s">
         <v>52</v>
       </c>
@@ -3289,7 +3289,7 @@
       <c r="Q57"/>
       <c r="R57"/>
     </row>
-    <row r="58" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="58" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A58" t="s">
         <v>53</v>
       </c>
@@ -3323,7 +3323,7 @@
       <c r="Q58"/>
       <c r="R58"/>
     </row>
-    <row r="59" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="59" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A59" t="s">
         <v>43</v>
       </c>
@@ -3357,7 +3357,7 @@
       <c r="Q59"/>
       <c r="R59"/>
     </row>
-    <row r="60" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="60" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A60" t="s">
         <v>46</v>
       </c>
@@ -3391,7 +3391,7 @@
       <c r="Q60"/>
       <c r="R60"/>
     </row>
-    <row r="61" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="61" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A61" t="s">
         <v>27</v>
       </c>
@@ -3424,7 +3424,7 @@
       <c r="Q61"/>
       <c r="R61"/>
     </row>
-    <row r="62" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="62" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A62" t="s">
         <v>21</v>
       </c>
@@ -3457,7 +3457,7 @@
       <c r="Q62"/>
       <c r="R62"/>
     </row>
-    <row r="63" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="63" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A63" t="s">
         <v>24</v>
       </c>
@@ -3486,7 +3486,7 @@
       <c r="Q63" s="20"/>
       <c r="R63"/>
     </row>
-    <row r="64" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="64" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A64" t="s">
         <v>51</v>
       </c>
@@ -3555,7 +3555,7 @@
       <c r="AG65" s="47"/>
       <c r="AH65" s="47"/>
     </row>
-    <row r="66" spans="1:34" ht="15.75">
+    <row r="66" spans="1:34" ht="15.6">
       <c r="A66" s="18" t="s">
         <v>1</v>
       </c>
@@ -3617,13 +3617,13 @@
         <v>13</v>
       </c>
     </row>
-    <row r="74" spans="1:34" ht="15.75">
+    <row r="74" spans="1:34" ht="15.6">
       <c r="A74" s="18" t="s">
         <v>7</v>
       </c>
       <c r="B74"/>
     </row>
-    <row r="75" spans="1:34" ht="15.75">
+    <row r="75" spans="1:34" ht="15.6">
       <c r="A75" s="18" t="s">
         <v>8</v>
       </c>
@@ -17062,7 +17062,7 @@
       </c>
       <c r="B458"/>
     </row>
-    <row r="459" spans="1:34" ht="15.75">
+    <row r="459" spans="1:34" ht="15.6">
       <c r="A459" s="18" t="s">
         <v>7</v>
       </c>
@@ -17459,7 +17459,7 @@
       </c>
       <c r="B482"/>
     </row>
-    <row r="483" spans="1:9" ht="15.75">
+    <row r="483" spans="1:9" ht="15.6">
       <c r="A483" s="18" t="s">
         <v>7</v>
       </c>
@@ -18036,7 +18036,7 @@
       </c>
       <c r="B514"/>
     </row>
-    <row r="515" spans="1:9" ht="15.75">
+    <row r="515" spans="1:9" ht="15.6">
       <c r="A515" s="18" t="s">
         <v>7</v>
       </c>
@@ -18613,7 +18613,7 @@
       </c>
       <c r="B546"/>
     </row>
-    <row r="547" spans="1:9" ht="15.75">
+    <row r="547" spans="1:9" ht="15.6">
       <c r="A547" s="18" t="s">
         <v>7</v>
       </c>
@@ -19190,7 +19190,7 @@
       </c>
       <c r="B578"/>
     </row>
-    <row r="579" spans="1:9" ht="15.75">
+    <row r="579" spans="1:9" ht="15.6">
       <c r="A579" s="18" t="s">
         <v>7</v>
       </c>
@@ -19767,7 +19767,7 @@
       </c>
       <c r="B610"/>
     </row>
-    <row r="611" spans="1:9" ht="15.75">
+    <row r="611" spans="1:9" ht="15.6">
       <c r="A611" s="18" t="s">
         <v>7</v>
       </c>
@@ -20164,7 +20164,7 @@
       </c>
       <c r="B634"/>
     </row>
-    <row r="635" spans="1:9" ht="15.75">
+    <row r="635" spans="1:9" ht="15.6">
       <c r="A635" s="18" t="s">
         <v>7</v>
       </c>
@@ -20741,7 +20741,7 @@
       </c>
       <c r="B666"/>
     </row>
-    <row r="667" spans="1:9" ht="15.75">
+    <row r="667" spans="1:9" ht="15.6">
       <c r="A667" s="18" t="s">
         <v>7</v>
       </c>
@@ -21318,7 +21318,7 @@
       </c>
       <c r="B698"/>
     </row>
-    <row r="699" spans="1:9" ht="15.75">
+    <row r="699" spans="1:9" ht="15.6">
       <c r="A699" s="18" t="s">
         <v>7</v>
       </c>
@@ -21896,7 +21896,7 @@
       </c>
       <c r="B730"/>
     </row>
-    <row r="731" spans="1:9" ht="15.75">
+    <row r="731" spans="1:9" ht="15.6">
       <c r="A731" s="18" t="s">
         <v>7</v>
       </c>
@@ -22475,7 +22475,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="763" spans="1:21" ht="15.75">
+    <row r="763" spans="1:21" ht="15.6">
       <c r="A763" s="18" t="s">
         <v>7</v>
       </c>
@@ -24732,7 +24732,7 @@
       <c r="H887" s="49"/>
       <c r="I887" s="49"/>
     </row>
-    <row r="888" spans="1:10" ht="15.75">
+    <row r="888" spans="1:10" ht="15.6">
       <c r="A888" s="18" t="s">
         <v>1</v>
       </c>
@@ -24794,7 +24794,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="895" spans="1:10" ht="15.75">
+    <row r="895" spans="1:10" ht="15.6">
       <c r="A895" s="18" t="s">
         <v>7</v>
       </c>
@@ -25458,7 +25458,7 @@
       <c r="H924" s="49"/>
       <c r="I924" s="49"/>
     </row>
-    <row r="925" spans="1:10" ht="15.75">
+    <row r="925" spans="1:10" ht="15.6">
       <c r="A925" s="18" t="s">
         <v>1</v>
       </c>
@@ -25520,7 +25520,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="932" spans="1:9" ht="15.75">
+    <row r="932" spans="1:9" ht="15.6">
       <c r="A932" s="18" t="s">
         <v>7</v>
       </c>
@@ -26187,7 +26187,7 @@
       <c r="H961" s="49"/>
       <c r="I961" s="49"/>
     </row>
-    <row r="962" spans="1:10" ht="15.75">
+    <row r="962" spans="1:10" ht="15.6">
       <c r="A962" s="18" t="s">
         <v>1</v>
       </c>
@@ -26249,7 +26249,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="969" spans="1:10" ht="15.75">
+    <row r="969" spans="1:10" ht="15.6">
       <c r="A969" s="18" t="s">
         <v>7</v>
       </c>
@@ -26465,7 +26465,7 @@
       <c r="H979" s="49"/>
       <c r="I979" s="49"/>
     </row>
-    <row r="980" spans="1:10" ht="15.75">
+    <row r="980" spans="1:10" ht="15.6">
       <c r="A980" s="18" t="s">
         <v>1</v>
       </c>
@@ -26527,7 +26527,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="987" spans="1:10" ht="15.75">
+    <row r="987" spans="1:10" ht="15.6">
       <c r="A987" s="18" t="s">
         <v>7</v>
       </c>
@@ -26722,7 +26722,7 @@
       <c r="H996" s="49"/>
       <c r="I996" s="49"/>
     </row>
-    <row r="997" spans="1:10" ht="15.75">
+    <row r="997" spans="1:10" ht="15.6">
       <c r="A997" s="18" t="s">
         <v>1</v>
       </c>
@@ -26784,7 +26784,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="1004" spans="1:10" ht="15.75">
+    <row r="1004" spans="1:10" ht="15.6">
       <c r="A1004" s="18" t="s">
         <v>7</v>
       </c>
@@ -26999,7 +26999,7 @@
       <c r="H1014" s="49"/>
       <c r="I1014" s="49"/>
     </row>
-    <row r="1015" spans="1:10" ht="15.75">
+    <row r="1015" spans="1:10" ht="15.6">
       <c r="A1015" s="18" t="s">
         <v>1</v>
       </c>
@@ -27061,7 +27061,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="1022" spans="1:10" ht="15.75">
+    <row r="1022" spans="1:10" ht="15.6">
       <c r="A1022" s="18" t="s">
         <v>7</v>
       </c>
@@ -27340,7 +27340,7 @@
       <c r="H1035" s="49"/>
       <c r="I1035" s="49"/>
     </row>
-    <row r="1036" spans="1:10" ht="15.75">
+    <row r="1036" spans="1:10" ht="15.6">
       <c r="A1036" s="18" t="s">
         <v>1</v>
       </c>
@@ -27402,7 +27402,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="1043" spans="1:9" ht="15.75">
+    <row r="1043" spans="1:9" ht="15.6">
       <c r="A1043" s="18" t="s">
         <v>7</v>
       </c>
@@ -27642,7 +27642,7 @@
       <c r="H1054" s="49"/>
       <c r="I1054" s="49"/>
     </row>
-    <row r="1055" spans="1:9" ht="15.75">
+    <row r="1055" spans="1:9" ht="15.6">
       <c r="A1055" s="18" t="s">
         <v>1</v>
       </c>
@@ -27704,7 +27704,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="1062" spans="1:10" ht="15.75">
+    <row r="1062" spans="1:10" ht="15.6">
       <c r="A1062" s="18" t="s">
         <v>7</v>
       </c>
@@ -27957,7 +27957,7 @@
       <c r="H1074" s="49"/>
       <c r="I1074" s="49"/>
     </row>
-    <row r="1075" spans="1:10" ht="15.75">
+    <row r="1075" spans="1:10" ht="15.6">
       <c r="A1075" s="18" t="s">
         <v>1</v>
       </c>
@@ -28017,7 +28017,7 @@
       </c>
       <c r="B1081"/>
     </row>
-    <row r="1082" spans="1:10" ht="15.75">
+    <row r="1082" spans="1:10" ht="15.6">
       <c r="A1082" s="18" t="s">
         <v>7</v>
       </c>
@@ -28110,7 +28110,7 @@
       <c r="H1086" s="49"/>
       <c r="I1086" s="49"/>
     </row>
-    <row r="1087" spans="1:10" ht="15.75">
+    <row r="1087" spans="1:10" ht="15.6">
       <c r="A1087" s="18" t="s">
         <v>1</v>
       </c>
@@ -28172,7 +28172,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="1094" spans="1:10" ht="15.75">
+    <row r="1094" spans="1:10" ht="15.6">
       <c r="A1094" s="18" t="s">
         <v>7</v>
       </c>
@@ -28268,7 +28268,7 @@
         <v>35</v>
       </c>
       <c r="G1098" t="s">
-        <v>28</v>
+        <v>134</v>
       </c>
       <c r="H1098" t="s">
         <v>12</v>
@@ -28288,7 +28288,7 @@
         <v>13</v>
       </c>
       <c r="G1099" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H1099" t="s">
         <v>12</v>
@@ -28308,7 +28308,7 @@
         <v>13</v>
       </c>
       <c r="G1100" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H1100" t="s">
         <v>12</v>
@@ -28328,7 +28328,7 @@
         <v>13</v>
       </c>
       <c r="G1101" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H1101" t="s">
         <v>12</v>

</xml_diff>

<commit_message>
Heat in biomethane regionalized to France TODO: Solve message "unlinked activity"
</commit_message>
<xml_diff>
--- a/inventories/lci-Tr2050.xlsx
+++ b/inventories/lci-Tr2050.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engie-my.sharepoint.com/personal/db6421_engie_com/Documents/Documents/Local_repo/ADEME_scenarios_premise_gas/inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="53" documentId="13_ncr:1_{D0F9393E-493D-4D41-96B2-57E4008F0D51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F2923EAE-C4AC-4684-B8DD-E84291BF29D9}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="13_ncr:1_{D0F9393E-493D-4D41-96B2-57E4008F0D51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0899827B-D536-48BF-AD09-1FF2BD22290A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23543,7 +23543,7 @@
       </c>
       <c r="E820" s="31"/>
       <c r="G820" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H820" s="31" t="s">
         <v>12</v>
@@ -23759,7 +23759,7 @@
       </c>
       <c r="E835" s="31"/>
       <c r="G835" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H835" s="31" t="s">
         <v>12</v>

</xml_diff>

<commit_message>
Created activity for heat production using biomethane in a boiler. It allows to account for changes in the composition of the natural gas mix.
</commit_message>
<xml_diff>
--- a/inventories/lci-Tr2050.xlsx
+++ b/inventories/lci-Tr2050.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engie-my.sharepoint.com/personal/db6421_engie_com/Documents/Documents/Local_repo/ADEME_scenarios_premise_gas/inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="93" documentId="13_ncr:1_{D0F9393E-493D-4D41-96B2-57E4008F0D51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0BF21A1-1BE6-4754-B44D-508832EE6212}"/>
+  <xr:revisionPtr revIDLastSave="225" documentId="13_ncr:1_{D0F9393E-493D-4D41-96B2-57E4008F0D51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC1276D8-0E19-4090-8BE4-B42B2CA7BEE6}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="lci" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4580" uniqueCount="522">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4632" uniqueCount="523">
   <si>
     <t>Database</t>
   </si>
@@ -1602,6 +1602,9 @@
   </si>
   <si>
     <t>Adapted from premise (US inventory). Transport is removed and absorbed CO2 set to zero as it is already considered in the anaerobic digestion activity. Electricity, diesel, petrol and natural gas inputs are specified to France.</t>
+  </si>
+  <si>
+    <t>heat, biomethane</t>
   </si>
 </sst>
 </file>
@@ -1615,7 +1618,7 @@
     <numFmt numFmtId="167" formatCode="0.0000"/>
     <numFmt numFmtId="168" formatCode="0.000%"/>
     <numFmt numFmtId="169" formatCode="0.00000"/>
-    <numFmt numFmtId="173" formatCode="0.0000E+00"/>
+    <numFmt numFmtId="170" formatCode="0.0000E+00"/>
   </numFmts>
   <fonts count="16">
     <font>
@@ -1851,7 +1854,7 @@
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="173" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -2138,7 +2141,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AH1100"/>
+  <dimension ref="A1:AH1116"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="73.140625" customWidth="1"/>
@@ -28148,6 +28151,237 @@
         <v>12</v>
       </c>
     </row>
+    <row r="1101" spans="1:10">
+      <c r="A1101" s="49"/>
+      <c r="B1101" s="50"/>
+      <c r="C1101" s="49"/>
+      <c r="D1101" s="49"/>
+      <c r="E1101" s="49"/>
+      <c r="F1101" s="49"/>
+      <c r="G1101" s="49"/>
+      <c r="H1101" s="49"/>
+      <c r="I1101" s="49"/>
+    </row>
+    <row r="1102" spans="1:10" ht="15.75">
+      <c r="A1102" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1102" s="13" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="1103" spans="1:10">
+      <c r="A1103" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1103" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1103" s="55"/>
+    </row>
+    <row r="1104" spans="1:10">
+      <c r="A1104" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1104" s="13">
+        <v>1</v>
+      </c>
+      <c r="F1104" s="13"/>
+      <c r="H1104" s="13"/>
+    </row>
+    <row r="1105" spans="1:10">
+      <c r="A1105" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1105" s="13" t="s">
+        <v>522</v>
+      </c>
+      <c r="F1105" s="13"/>
+      <c r="J1105" s="56"/>
+    </row>
+    <row r="1106" spans="1:10">
+      <c r="A1106" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1106" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1106" s="20"/>
+    </row>
+    <row r="1107" spans="1:10">
+      <c r="A1107" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1107" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="1108" spans="1:10">
+      <c r="A1108" s="24" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="1109" spans="1:10" ht="15.75">
+      <c r="A1109" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1109" s="25"/>
+      <c r="D1109" s="26"/>
+      <c r="E1109" s="26"/>
+      <c r="F1109" s="26"/>
+      <c r="G1109" s="26"/>
+      <c r="H1109" s="26"/>
+      <c r="I1109" s="26"/>
+    </row>
+    <row r="1110" spans="1:10">
+      <c r="A1110" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1110" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1110" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1110" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1110" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="F1110" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1110" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1110" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1110" s="24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1111" spans="1:10">
+      <c r="A1111" s="13" t="s">
+        <v>439</v>
+      </c>
+      <c r="B1111" s="13" t="s">
+        <v>522</v>
+      </c>
+      <c r="C1111">
+        <v>1</v>
+      </c>
+      <c r="D1111" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1111" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1111" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="1112" spans="1:10">
+      <c r="A1112" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1112" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="C1112" s="13">
+        <v>6.4679999999999703E-7</v>
+      </c>
+      <c r="D1112" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1112" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1112" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1113" spans="1:10">
+      <c r="A1113" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1113" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1113">
+        <v>2.7243999999999801E-3</v>
+      </c>
+      <c r="D1113" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1113" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1113" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1114" spans="1:10">
+      <c r="A1114" t="s">
+        <v>285</v>
+      </c>
+      <c r="B1114" s="13" t="s">
+        <v>170</v>
+      </c>
+      <c r="C1114">
+        <v>2.8801990359849587E-2</v>
+      </c>
+      <c r="D1114" t="s">
+        <v>91</v>
+      </c>
+      <c r="G1114" t="s">
+        <v>134</v>
+      </c>
+      <c r="H1114" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1115" spans="1:10">
+      <c r="A1115" t="s">
+        <v>138</v>
+      </c>
+      <c r="C1115">
+        <v>5.6806759804485539E-2</v>
+      </c>
+      <c r="D1115" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1115" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1115" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1115" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1116" spans="1:10">
+      <c r="A1116" t="s">
+        <v>110</v>
+      </c>
+      <c r="C1116">
+        <v>2.002793296089165E-6</v>
+      </c>
+      <c r="D1116" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1116" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1116" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1116" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="14" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added additional emissions to heat production using biomethane
</commit_message>
<xml_diff>
--- a/inventories/lci-Tr2050.xlsx
+++ b/inventories/lci-Tr2050.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engie-my.sharepoint.com/personal/db6421_engie_com/Documents/Documents/Local_repo/ADEME_scenarios_premise_gas/inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="225" documentId="13_ncr:1_{D0F9393E-493D-4D41-96B2-57E4008F0D51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC1276D8-0E19-4090-8BE4-B42B2CA7BEE6}"/>
+  <xr:revisionPtr revIDLastSave="244" documentId="13_ncr:1_{D0F9393E-493D-4D41-96B2-57E4008F0D51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2EDCD6C-09BE-4CDF-BF6D-716DA194E047}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="lci" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4632" uniqueCount="523">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4742" uniqueCount="536">
   <si>
     <t>Database</t>
   </si>
@@ -776,9 +776,6 @@
     <t>biomethane AD transport</t>
   </si>
   <si>
-    <t>heat, central or small-scale, biomethane</t>
-  </si>
-  <si>
     <t>methane, from electrochemical methanation, transport</t>
   </si>
   <si>
@@ -1605,6 +1602,48 @@
   </si>
   <si>
     <t>heat, biomethane</t>
+  </si>
+  <si>
+    <t>Acetic acid</t>
+  </si>
+  <si>
+    <t>Benzene</t>
+  </si>
+  <si>
+    <t>Benzo(a)pyrene</t>
+  </si>
+  <si>
+    <t>Dioxins, measured as 2,3,7,8-tetrachlorodibenzo-p-dioxin</t>
+  </si>
+  <si>
+    <t>Formaldehyde</t>
+  </si>
+  <si>
+    <t>Mercury II</t>
+  </si>
+  <si>
+    <t>PAH, polycyclic aromatic hydrocarbons</t>
+  </si>
+  <si>
+    <t>Particulate Matter, &lt; 2.5 um</t>
+  </si>
+  <si>
+    <t>Pentane</t>
+  </si>
+  <si>
+    <t>Propionic acid</t>
+  </si>
+  <si>
+    <t>Toluene</t>
+  </si>
+  <si>
+    <t>Nitrite</t>
+  </si>
+  <si>
+    <t>Sulfate</t>
+  </si>
+  <si>
+    <t>Sulfite</t>
   </si>
 </sst>
 </file>
@@ -2141,7 +2180,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AH1116"/>
+  <dimension ref="A1:AH1138"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="73.140625" customWidth="1"/>
@@ -3718,7 +3757,7 @@
         <v>11</v>
       </c>
       <c r="B79" s="26" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C79" s="25"/>
       <c r="D79" s="26"/>
@@ -4824,7 +4863,7 @@
         <v>11</v>
       </c>
       <c r="B103" s="26" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C103" s="25"/>
       <c r="D103" s="26"/>
@@ -5880,7 +5919,7 @@
         <v>11</v>
       </c>
       <c r="B126" s="26" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C126" s="25"/>
       <c r="D126" s="26"/>
@@ -6936,7 +6975,7 @@
         <v>11</v>
       </c>
       <c r="B149" s="26" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C149" s="25"/>
       <c r="D149" s="26"/>
@@ -8020,7 +8059,7 @@
         <v>11</v>
       </c>
       <c r="B173" s="26" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C173" s="25"/>
       <c r="D173" s="26"/>
@@ -8889,7 +8928,7 @@
         <v>11</v>
       </c>
       <c r="B197" s="26" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C197" s="25"/>
       <c r="D197" s="26"/>
@@ -9266,10 +9305,10 @@
     </row>
     <row r="206" spans="1:34">
       <c r="A206" s="26" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B206" s="26" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C206" s="32">
         <v>5.225162630331126</v>
@@ -9924,7 +9963,7 @@
         <v>11</v>
       </c>
       <c r="B221" s="26" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C221" s="25"/>
       <c r="D221" s="26"/>
@@ -10738,7 +10777,7 @@
         <v>11</v>
       </c>
       <c r="B245" s="26" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C245" s="25"/>
       <c r="D245" s="26"/>
@@ -11517,7 +11556,7 @@
         <v>1</v>
       </c>
       <c r="B268" s="24" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C268" s="22"/>
       <c r="D268" s="22"/>
@@ -11577,7 +11616,7 @@
         <v>4</v>
       </c>
       <c r="B271" s="22" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C271" s="22"/>
       <c r="D271" s="22"/>
@@ -11597,7 +11636,7 @@
         <v>57</v>
       </c>
       <c r="B272" s="31" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="C272" s="22"/>
       <c r="D272" s="22"/>
@@ -11681,10 +11720,10 @@
     </row>
     <row r="276" spans="1:14">
       <c r="A276" s="22" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B276" s="22" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C276" s="22">
         <v>1</v>
@@ -11707,10 +11746,10 @@
     </row>
     <row r="277" spans="1:14">
       <c r="A277" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B277" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C277" s="13">
         <v>0.21599526407159997</v>
@@ -11728,7 +11767,7 @@
         <v>12</v>
       </c>
       <c r="I277" s="22" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="K277" s="22"/>
       <c r="L277" s="22"/>
@@ -11737,10 +11776,10 @@
     </row>
     <row r="278" spans="1:14">
       <c r="A278" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B278" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="C278" s="13">
         <v>3.331311572796599E-2</v>
@@ -11758,7 +11797,7 @@
         <v>12</v>
       </c>
       <c r="I278" s="22" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="K278" s="22"/>
       <c r="L278" s="22"/>
@@ -11767,10 +11806,10 @@
     </row>
     <row r="279" spans="1:14">
       <c r="A279" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B279" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C279" s="13">
         <v>6.2514013928414991E-2</v>
@@ -11788,7 +11827,7 @@
         <v>12</v>
       </c>
       <c r="I279" s="22" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="K279" s="22"/>
       <c r="L279" s="22"/>
@@ -11818,7 +11857,7 @@
         <v>12</v>
       </c>
       <c r="I280" s="22" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="K280" s="22"/>
       <c r="L280" s="22"/>
@@ -11855,10 +11894,10 @@
     </row>
     <row r="282" spans="1:14">
       <c r="A282" t="s">
+        <v>319</v>
+      </c>
+      <c r="B282" t="s">
         <v>320</v>
-      </c>
-      <c r="B282" t="s">
-        <v>321</v>
       </c>
       <c r="C282" s="13">
         <v>5.9291219999999993E-3</v>
@@ -11883,10 +11922,10 @@
     </row>
     <row r="283" spans="1:14">
       <c r="A283" t="s">
+        <v>321</v>
+      </c>
+      <c r="B283" t="s">
         <v>322</v>
-      </c>
-      <c r="B283" t="s">
-        <v>323</v>
       </c>
       <c r="C283" s="13">
         <v>5.9960509999999988E-3</v>
@@ -11911,10 +11950,10 @@
     </row>
     <row r="284" spans="1:14">
       <c r="A284" s="59" t="s">
+        <v>323</v>
+      </c>
+      <c r="B284" t="s">
         <v>324</v>
-      </c>
-      <c r="B284" t="s">
-        <v>325</v>
       </c>
       <c r="C284" s="13">
         <v>5.7362089999999998E-2</v>
@@ -11939,10 +11978,10 @@
     </row>
     <row r="285" spans="1:14">
       <c r="A285" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="B285" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="C285" s="13">
         <v>4.9173129999999992E-7</v>
@@ -11960,7 +11999,7 @@
         <v>12</v>
       </c>
       <c r="I285" s="22" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="K285" s="22"/>
       <c r="L285" s="22"/>
@@ -11969,10 +12008,10 @@
     </row>
     <row r="286" spans="1:14">
       <c r="A286" t="s">
+        <v>317</v>
+      </c>
+      <c r="B286" t="s">
         <v>318</v>
-      </c>
-      <c r="B286" t="s">
-        <v>319</v>
       </c>
       <c r="C286" s="13">
         <v>2.3043064149999999E-4</v>
@@ -11990,7 +12029,7 @@
         <v>12</v>
       </c>
       <c r="I286" s="22" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="K286" s="22"/>
       <c r="L286" s="22"/>
@@ -11999,10 +12038,10 @@
     </row>
     <row r="287" spans="1:14">
       <c r="A287" t="s">
+        <v>315</v>
+      </c>
+      <c r="B287" t="s">
         <v>316</v>
-      </c>
-      <c r="B287" t="s">
-        <v>317</v>
       </c>
       <c r="C287" s="13">
         <v>3.2200000000000002E-3</v>
@@ -12020,7 +12059,7 @@
         <v>12</v>
       </c>
       <c r="I287" s="22" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="K287" s="22"/>
       <c r="L287" s="22"/>
@@ -12029,10 +12068,10 @@
     </row>
     <row r="288" spans="1:14">
       <c r="A288" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="B288" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="C288" s="13">
         <v>8.2529999999999998E-5</v>
@@ -12050,7 +12089,7 @@
         <v>12</v>
       </c>
       <c r="I288" s="22" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="J288" s="22"/>
       <c r="K288" s="22"/>
@@ -12060,10 +12099,10 @@
     </row>
     <row r="289" spans="1:14">
       <c r="A289" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="B289" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="C289" s="13">
         <v>0.24474000000000001</v>
@@ -12081,7 +12120,7 @@
         <v>12</v>
       </c>
       <c r="I289" s="22" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="J289" s="22"/>
       <c r="K289" s="22"/>
@@ -12111,7 +12150,7 @@
         <v>15</v>
       </c>
       <c r="I290" s="22" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="J290" s="22"/>
       <c r="K290" s="22"/>
@@ -12121,7 +12160,7 @@
     </row>
     <row r="291" spans="1:14">
       <c r="A291" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C291" s="13">
         <v>13.622223068650793</v>
@@ -12134,13 +12173,13 @@
       </c>
       <c r="F291" s="22"/>
       <c r="G291" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="H291" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I291" s="22" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="J291" s="22"/>
       <c r="K291" s="22"/>
@@ -12169,7 +12208,7 @@
         <v>15</v>
       </c>
       <c r="I292" s="22" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="J292" s="22"/>
       <c r="K292" s="22"/>
@@ -12179,7 +12218,7 @@
     </row>
     <row r="293" spans="1:14">
       <c r="A293" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="C293" s="13">
         <v>3.6196777999999996E-4</v>
@@ -12198,7 +12237,7 @@
         <v>15</v>
       </c>
       <c r="I293" s="22" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="J293" s="22"/>
       <c r="K293" s="22"/>
@@ -12227,7 +12266,7 @@
         <v>15</v>
       </c>
       <c r="I294" s="22" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="J294" s="22"/>
       <c r="K294" s="22"/>
@@ -12256,7 +12295,7 @@
         <v>15</v>
       </c>
       <c r="I295" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J295" s="22"/>
       <c r="K295" s="22"/>
@@ -12285,7 +12324,7 @@
         <v>15</v>
       </c>
       <c r="I296" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J296" s="22"/>
       <c r="K296" s="22"/>
@@ -12314,7 +12353,7 @@
         <v>15</v>
       </c>
       <c r="I297" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J297" s="22"/>
       <c r="K297" s="22"/>
@@ -12324,7 +12363,7 @@
     </row>
     <row r="298" spans="1:14">
       <c r="A298" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C298" s="13">
         <v>0.47991081325301199</v>
@@ -12343,7 +12382,7 @@
         <v>15</v>
       </c>
       <c r="I298" s="22" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="J298" s="22"/>
       <c r="K298" s="22"/>
@@ -12353,7 +12392,7 @@
     </row>
     <row r="299" spans="1:14">
       <c r="A299" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C299" s="13">
         <v>0.47991081325301199</v>
@@ -12372,7 +12411,7 @@
         <v>15</v>
       </c>
       <c r="I299" s="22" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="J299" s="22"/>
       <c r="K299" s="22"/>
@@ -12382,7 +12421,7 @@
     </row>
     <row r="300" spans="1:14">
       <c r="A300" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C300" s="13">
         <v>0.95982162650602398</v>
@@ -12401,7 +12440,7 @@
         <v>15</v>
       </c>
       <c r="I300" s="22" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J300" s="22"/>
       <c r="K300" s="22"/>
@@ -12411,7 +12450,7 @@
     </row>
     <row r="301" spans="1:14">
       <c r="A301" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C301" s="13">
         <v>1.0107999999999999E-6</v>
@@ -12424,13 +12463,13 @@
       </c>
       <c r="F301" s="22"/>
       <c r="G301" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H301" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I301" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J301" s="22"/>
       <c r="K301" s="22"/>
@@ -12440,7 +12479,7 @@
     </row>
     <row r="302" spans="1:14">
       <c r="A302" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C302" s="13">
         <v>6.1366999999999996E-7</v>
@@ -12453,13 +12492,13 @@
       </c>
       <c r="F302" s="22"/>
       <c r="G302" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H302" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I302" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J302" s="22"/>
       <c r="K302" s="22"/>
@@ -12469,7 +12508,7 @@
     </row>
     <row r="303" spans="1:14">
       <c r="A303" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C303" s="13">
         <v>4.8131000000000003E-9</v>
@@ -12482,13 +12521,13 @@
       </c>
       <c r="F303" s="22"/>
       <c r="G303" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H303" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I303" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J303" s="22"/>
       <c r="K303" s="22"/>
@@ -12498,7 +12537,7 @@
     </row>
     <row r="304" spans="1:14">
       <c r="A304" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C304" s="13">
         <v>6.4977000000000003E-7</v>
@@ -12511,13 +12550,13 @@
       </c>
       <c r="F304" s="22"/>
       <c r="G304" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H304" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I304" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J304" s="22"/>
       <c r="K304" s="22"/>
@@ -12527,7 +12566,7 @@
     </row>
     <row r="305" spans="1:14">
       <c r="A305" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C305" s="13">
         <v>-1.5040999999999999E-6</v>
@@ -12540,13 +12579,13 @@
       </c>
       <c r="F305" s="22"/>
       <c r="G305" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H305" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I305" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J305" s="22"/>
       <c r="K305" s="22"/>
@@ -12556,7 +12595,7 @@
     </row>
     <row r="306" spans="1:14">
       <c r="A306" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C306" s="13">
         <v>1.2032999999999999E-7</v>
@@ -12569,13 +12608,13 @@
       </c>
       <c r="F306" s="22"/>
       <c r="G306" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H306" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I306" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J306" s="22"/>
       <c r="K306" s="22"/>
@@ -12585,7 +12624,7 @@
     </row>
     <row r="307" spans="1:14">
       <c r="A307" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C307" s="13">
         <v>2.4787000000000001E-6</v>
@@ -12598,13 +12637,13 @@
       </c>
       <c r="F307" s="22"/>
       <c r="G307" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H307" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I307" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J307" s="22"/>
       <c r="K307" s="22"/>
@@ -12614,7 +12653,7 @@
     </row>
     <row r="308" spans="1:14">
       <c r="A308" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C308" s="13">
         <v>1.0829E-7</v>
@@ -12627,13 +12666,13 @@
       </c>
       <c r="F308" s="22"/>
       <c r="G308" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H308" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I308" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J308" s="22"/>
       <c r="K308" s="22"/>
@@ -12643,7 +12682,7 @@
     </row>
     <row r="309" spans="1:14">
       <c r="A309" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C309" s="13">
         <v>1.0107999999999999E-6</v>
@@ -12656,13 +12695,13 @@
       </c>
       <c r="F309" s="22"/>
       <c r="G309" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H309" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I309" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J309" s="22"/>
       <c r="K309" s="22"/>
@@ -12672,7 +12711,7 @@
     </row>
     <row r="310" spans="1:14">
       <c r="A310" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C310" s="13">
         <v>2.4065000000000001E-8</v>
@@ -12685,13 +12724,13 @@
       </c>
       <c r="F310" s="22"/>
       <c r="G310" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H310" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I310" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J310" s="22"/>
       <c r="K310" s="22"/>
@@ -12701,7 +12740,7 @@
     </row>
     <row r="311" spans="1:14">
       <c r="A311" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C311" s="13">
         <v>-3.2893999999999998E-7</v>
@@ -12714,13 +12753,13 @@
       </c>
       <c r="F311" s="22"/>
       <c r="G311" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H311" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I311" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J311" s="22"/>
       <c r="K311" s="22"/>
@@ -12730,7 +12769,7 @@
     </row>
     <row r="312" spans="1:14">
       <c r="A312" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C312" s="13">
         <v>7.9416000000000001E-7</v>
@@ -12743,13 +12782,13 @@
       </c>
       <c r="F312" s="22"/>
       <c r="G312" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H312" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I312" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J312" s="22"/>
       <c r="K312" s="22"/>
@@ -12759,7 +12798,7 @@
     </row>
     <row r="313" spans="1:14">
       <c r="A313" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C313" s="13">
         <v>4.1393000000000003E-6</v>
@@ -12772,13 +12811,13 @@
       </c>
       <c r="F313" s="22"/>
       <c r="G313" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H313" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I313" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J313" s="22"/>
       <c r="K313" s="22"/>
@@ -12788,7 +12827,7 @@
     </row>
     <row r="314" spans="1:14">
       <c r="A314" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C314" s="13">
         <v>5.0537999999999999E-8</v>
@@ -12801,13 +12840,13 @@
       </c>
       <c r="F314" s="22"/>
       <c r="G314" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H314" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I314" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J314" s="22"/>
       <c r="K314" s="22"/>
@@ -12817,7 +12856,7 @@
     </row>
     <row r="315" spans="1:14">
       <c r="A315" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C315" s="13">
         <v>-5.9000999999999996E-6</v>
@@ -12830,13 +12869,13 @@
       </c>
       <c r="F315" s="22"/>
       <c r="G315" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H315" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I315" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J315" s="22"/>
       <c r="K315" s="22"/>
@@ -12846,7 +12885,7 @@
     </row>
     <row r="316" spans="1:14">
       <c r="A316" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C316" s="13">
         <v>1.5643E-6</v>
@@ -12859,13 +12898,13 @@
       </c>
       <c r="F316" s="22"/>
       <c r="G316" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H316" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I316" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J316" s="22"/>
       <c r="K316" s="22"/>
@@ -12875,7 +12914,7 @@
     </row>
     <row r="317" spans="1:14">
       <c r="A317" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C317" s="13">
         <v>2.6952999999999998E-6</v>
@@ -12888,13 +12927,13 @@
       </c>
       <c r="F317" s="22"/>
       <c r="G317" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H317" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I317" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J317" s="22"/>
       <c r="K317" s="22"/>
@@ -12904,7 +12943,7 @@
     </row>
     <row r="318" spans="1:14">
       <c r="A318" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C318" s="13">
         <v>4.4454999999999997E-8</v>
@@ -12917,13 +12956,13 @@
       </c>
       <c r="F318" s="22"/>
       <c r="G318" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H318" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I318" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J318" s="22"/>
       <c r="K318" s="22"/>
@@ -12933,7 +12972,7 @@
     </row>
     <row r="319" spans="1:14">
       <c r="A319" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C319" s="13">
         <v>3.6097999999999997E-8</v>
@@ -12946,13 +12985,13 @@
       </c>
       <c r="F319" s="22"/>
       <c r="G319" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H319" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I319" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J319" s="22"/>
       <c r="K319" s="22"/>
@@ -12962,7 +13001,7 @@
     </row>
     <row r="320" spans="1:14">
       <c r="A320" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C320" s="13">
         <v>2.1659000000000001E-7</v>
@@ -12975,13 +13014,13 @@
       </c>
       <c r="F320" s="22"/>
       <c r="G320" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H320" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I320" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J320" s="22"/>
       <c r="K320" s="22"/>
@@ -12991,7 +13030,7 @@
     </row>
     <row r="321" spans="1:14">
       <c r="A321" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="C321" s="13">
         <v>-1.8835E-8</v>
@@ -13004,13 +13043,13 @@
       </c>
       <c r="F321" s="22"/>
       <c r="G321" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H321" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I321" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J321" s="22"/>
       <c r="K321" s="22"/>
@@ -13020,7 +13059,7 @@
     </row>
     <row r="322" spans="1:14">
       <c r="A322" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C322" s="13">
         <v>4.2885E-5</v>
@@ -13033,13 +13072,13 @@
       </c>
       <c r="F322" s="22"/>
       <c r="G322" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H322" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I322" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J322" s="22"/>
       <c r="K322" s="22"/>
@@ -13049,7 +13088,7 @@
     </row>
     <row r="323" spans="1:14">
       <c r="A323" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C323" s="13">
         <v>9.2460000000000006E-5</v>
@@ -13062,13 +13101,13 @@
       </c>
       <c r="F323" s="22"/>
       <c r="G323" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H323" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I323" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J323" s="22"/>
       <c r="K323" s="22"/>
@@ -13078,7 +13117,7 @@
     </row>
     <row r="324" spans="1:14">
       <c r="A324" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C324" s="13">
         <v>5.0297000000000003E-6</v>
@@ -13091,13 +13130,13 @@
       </c>
       <c r="F324" s="22"/>
       <c r="G324" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H324" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I324" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J324" s="22"/>
       <c r="K324" s="22"/>
@@ -13107,7 +13146,7 @@
     </row>
     <row r="325" spans="1:14">
       <c r="A325" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C325" s="13">
         <v>2.4306000000000001E-6</v>
@@ -13120,13 +13159,13 @@
       </c>
       <c r="F325" s="22"/>
       <c r="G325" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H325" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I325" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J325" s="22"/>
       <c r="K325" s="22"/>
@@ -13136,7 +13175,7 @@
     </row>
     <row r="326" spans="1:14">
       <c r="A326" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C326" s="13">
         <v>1.7326999999999999E-6</v>
@@ -13149,13 +13188,13 @@
       </c>
       <c r="F326" s="22"/>
       <c r="G326" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H326" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I326" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J326" s="22"/>
       <c r="K326" s="22"/>
@@ -13165,7 +13204,7 @@
     </row>
     <row r="327" spans="1:14">
       <c r="A327" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C327" s="13">
         <v>2.8878999999999998E-7</v>
@@ -13178,13 +13217,13 @@
       </c>
       <c r="F327" s="22"/>
       <c r="G327" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H327" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I327" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J327" s="22"/>
       <c r="K327" s="22"/>
@@ -13194,7 +13233,7 @@
     </row>
     <row r="328" spans="1:14">
       <c r="A328" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C328" s="13">
         <v>1.9661999999999999E-5</v>
@@ -13207,13 +13246,13 @@
       </c>
       <c r="F328" s="22"/>
       <c r="G328" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H328" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I328" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J328" s="22"/>
       <c r="K328" s="22"/>
@@ -13223,7 +13262,7 @@
     </row>
     <row r="329" spans="1:14">
       <c r="A329" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C329" s="13">
         <v>1.1911999999999999E-6</v>
@@ -13236,13 +13275,13 @@
       </c>
       <c r="F329" s="22"/>
       <c r="G329" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H329" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I329" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J329" s="22"/>
       <c r="K329" s="22"/>
@@ -13252,7 +13291,7 @@
     </row>
     <row r="330" spans="1:14">
       <c r="A330" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C330" s="13">
         <v>1.9252000000000001E-7</v>
@@ -13265,13 +13304,13 @@
       </c>
       <c r="F330" s="22"/>
       <c r="G330" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H330" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I330" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J330" s="22"/>
       <c r="K330" s="22"/>
@@ -13281,7 +13320,7 @@
     </row>
     <row r="331" spans="1:14">
       <c r="A331" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C331" s="13">
         <v>3.0442999999999998E-6</v>
@@ -13294,13 +13333,13 @@
       </c>
       <c r="F331" s="22"/>
       <c r="G331" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H331" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I331" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J331" s="22"/>
       <c r="K331" s="22"/>
@@ -13310,7 +13349,7 @@
     </row>
     <row r="332" spans="1:14">
       <c r="A332" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C332" s="13">
         <v>4.8130999999999997E-6</v>
@@ -13323,13 +13362,13 @@
       </c>
       <c r="F332" s="22"/>
       <c r="G332" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H332" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I332" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J332" s="22"/>
       <c r="K332" s="22"/>
@@ -13339,7 +13378,7 @@
     </row>
     <row r="333" spans="1:14">
       <c r="A333" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C333" s="13">
         <v>5.9441999999999998E-5</v>
@@ -13352,13 +13391,13 @@
       </c>
       <c r="F333" s="22"/>
       <c r="G333" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H333" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I333" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J333" s="22"/>
       <c r="K333" s="22"/>
@@ -13368,7 +13407,7 @@
     </row>
     <row r="334" spans="1:14">
       <c r="A334" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C334" s="13">
         <v>3.3691999999999998E-7</v>
@@ -13381,13 +13420,13 @@
       </c>
       <c r="F334" s="22"/>
       <c r="G334" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H334" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I334" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J334" s="22"/>
       <c r="K334" s="22"/>
@@ -13397,7 +13436,7 @@
     </row>
     <row r="335" spans="1:14">
       <c r="A335" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C335" s="13">
         <v>1.6846000000000001E-8</v>
@@ -13410,13 +13449,13 @@
       </c>
       <c r="F335" s="22"/>
       <c r="G335" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H335" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I335" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J335" s="22"/>
       <c r="K335" s="22"/>
@@ -13426,7 +13465,7 @@
     </row>
     <row r="336" spans="1:14">
       <c r="A336" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C336" s="13">
         <v>5.7757E-7</v>
@@ -13439,13 +13478,13 @@
       </c>
       <c r="F336" s="22"/>
       <c r="G336" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H336" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I336" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J336" s="22"/>
       <c r="K336" s="22"/>
@@ -13455,7 +13494,7 @@
     </row>
     <row r="337" spans="1:34">
       <c r="A337" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C337" s="13">
         <v>2.1658999999999999E-8</v>
@@ -13468,13 +13507,13 @@
       </c>
       <c r="F337" s="22"/>
       <c r="G337" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H337" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I337" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J337" s="22"/>
       <c r="K337" s="22"/>
@@ -13484,7 +13523,7 @@
     </row>
     <row r="338" spans="1:34">
       <c r="A338" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C338" s="13">
         <v>3.6097999999999997E-8</v>
@@ -13497,13 +13536,13 @@
       </c>
       <c r="F338" s="22"/>
       <c r="G338" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H338" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I338" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J338" s="22"/>
       <c r="K338" s="22"/>
@@ -13513,7 +13552,7 @@
     </row>
     <row r="339" spans="1:34">
       <c r="A339" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C339" s="13">
         <v>2.6472E-7</v>
@@ -13526,13 +13565,13 @@
       </c>
       <c r="F339" s="22"/>
       <c r="G339" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H339" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I339" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J339" s="22"/>
       <c r="K339" s="22"/>
@@ -13542,7 +13581,7 @@
     </row>
     <row r="340" spans="1:34">
       <c r="A340" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C340" s="13">
         <v>1.2032999999999999E-7</v>
@@ -13555,13 +13594,13 @@
       </c>
       <c r="F340" s="22"/>
       <c r="G340" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H340" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I340" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J340" s="22"/>
       <c r="K340" s="22"/>
@@ -13571,7 +13610,7 @@
     </row>
     <row r="341" spans="1:34">
       <c r="A341" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C341" s="13">
         <v>2.6436999999999998E-7</v>
@@ -13584,13 +13623,13 @@
       </c>
       <c r="F341" s="22"/>
       <c r="G341" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H341" s="22" t="s">
         <v>15</v>
       </c>
       <c r="I341" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J341" s="22"/>
       <c r="K341" s="22"/>
@@ -13619,7 +13658,7 @@
         <v>15</v>
       </c>
       <c r="I342" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J342" s="22"/>
       <c r="K342" s="22"/>
@@ -13648,7 +13687,7 @@
         <v>15</v>
       </c>
       <c r="I343" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J343" s="22"/>
       <c r="K343" s="22"/>
@@ -13677,7 +13716,7 @@
         <v>15</v>
       </c>
       <c r="I344" s="22" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J344" s="22"/>
       <c r="K344" s="22"/>
@@ -13687,7 +13726,7 @@
     </row>
     <row r="345" spans="1:34">
       <c r="A345" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C345" s="13">
         <v>9.7541999999999995E-5</v>
@@ -13706,7 +13745,7 @@
         <v>15</v>
       </c>
       <c r="I345" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J345" s="22"/>
       <c r="K345" s="22"/>
@@ -13716,7 +13755,7 @@
     </row>
     <row r="346" spans="1:34">
       <c r="A346" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C346" s="13">
         <v>7.5147999999999996E-6</v>
@@ -13733,7 +13772,7 @@
         <v>15</v>
       </c>
       <c r="I346" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J346" s="22"/>
       <c r="K346" s="22"/>
@@ -13743,7 +13782,7 @@
     </row>
     <row r="347" spans="1:34">
       <c r="A347" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C347" s="13">
         <v>0</v>
@@ -13760,7 +13799,7 @@
         <v>15</v>
       </c>
       <c r="I347" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="J347" s="22"/>
       <c r="K347" s="22"/>
@@ -13824,7 +13863,7 @@
         <v>11</v>
       </c>
       <c r="B350" s="26" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C350" s="25"/>
       <c r="D350" s="26"/>
@@ -14000,10 +14039,10 @@
     </row>
     <row r="360" spans="1:34">
       <c r="A360" s="31" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B360" s="22" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C360" s="32">
         <v>1</v>
@@ -14131,7 +14170,7 @@
         <v>11</v>
       </c>
       <c r="B365" s="26" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C365" s="25"/>
       <c r="D365" s="26"/>
@@ -14418,7 +14457,7 @@
         <v>11</v>
       </c>
       <c r="B379" s="26" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C379" s="25"/>
       <c r="D379" s="26"/>
@@ -14678,7 +14717,7 @@
         <v>11</v>
       </c>
       <c r="B391" s="26" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C391" s="25"/>
       <c r="D391" s="26"/>
@@ -15242,7 +15281,7 @@
         <v>11</v>
       </c>
       <c r="B405" s="26" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C405" s="25"/>
       <c r="D405" s="26"/>
@@ -15516,7 +15555,7 @@
         <v>1</v>
       </c>
       <c r="B418" s="24" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C418" s="25"/>
       <c r="D418" s="26"/>
@@ -15556,7 +15595,7 @@
         <v>11</v>
       </c>
       <c r="B419" s="26" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C419" s="25"/>
       <c r="D419" s="26"/>
@@ -15636,7 +15675,7 @@
         <v>4</v>
       </c>
       <c r="B421" s="26" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C421" s="25"/>
       <c r="D421" s="26"/>
@@ -15756,7 +15795,7 @@
         <v>57</v>
       </c>
       <c r="B424" s="26" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C424" s="25"/>
       <c r="D424" s="29"/>
@@ -15885,10 +15924,10 @@
     </row>
     <row r="427" spans="1:34">
       <c r="A427" s="31" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B427" s="31" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C427" s="32">
         <v>1</v>
@@ -15987,10 +16026,10 @@
     </row>
     <row r="429" spans="1:34">
       <c r="A429" s="31" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B429" s="31" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C429" s="32">
         <v>0</v>
@@ -16037,10 +16076,10 @@
     </row>
     <row r="430" spans="1:34">
       <c r="A430" s="31" t="s">
+        <v>257</v>
+      </c>
+      <c r="B430" s="31" t="s">
         <v>258</v>
-      </c>
-      <c r="B430" s="31" t="s">
-        <v>259</v>
       </c>
       <c r="C430" s="32">
         <v>0</v>
@@ -16087,10 +16126,10 @@
     </row>
     <row r="431" spans="1:34">
       <c r="A431" s="31" t="s">
+        <v>259</v>
+      </c>
+      <c r="B431" s="31" t="s">
         <v>260</v>
-      </c>
-      <c r="B431" s="31" t="s">
-        <v>261</v>
       </c>
       <c r="C431" s="32">
         <v>1</v>
@@ -16137,10 +16176,10 @@
     </row>
     <row r="432" spans="1:34">
       <c r="A432" s="31" t="s">
+        <v>263</v>
+      </c>
+      <c r="B432" s="31" t="s">
         <v>264</v>
-      </c>
-      <c r="B432" s="31" t="s">
-        <v>265</v>
       </c>
       <c r="C432" s="32">
         <v>0</v>
@@ -16187,10 +16226,10 @@
     </row>
     <row r="433" spans="1:34">
       <c r="A433" s="31" t="s">
+        <v>265</v>
+      </c>
+      <c r="B433" s="31" t="s">
         <v>266</v>
-      </c>
-      <c r="B433" s="31" t="s">
-        <v>267</v>
       </c>
       <c r="C433" s="32">
         <v>0</v>
@@ -16237,10 +16276,10 @@
     </row>
     <row r="434" spans="1:34">
       <c r="A434" s="31" t="s">
+        <v>267</v>
+      </c>
+      <c r="B434" s="31" t="s">
         <v>268</v>
-      </c>
-      <c r="B434" s="31" t="s">
-        <v>269</v>
       </c>
       <c r="C434" s="32">
         <v>0</v>
@@ -16259,7 +16298,7 @@
         <v>12</v>
       </c>
       <c r="I434" s="31" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="J434" s="31"/>
       <c r="K434" s="31"/>
@@ -16289,10 +16328,10 @@
     </row>
     <row r="435" spans="1:34">
       <c r="A435" s="31" t="s">
+        <v>301</v>
+      </c>
+      <c r="B435" s="31" t="s">
         <v>302</v>
-      </c>
-      <c r="B435" s="31" t="s">
-        <v>303</v>
       </c>
       <c r="C435" s="32">
         <v>0</v>
@@ -16378,7 +16417,7 @@
         <v>1</v>
       </c>
       <c r="B437" s="24" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C437" s="25"/>
       <c r="D437" s="26"/>
@@ -16418,7 +16457,7 @@
         <v>11</v>
       </c>
       <c r="B438" s="26" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C438" s="25"/>
       <c r="D438" s="26"/>
@@ -16498,7 +16537,7 @@
         <v>4</v>
       </c>
       <c r="B440" s="26" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C440" s="25"/>
       <c r="D440" s="26"/>
@@ -16618,7 +16657,7 @@
         <v>57</v>
       </c>
       <c r="B443" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C443" s="25"/>
       <c r="D443" s="29"/>
@@ -16747,10 +16786,10 @@
     </row>
     <row r="446" spans="1:34">
       <c r="A446" s="31" t="s">
+        <v>259</v>
+      </c>
+      <c r="B446" s="31" t="s">
         <v>260</v>
-      </c>
-      <c r="B446" s="31" t="s">
-        <v>261</v>
       </c>
       <c r="C446" s="32">
         <v>1</v>
@@ -16937,7 +16976,7 @@
         <v>11</v>
       </c>
       <c r="B452" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="453" spans="1:9">
@@ -17151,7 +17190,7 @@
     </row>
     <row r="466" spans="1:9">
       <c r="A466" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B466" s="13" t="s">
         <v>121</v>
@@ -17334,7 +17373,7 @@
         <v>11</v>
       </c>
       <c r="B476" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="477" spans="1:9">
@@ -17548,7 +17587,7 @@
     </row>
     <row r="490" spans="1:9">
       <c r="A490" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B490" s="13" t="s">
         <v>121</v>
@@ -17911,7 +17950,7 @@
         <v>11</v>
       </c>
       <c r="B508" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="509" spans="1:8">
@@ -18125,7 +18164,7 @@
     </row>
     <row r="522" spans="1:9">
       <c r="A522" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B522" s="13" t="s">
         <v>121</v>
@@ -18488,7 +18527,7 @@
         <v>11</v>
       </c>
       <c r="B540" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="541" spans="1:8">
@@ -18702,7 +18741,7 @@
     </row>
     <row r="554" spans="1:9">
       <c r="A554" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B554" s="13" t="s">
         <v>121</v>
@@ -19065,7 +19104,7 @@
         <v>11</v>
       </c>
       <c r="B572" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="573" spans="1:8">
@@ -19279,7 +19318,7 @@
     </row>
     <row r="586" spans="1:9">
       <c r="A586" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B586" s="13" t="s">
         <v>121</v>
@@ -19642,7 +19681,7 @@
         <v>11</v>
       </c>
       <c r="B604" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="605" spans="1:8">
@@ -19856,7 +19895,7 @@
     </row>
     <row r="618" spans="1:9">
       <c r="A618" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B618" s="13" t="s">
         <v>121</v>
@@ -20039,7 +20078,7 @@
         <v>11</v>
       </c>
       <c r="B628" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="629" spans="1:9">
@@ -20253,7 +20292,7 @@
     </row>
     <row r="642" spans="1:9">
       <c r="A642" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B642" s="13" t="s">
         <v>121</v>
@@ -20616,7 +20655,7 @@
         <v>11</v>
       </c>
       <c r="B660" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="661" spans="1:9">
@@ -20830,7 +20869,7 @@
     </row>
     <row r="674" spans="1:9">
       <c r="A674" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B674" s="13" t="s">
         <v>121</v>
@@ -21193,7 +21232,7 @@
         <v>11</v>
       </c>
       <c r="B692" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="693" spans="1:9">
@@ -21407,7 +21446,7 @@
     </row>
     <row r="706" spans="1:9">
       <c r="A706" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B706" s="13" t="s">
         <v>121</v>
@@ -21770,7 +21809,7 @@
         <v>11</v>
       </c>
       <c r="B724" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="725" spans="1:9">
@@ -21985,7 +22024,7 @@
     </row>
     <row r="738" spans="1:9">
       <c r="A738" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B738" s="13" t="s">
         <v>121</v>
@@ -22348,7 +22387,7 @@
         <v>11</v>
       </c>
       <c r="B756" s="13" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="757" spans="1:20">
@@ -22561,10 +22600,10 @@
     </row>
     <row r="769" spans="1:11" s="26" customFormat="1">
       <c r="A769" s="31" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B769" s="31" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C769" s="45">
         <v>1</v>
@@ -23294,7 +23333,7 @@
         <v>11</v>
       </c>
       <c r="B811" s="31" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="812" spans="1:11" s="26" customFormat="1">
@@ -23402,10 +23441,10 @@
     </row>
     <row r="820" spans="1:9">
       <c r="A820" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B820" s="31" t="s">
-        <v>246</v>
+        <v>521</v>
       </c>
       <c r="C820" s="46">
         <v>0.1764792</v>
@@ -23441,7 +23480,7 @@
         <v>12</v>
       </c>
       <c r="I821" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="822" spans="1:9">
@@ -23465,7 +23504,7 @@
         <v>15</v>
       </c>
       <c r="I822" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="823" spans="1:9">
@@ -23489,7 +23528,7 @@
         <v>15</v>
       </c>
       <c r="I823" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="824" spans="1:9" s="49" customFormat="1">
@@ -23500,7 +23539,7 @@
         <v>1</v>
       </c>
       <c r="B825" s="43" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C825" s="25"/>
     </row>
@@ -23509,7 +23548,7 @@
         <v>11</v>
       </c>
       <c r="B826" s="31" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="827" spans="1:9" s="26" customFormat="1">
@@ -23526,7 +23565,7 @@
         <v>4</v>
       </c>
       <c r="B828" s="31" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C828" s="25"/>
     </row>
@@ -23595,10 +23634,10 @@
     </row>
     <row r="834" spans="1:9" s="26" customFormat="1">
       <c r="A834" s="31" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B834" s="31" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C834" s="45">
         <v>1</v>
@@ -23618,10 +23657,10 @@
     </row>
     <row r="835" spans="1:9">
       <c r="A835" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B835" s="31" t="s">
-        <v>246</v>
+        <v>521</v>
       </c>
       <c r="C835" s="46">
         <v>0.1764792</v>
@@ -23657,7 +23696,7 @@
         <v>12</v>
       </c>
       <c r="I836" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="837" spans="1:9">
@@ -23681,7 +23720,7 @@
         <v>15</v>
       </c>
       <c r="I837" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="838" spans="1:9" s="49" customFormat="1">
@@ -23692,7 +23731,7 @@
         <v>1</v>
       </c>
       <c r="B839" s="43" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C839" s="25"/>
       <c r="D839" s="26"/>
@@ -23707,7 +23746,7 @@
         <v>11</v>
       </c>
       <c r="B840" s="31" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C840" s="26"/>
       <c r="D840" s="26"/>
@@ -23834,7 +23873,7 @@
     </row>
     <row r="848" spans="1:9">
       <c r="A848" s="31" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B848" s="31" t="s">
         <v>99</v>
@@ -23856,10 +23895,10 @@
     </row>
     <row r="849" spans="1:9">
       <c r="A849" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B849" s="13" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C849" s="41">
         <v>0.1764792</v>
@@ -23874,12 +23913,12 @@
         <v>12</v>
       </c>
       <c r="I849" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="850" spans="1:9">
       <c r="A850" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B850" s="13" t="s">
         <v>99</v>
@@ -23899,7 +23938,7 @@
     </row>
     <row r="851" spans="1:9">
       <c r="A851" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B851" s="13" t="s">
         <v>99</v>
@@ -23919,7 +23958,7 @@
     </row>
     <row r="852" spans="1:9">
       <c r="A852" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B852" s="13" t="s">
         <v>99</v>
@@ -23939,7 +23978,7 @@
     </row>
     <row r="853" spans="1:9">
       <c r="A853" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B853" s="13" t="s">
         <v>99</v>
@@ -23959,7 +23998,7 @@
     </row>
     <row r="854" spans="1:9">
       <c r="A854" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B854" s="13" t="s">
         <v>99</v>
@@ -23979,7 +24018,7 @@
     </row>
     <row r="855" spans="1:9">
       <c r="A855" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B855" s="13" t="s">
         <v>99</v>
@@ -23999,7 +24038,7 @@
     </row>
     <row r="856" spans="1:9">
       <c r="A856" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B856" s="13" t="s">
         <v>99</v>
@@ -24038,7 +24077,7 @@
         <v>15</v>
       </c>
       <c r="I857" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="858" spans="1:9">
@@ -24062,12 +24101,12 @@
         <v>15</v>
       </c>
       <c r="I858" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="859" spans="1:9">
       <c r="A859" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C859" s="13">
         <v>5.5436706695375997E-4</v>
@@ -24086,7 +24125,7 @@
         <v>15</v>
       </c>
       <c r="I859" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="860" spans="1:9">
@@ -24109,7 +24148,7 @@
         <v>15</v>
       </c>
       <c r="I860" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="861" spans="1:9">
@@ -24133,7 +24172,7 @@
         <v>15</v>
       </c>
       <c r="I861" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="862" spans="1:9">
@@ -24157,7 +24196,7 @@
         <v>15</v>
       </c>
       <c r="I862" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="863" spans="1:9">
@@ -24176,7 +24215,7 @@
         <v>1</v>
       </c>
       <c r="B864" s="43" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C864" s="25"/>
       <c r="D864" s="26"/>
@@ -24191,7 +24230,7 @@
         <v>11</v>
       </c>
       <c r="B865" s="31" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C865" s="26"/>
       <c r="D865" s="26"/>
@@ -24266,7 +24305,7 @@
         <v>57</v>
       </c>
       <c r="B870" s="26" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C870" s="25"/>
       <c r="D870" s="29"/>
@@ -24320,7 +24359,7 @@
     </row>
     <row r="873" spans="1:9">
       <c r="A873" s="31" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B873" s="31" t="s">
         <v>170</v>
@@ -24342,7 +24381,7 @@
     </row>
     <row r="874" spans="1:9">
       <c r="A874" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B874" s="31" t="s">
         <v>170</v>
@@ -24376,7 +24415,7 @@
         <v>1</v>
       </c>
       <c r="B876" s="43" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C876" s="25"/>
       <c r="D876" s="26"/>
@@ -24391,7 +24430,7 @@
         <v>11</v>
       </c>
       <c r="B877" s="31" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C877" s="26"/>
       <c r="D877" s="26"/>
@@ -24421,7 +24460,7 @@
         <v>4</v>
       </c>
       <c r="B879" s="31" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C879" s="25"/>
       <c r="D879" s="26"/>
@@ -24518,10 +24557,10 @@
     </row>
     <row r="885" spans="1:10">
       <c r="A885" s="31" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B885" s="31" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C885" s="26">
         <v>1</v>
@@ -24554,7 +24593,7 @@
         <v>1</v>
       </c>
       <c r="B887" s="43" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="888" spans="1:10">
@@ -24581,7 +24620,7 @@
         <v>4</v>
       </c>
       <c r="B890" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="F890" s="13"/>
       <c r="J890" s="56"/>
@@ -24667,7 +24706,7 @@
         <v>15</v>
       </c>
       <c r="I896" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="897" spans="1:9">
@@ -24691,7 +24730,7 @@
         <v>15</v>
       </c>
       <c r="I897" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="898" spans="1:9">
@@ -24715,7 +24754,7 @@
         <v>15</v>
       </c>
       <c r="I898" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="899" spans="1:9">
@@ -24744,7 +24783,7 @@
     </row>
     <row r="900" spans="1:9">
       <c r="A900" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B900"/>
       <c r="C900">
@@ -24789,7 +24828,7 @@
     </row>
     <row r="902" spans="1:9">
       <c r="A902" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B902"/>
       <c r="C902">
@@ -24813,10 +24852,10 @@
     </row>
     <row r="903" spans="1:9">
       <c r="A903" t="s">
+        <v>385</v>
+      </c>
+      <c r="B903" t="s">
         <v>386</v>
-      </c>
-      <c r="B903" t="s">
-        <v>387</v>
       </c>
       <c r="C903">
         <v>1</v>
@@ -24836,7 +24875,7 @@
     </row>
     <row r="904" spans="1:9">
       <c r="A904" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B904"/>
       <c r="C904">
@@ -24852,12 +24891,12 @@
         <v>12</v>
       </c>
       <c r="I904" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="905" spans="1:9">
       <c r="A905" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B905"/>
       <c r="C905">
@@ -24873,15 +24912,15 @@
         <v>12</v>
       </c>
       <c r="I905" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="906" spans="1:9">
       <c r="A906" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B906" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C906">
         <v>9.5E-4</v>
@@ -24896,15 +24935,15 @@
         <v>12</v>
       </c>
       <c r="I906" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="907" spans="1:9">
       <c r="A907" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B907" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C907">
         <v>1.7399999999999999E-5</v>
@@ -24919,15 +24958,15 @@
         <v>12</v>
       </c>
       <c r="I907" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="908" spans="1:9">
       <c r="A908" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B908" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C908">
         <v>5.7600000000000001E-4</v>
@@ -24942,15 +24981,15 @@
         <v>12</v>
       </c>
       <c r="I908" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="909" spans="1:9">
       <c r="A909" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B909" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="C909">
         <v>1.1600000000000001E-11</v>
@@ -24965,7 +25004,7 @@
         <v>12</v>
       </c>
       <c r="I909" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="910" spans="1:9">
@@ -24988,7 +25027,7 @@
         <v>12</v>
       </c>
       <c r="I910" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="911" spans="1:9">
@@ -25011,7 +25050,7 @@
         <v>12</v>
       </c>
       <c r="I911" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="912" spans="1:9">
@@ -25034,15 +25073,15 @@
         <v>12</v>
       </c>
       <c r="I912" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="913" spans="1:10">
       <c r="A913" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="B913" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C913">
         <v>0.1020326</v>
@@ -25057,12 +25096,12 @@
         <v>12</v>
       </c>
       <c r="I913" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="914" spans="1:10">
       <c r="A914" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B914" t="s">
         <v>33</v>
@@ -25074,7 +25113,7 @@
         <v>19</v>
       </c>
       <c r="G914" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="H914" t="s">
         <v>12</v>
@@ -25085,10 +25124,10 @@
     </row>
     <row r="915" spans="1:10">
       <c r="A915" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="B915" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C915">
         <v>1.1600000000000001E-11</v>
@@ -25097,21 +25136,21 @@
         <v>13</v>
       </c>
       <c r="G915" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="H915" t="s">
         <v>12</v>
       </c>
       <c r="I915" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="916" spans="1:10">
       <c r="A916" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B916" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C916">
         <v>-2.0200000000000001E-3</v>
@@ -25126,15 +25165,15 @@
         <v>12</v>
       </c>
       <c r="I916" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="917" spans="1:10">
       <c r="A917" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B917" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="C917">
         <v>-1.1600000000000001E-11</v>
@@ -25149,15 +25188,15 @@
         <v>12</v>
       </c>
       <c r="I917" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="918" spans="1:10">
       <c r="A918" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B918" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C918">
         <v>-1.1600000000000001E-11</v>
@@ -25172,15 +25211,15 @@
         <v>12</v>
       </c>
       <c r="I918" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="919" spans="1:10">
       <c r="A919" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B919" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="C919">
         <v>-5.63E-5</v>
@@ -25195,15 +25234,15 @@
         <v>12</v>
       </c>
       <c r="I919" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="920" spans="1:10">
       <c r="A920" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="B920" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C920">
         <v>-9.4499999999999998E-4</v>
@@ -25218,15 +25257,15 @@
         <v>12</v>
       </c>
       <c r="I920" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="921" spans="1:10">
       <c r="A921" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B921" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C921">
         <v>6.28E-6</v>
@@ -25241,15 +25280,15 @@
         <v>12</v>
       </c>
       <c r="I921" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="922" spans="1:10">
       <c r="A922" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B922" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C922" s="13">
         <v>0.15468000000000001</v>
@@ -25280,7 +25319,7 @@
         <v>1</v>
       </c>
       <c r="B924" s="43" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="925" spans="1:10">
@@ -25307,7 +25346,7 @@
         <v>4</v>
       </c>
       <c r="B927" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F927" s="13"/>
       <c r="J927" s="56"/>
@@ -25416,7 +25455,7 @@
         <v>15</v>
       </c>
       <c r="I934" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="935" spans="1:9">
@@ -25440,7 +25479,7 @@
         <v>15</v>
       </c>
       <c r="I935" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="936" spans="1:9">
@@ -25464,7 +25503,7 @@
         <v>15</v>
       </c>
       <c r="I936" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="937" spans="1:9">
@@ -25493,7 +25532,7 @@
     </row>
     <row r="938" spans="1:9">
       <c r="A938" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B938"/>
       <c r="C938">
@@ -25538,7 +25577,7 @@
     </row>
     <row r="940" spans="1:9">
       <c r="A940" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B940"/>
       <c r="C940">
@@ -25562,10 +25601,10 @@
     </row>
     <row r="941" spans="1:9">
       <c r="A941" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B941" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="C941">
         <v>1</v>
@@ -25585,7 +25624,7 @@
     </row>
     <row r="942" spans="1:9">
       <c r="A942" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B942"/>
       <c r="C942">
@@ -25601,12 +25640,12 @@
         <v>12</v>
       </c>
       <c r="I942" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="943" spans="1:9">
       <c r="A943" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B943"/>
       <c r="C943">
@@ -25622,15 +25661,15 @@
         <v>12</v>
       </c>
       <c r="I943" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="944" spans="1:9">
       <c r="A944" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B944" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C944">
         <v>9.5E-4</v>
@@ -25645,15 +25684,15 @@
         <v>12</v>
       </c>
       <c r="I944" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="945" spans="1:9">
       <c r="A945" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B945" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C945">
         <v>1.7399999999999999E-5</v>
@@ -25668,15 +25707,15 @@
         <v>12</v>
       </c>
       <c r="I945" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="946" spans="1:9">
       <c r="A946" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B946" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C946">
         <v>5.7600000000000001E-4</v>
@@ -25691,15 +25730,15 @@
         <v>12</v>
       </c>
       <c r="I946" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="947" spans="1:9">
       <c r="A947" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B947" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="C947">
         <v>1.1600000000000001E-11</v>
@@ -25714,7 +25753,7 @@
         <v>12</v>
       </c>
       <c r="I947" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="948" spans="1:9">
@@ -25737,7 +25776,7 @@
         <v>12</v>
       </c>
       <c r="I948" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="949" spans="1:9">
@@ -25760,7 +25799,7 @@
         <v>12</v>
       </c>
       <c r="I949" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="950" spans="1:9">
@@ -25783,15 +25822,15 @@
         <v>12</v>
       </c>
       <c r="I950" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="951" spans="1:9">
       <c r="A951" s="31" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B951" s="31" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C951">
         <v>0.1020326</v>
@@ -25806,12 +25845,12 @@
         <v>12</v>
       </c>
       <c r="I951" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="952" spans="1:9">
       <c r="A952" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B952" t="s">
         <v>33</v>
@@ -25823,7 +25862,7 @@
         <v>19</v>
       </c>
       <c r="G952" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="H952" t="s">
         <v>12</v>
@@ -25834,10 +25873,10 @@
     </row>
     <row r="953" spans="1:9">
       <c r="A953" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="B953" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C953">
         <v>1.1600000000000001E-11</v>
@@ -25846,21 +25885,21 @@
         <v>13</v>
       </c>
       <c r="G953" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="H953" t="s">
         <v>12</v>
       </c>
       <c r="I953" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="954" spans="1:9">
       <c r="A954" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B954" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C954">
         <v>-2.0200000000000001E-3</v>
@@ -25875,15 +25914,15 @@
         <v>12</v>
       </c>
       <c r="I954" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="955" spans="1:9">
       <c r="A955" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B955" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="C955">
         <v>-1.1600000000000001E-11</v>
@@ -25898,15 +25937,15 @@
         <v>12</v>
       </c>
       <c r="I955" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="956" spans="1:9">
       <c r="A956" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B956" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C956">
         <v>-1.1600000000000001E-11</v>
@@ -25921,15 +25960,15 @@
         <v>12</v>
       </c>
       <c r="I956" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="957" spans="1:9">
       <c r="A957" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B957" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="C957">
         <v>-5.63E-5</v>
@@ -25944,15 +25983,15 @@
         <v>12</v>
       </c>
       <c r="I957" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="958" spans="1:9">
       <c r="A958" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="B958" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C958">
         <v>-9.4499999999999998E-4</v>
@@ -25967,15 +26006,15 @@
         <v>12</v>
       </c>
       <c r="I958" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="959" spans="1:9">
       <c r="A959" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B959" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C959">
         <v>6.28E-6</v>
@@ -25990,7 +26029,7 @@
         <v>12</v>
       </c>
       <c r="I959" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="960" spans="1:9">
@@ -26009,7 +26048,7 @@
         <v>1</v>
       </c>
       <c r="B961" s="43" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="962" spans="1:10">
@@ -26036,7 +26075,7 @@
         <v>4</v>
       </c>
       <c r="B964" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="F964" s="13"/>
       <c r="J964" s="56"/>
@@ -26063,7 +26102,7 @@
         <v>57</v>
       </c>
       <c r="B967" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="968" spans="1:10" ht="15.75">
@@ -26110,10 +26149,10 @@
     </row>
     <row r="970" spans="1:10">
       <c r="A970" s="31" t="s">
+        <v>444</v>
+      </c>
+      <c r="B970" s="31" t="s">
         <v>445</v>
-      </c>
-      <c r="B970" s="31" t="s">
-        <v>446</v>
       </c>
       <c r="C970" s="26">
         <v>1</v>
@@ -26132,10 +26171,10 @@
     </row>
     <row r="971" spans="1:10">
       <c r="A971" s="26" t="s">
+        <v>451</v>
+      </c>
+      <c r="B971" s="13" t="s">
         <v>452</v>
-      </c>
-      <c r="B971" s="13" t="s">
-        <v>453</v>
       </c>
       <c r="C971" s="41">
         <v>1.7509999999999999</v>
@@ -26172,10 +26211,10 @@
     </row>
     <row r="973" spans="1:10">
       <c r="A973" s="31" t="s">
+        <v>453</v>
+      </c>
+      <c r="B973" s="31" t="s">
         <v>454</v>
-      </c>
-      <c r="B973" s="31" t="s">
-        <v>455</v>
       </c>
       <c r="C973">
         <v>0.17513974577662458</v>
@@ -26212,10 +26251,10 @@
     </row>
     <row r="975" spans="1:10">
       <c r="A975" s="58" t="s">
+        <v>447</v>
+      </c>
+      <c r="B975" s="13" t="s">
         <v>448</v>
-      </c>
-      <c r="B975" s="13" t="s">
-        <v>449</v>
       </c>
       <c r="C975">
         <v>2E-3</v>
@@ -26232,10 +26271,10 @@
     </row>
     <row r="976" spans="1:10">
       <c r="A976" t="s">
+        <v>449</v>
+      </c>
+      <c r="B976" s="13" t="s">
         <v>450</v>
-      </c>
-      <c r="B976" s="13" t="s">
-        <v>451</v>
       </c>
       <c r="C976">
         <v>-4.7795029869960301E-2</v>
@@ -26287,7 +26326,7 @@
         <v>1</v>
       </c>
       <c r="B979" s="43" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="980" spans="1:10">
@@ -26314,7 +26353,7 @@
         <v>4</v>
       </c>
       <c r="B982" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="F982" s="13"/>
       <c r="J982" s="56"/>
@@ -26341,7 +26380,7 @@
         <v>57</v>
       </c>
       <c r="B985" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="986" spans="1:10" ht="15.75">
@@ -26388,10 +26427,10 @@
     </row>
     <row r="988" spans="1:10">
       <c r="A988" s="31" t="s">
+        <v>455</v>
+      </c>
+      <c r="B988" s="31" t="s">
         <v>456</v>
-      </c>
-      <c r="B988" s="31" t="s">
-        <v>457</v>
       </c>
       <c r="C988" s="26">
         <v>1</v>
@@ -26410,10 +26449,10 @@
     </row>
     <row r="989" spans="1:10">
       <c r="A989" s="31" t="s">
+        <v>444</v>
+      </c>
+      <c r="B989" s="31" t="s">
         <v>445</v>
-      </c>
-      <c r="B989" s="31" t="s">
-        <v>446</v>
       </c>
       <c r="C989" s="41">
         <v>1.02</v>
@@ -26450,10 +26489,10 @@
     </row>
     <row r="991" spans="1:10">
       <c r="A991" s="31" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="B991" s="31" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="C991">
         <v>7.6485543677358989E-4</v>
@@ -26510,10 +26549,10 @@
     </row>
     <row r="994" spans="1:10">
       <c r="A994" t="s">
+        <v>460</v>
+      </c>
+      <c r="B994" s="13" t="s">
         <v>461</v>
-      </c>
-      <c r="B994" s="13" t="s">
-        <v>462</v>
       </c>
       <c r="C994">
         <v>-0.02</v>
@@ -26544,7 +26583,7 @@
         <v>1</v>
       </c>
       <c r="B996" s="43" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="997" spans="1:10">
@@ -26571,7 +26610,7 @@
         <v>4</v>
       </c>
       <c r="B999" s="43" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="F999" s="13"/>
       <c r="J999" s="56"/>
@@ -26598,7 +26637,7 @@
         <v>57</v>
       </c>
       <c r="B1002" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="1003" spans="1:10" ht="15.75">
@@ -26645,10 +26684,10 @@
     </row>
     <row r="1005" spans="1:10">
       <c r="A1005" s="31" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="B1005" s="31" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C1005" s="26">
         <v>1</v>
@@ -26687,10 +26726,10 @@
     </row>
     <row r="1007" spans="1:10">
       <c r="A1007" s="58" t="s">
+        <v>447</v>
+      </c>
+      <c r="B1007" s="13" t="s">
         <v>448</v>
-      </c>
-      <c r="B1007" s="13" t="s">
-        <v>449</v>
       </c>
       <c r="C1007">
         <v>5.8150000000000004</v>
@@ -26707,10 +26746,10 @@
     </row>
     <row r="1008" spans="1:10">
       <c r="A1008" t="s">
+        <v>467</v>
+      </c>
+      <c r="B1008" s="13" t="s">
         <v>468</v>
-      </c>
-      <c r="B1008" s="13" t="s">
-        <v>469</v>
       </c>
       <c r="C1008" s="13">
         <v>1.2333333333333333E-2</v>
@@ -26727,10 +26766,10 @@
     </row>
     <row r="1009" spans="1:10">
       <c r="A1009" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B1009" s="13" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="C1009" s="13">
         <v>0.98766666666666669</v>
@@ -26739,7 +26778,7 @@
         <v>13</v>
       </c>
       <c r="G1009" s="13" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="H1009" t="s">
         <v>12</v>
@@ -26747,10 +26786,10 @@
     </row>
     <row r="1010" spans="1:10">
       <c r="A1010" s="31" t="s">
+        <v>469</v>
+      </c>
+      <c r="B1010" s="13" t="s">
         <v>470</v>
-      </c>
-      <c r="B1010" s="13" t="s">
-        <v>471</v>
       </c>
       <c r="C1010" s="13">
         <v>0.04</v>
@@ -26759,7 +26798,7 @@
         <v>13</v>
       </c>
       <c r="G1010" s="13" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="H1010" t="s">
         <v>12</v>
@@ -26821,7 +26860,7 @@
         <v>1</v>
       </c>
       <c r="B1014" s="43" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="1015" spans="1:10">
@@ -26848,7 +26887,7 @@
         <v>4</v>
       </c>
       <c r="B1017" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="F1017" s="13"/>
       <c r="J1017" s="56"/>
@@ -26875,7 +26914,7 @@
         <v>57</v>
       </c>
       <c r="B1020" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="1021" spans="1:10" ht="15.75">
@@ -26922,10 +26961,10 @@
     </row>
     <row r="1023" spans="1:10">
       <c r="A1023" s="31" t="s">
+        <v>462</v>
+      </c>
+      <c r="B1023" s="31" t="s">
         <v>463</v>
-      </c>
-      <c r="B1023" s="31" t="s">
-        <v>464</v>
       </c>
       <c r="C1023" s="26">
         <v>1</v>
@@ -26944,10 +26983,10 @@
     </row>
     <row r="1024" spans="1:10">
       <c r="A1024" s="31" t="s">
+        <v>455</v>
+      </c>
+      <c r="B1024" s="31" t="s">
         <v>456</v>
-      </c>
-      <c r="B1024" s="31" t="s">
-        <v>457</v>
       </c>
       <c r="C1024" s="41">
         <v>1.35</v>
@@ -27004,10 +27043,10 @@
     </row>
     <row r="1027" spans="1:10">
       <c r="A1027" s="31" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="B1027" s="31" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C1027">
         <v>2.966014848457161E-5</v>
@@ -27044,10 +27083,10 @@
     </row>
     <row r="1029" spans="1:10">
       <c r="A1029" s="58" t="s">
+        <v>447</v>
+      </c>
+      <c r="B1029" s="13" t="s">
         <v>448</v>
-      </c>
-      <c r="B1029" s="13" t="s">
-        <v>449</v>
       </c>
       <c r="C1029">
         <v>4.17</v>
@@ -27127,7 +27166,7 @@
     </row>
     <row r="1033" spans="1:10">
       <c r="A1033" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="C1033" s="13">
         <v>4.0000000000000001E-3</v>
@@ -27162,7 +27201,7 @@
         <v>1</v>
       </c>
       <c r="B1035" s="43" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="1036" spans="1:10">
@@ -27189,7 +27228,7 @@
         <v>4</v>
       </c>
       <c r="B1038" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="F1038" s="13"/>
       <c r="J1038" s="56"/>
@@ -27216,7 +27255,7 @@
         <v>57</v>
       </c>
       <c r="B1041" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="1042" spans="1:9" ht="15.75">
@@ -27263,10 +27302,10 @@
     </row>
     <row r="1044" spans="1:9">
       <c r="A1044" s="31" t="s">
+        <v>472</v>
+      </c>
+      <c r="B1044" t="s">
         <v>473</v>
-      </c>
-      <c r="B1044" t="s">
-        <v>474</v>
       </c>
       <c r="C1044" s="26">
         <v>1</v>
@@ -27282,15 +27321,15 @@
         <v>18</v>
       </c>
       <c r="I1044" s="26" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="1045" spans="1:9">
       <c r="A1045" s="31" t="s">
+        <v>462</v>
+      </c>
+      <c r="B1045" s="31" t="s">
         <v>463</v>
-      </c>
-      <c r="B1045" s="31" t="s">
-        <v>464</v>
       </c>
       <c r="C1045" s="41">
         <v>1.9251563934282565</v>
@@ -27327,10 +27366,10 @@
     </row>
     <row r="1047" spans="1:9">
       <c r="A1047" s="31" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="B1047" s="31" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C1047">
         <v>4.2272109117479624E-5</v>
@@ -27367,10 +27406,10 @@
     </row>
     <row r="1049" spans="1:9">
       <c r="A1049" s="58" t="s">
+        <v>447</v>
+      </c>
+      <c r="B1049" s="13" t="s">
         <v>448</v>
-      </c>
-      <c r="B1049" s="13" t="s">
-        <v>449</v>
       </c>
       <c r="C1049">
         <v>8.0279021605958292</v>
@@ -27464,7 +27503,7 @@
         <v>1</v>
       </c>
       <c r="B1054" s="24" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
     </row>
     <row r="1055" spans="1:9">
@@ -27491,7 +27530,7 @@
         <v>4</v>
       </c>
       <c r="B1057" s="26" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="F1057" s="13"/>
       <c r="J1057" s="56"/>
@@ -27510,7 +27549,7 @@
         <v>6</v>
       </c>
       <c r="B1059" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="1060" spans="1:10">
@@ -27518,7 +27557,7 @@
         <v>57</v>
       </c>
       <c r="B1060" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
     </row>
     <row r="1061" spans="1:10" ht="15.75">
@@ -27565,16 +27604,16 @@
     </row>
     <row r="1063" spans="1:10">
       <c r="A1063" s="26" t="s">
+        <v>485</v>
+      </c>
+      <c r="B1063" s="26" t="s">
         <v>486</v>
-      </c>
-      <c r="B1063" s="26" t="s">
-        <v>487</v>
       </c>
       <c r="C1063">
         <v>1</v>
       </c>
       <c r="D1063" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="G1063" t="s">
         <v>28</v>
@@ -27585,10 +27624,10 @@
     </row>
     <row r="1064" spans="1:10">
       <c r="A1064" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B1064" s="13" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="C1064">
         <v>6.1215814640472162E-10</v>
@@ -27605,10 +27644,10 @@
     </row>
     <row r="1065" spans="1:10">
       <c r="A1065" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B1065" s="13" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="C1065">
         <v>4.742138768774307E-10</v>
@@ -27625,10 +27664,10 @@
     </row>
     <row r="1066" spans="1:10">
       <c r="A1066" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B1066" s="13" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="C1066">
         <v>2.6426999999999999E-2</v>
@@ -27665,7 +27704,7 @@
     </row>
     <row r="1068" spans="1:10">
       <c r="A1068" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="C1068">
         <v>1.0312926008611849E-4</v>
@@ -27685,7 +27724,7 @@
     </row>
     <row r="1069" spans="1:10">
       <c r="A1069" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C1069">
         <v>9.6919104678861535E-6</v>
@@ -27745,7 +27784,7 @@
     </row>
     <row r="1072" spans="1:10">
       <c r="A1072" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="C1072">
         <v>2.219861016536204E-5</v>
@@ -27779,7 +27818,7 @@
         <v>1</v>
       </c>
       <c r="B1074" s="24" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="1075" spans="1:10">
@@ -27806,7 +27845,7 @@
         <v>4</v>
       </c>
       <c r="B1077" s="26" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="F1077" s="13"/>
       <c r="J1077" s="56"/>
@@ -27878,10 +27917,10 @@
     </row>
     <row r="1083" spans="1:10">
       <c r="A1083" s="26" t="s">
+        <v>488</v>
+      </c>
+      <c r="B1083" s="26" t="s">
         <v>489</v>
-      </c>
-      <c r="B1083" s="26" t="s">
-        <v>490</v>
       </c>
       <c r="C1083">
         <v>1</v>
@@ -27932,7 +27971,7 @@
         <v>1</v>
       </c>
       <c r="B1086" s="24" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="1087" spans="1:10">
@@ -27959,7 +27998,7 @@
         <v>4</v>
       </c>
       <c r="B1089" s="26" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="F1089" s="13"/>
       <c r="J1089" s="56"/>
@@ -27986,7 +28025,7 @@
         <v>57</v>
       </c>
       <c r="B1092" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
     </row>
     <row r="1093" spans="1:10" ht="15.75">
@@ -28033,10 +28072,10 @@
     </row>
     <row r="1095" spans="1:10">
       <c r="A1095" s="26" t="s">
+        <v>495</v>
+      </c>
+      <c r="B1095" s="26" t="s">
         <v>496</v>
-      </c>
-      <c r="B1095" s="26" t="s">
-        <v>497</v>
       </c>
       <c r="C1095">
         <v>1</v>
@@ -28073,10 +28112,10 @@
     </row>
     <row r="1097" spans="1:10">
       <c r="A1097" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="B1097" s="13" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="C1097">
         <v>6.25E-2</v>
@@ -28093,10 +28132,10 @@
     </row>
     <row r="1098" spans="1:10">
       <c r="A1098" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="B1098" s="13" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="C1098" s="41">
         <v>0.33329999999999999</v>
@@ -28113,10 +28152,10 @@
     </row>
     <row r="1099" spans="1:10">
       <c r="A1099" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B1099" s="13" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="C1099" s="41">
         <v>0.33329999999999999</v>
@@ -28133,10 +28172,10 @@
     </row>
     <row r="1100" spans="1:10">
       <c r="A1100" t="s">
+        <v>492</v>
+      </c>
+      <c r="B1100" s="13" t="s">
         <v>493</v>
-      </c>
-      <c r="B1100" s="13" t="s">
-        <v>494</v>
       </c>
       <c r="C1100" s="41">
         <v>0.33329999999999999</v>
@@ -28166,8 +28205,8 @@
       <c r="A1102" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B1102" s="13" t="s">
-        <v>439</v>
+      <c r="B1102" s="23" t="s">
+        <v>438</v>
       </c>
     </row>
     <row r="1103" spans="1:10">
@@ -28194,7 +28233,7 @@
         <v>4</v>
       </c>
       <c r="B1105" s="13" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="F1105" s="13"/>
       <c r="J1105" s="56"/>
@@ -28264,10 +28303,10 @@
     </row>
     <row r="1111" spans="1:10">
       <c r="A1111" s="13" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B1111" s="13" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="C1111">
         <v>1</v>
@@ -28324,7 +28363,7 @@
     </row>
     <row r="1114" spans="1:10">
       <c r="A1114" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B1114" s="13" t="s">
         <v>170</v>
@@ -28356,7 +28395,7 @@
         <v>83</v>
       </c>
       <c r="F1115" t="s">
-        <v>25</v>
+        <v>174</v>
       </c>
       <c r="H1115" t="s">
         <v>15</v>
@@ -28376,9 +28415,449 @@
         <v>83</v>
       </c>
       <c r="F1116" t="s">
-        <v>25</v>
+        <v>174</v>
       </c>
       <c r="H1116" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1117" spans="1:10">
+      <c r="A1117" t="s">
+        <v>82</v>
+      </c>
+      <c r="C1117" s="13">
+        <v>9.79999999999996E-10</v>
+      </c>
+      <c r="D1117" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1117" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1117" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1117" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1118" spans="1:10">
+      <c r="A1118" t="s">
+        <v>522</v>
+      </c>
+      <c r="C1118" s="13">
+        <v>1.46999999999999E-7</v>
+      </c>
+      <c r="D1118" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1118" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1118" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1118" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1119" spans="1:10">
+      <c r="A1119" t="s">
+        <v>523</v>
+      </c>
+      <c r="C1119" s="13">
+        <v>3.91999999999998E-7</v>
+      </c>
+      <c r="D1119" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1119" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1119" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1119" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1120" spans="1:10">
+      <c r="A1120" t="s">
+        <v>524</v>
+      </c>
+      <c r="C1120" s="13">
+        <v>9.7999999999999607E-12</v>
+      </c>
+      <c r="D1120" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1120" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1120" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1120" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1121" spans="1:8">
+      <c r="A1121" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1121" s="13">
+        <v>6.8599999999999701E-7</v>
+      </c>
+      <c r="D1121" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1121" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1121" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1121" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1122" spans="1:8">
+      <c r="A1122" t="s">
+        <v>140</v>
+      </c>
+      <c r="C1122" s="13">
+        <v>5.7819999999999702E-6</v>
+      </c>
+      <c r="D1122" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1122" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1122" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1122" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1123" spans="1:8">
+      <c r="A1123" t="s">
+        <v>85</v>
+      </c>
+      <c r="C1123" s="13">
+        <v>4.8999999999999796E-7</v>
+      </c>
+      <c r="D1123" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1123" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1123" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1123" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1124" spans="1:8">
+      <c r="A1124" t="s">
+        <v>525</v>
+      </c>
+      <c r="C1124" s="13">
+        <v>2.9399999999999797E-17</v>
+      </c>
+      <c r="D1124" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1124" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1124" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1124" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1125" spans="1:8">
+      <c r="A1125" t="s">
+        <v>526</v>
+      </c>
+      <c r="C1125" s="13">
+        <v>9.7999999999999594E-8</v>
+      </c>
+      <c r="D1125" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1125" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1125" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1125" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1126" spans="1:8">
+      <c r="A1126" t="s">
+        <v>527</v>
+      </c>
+      <c r="C1126" s="13">
+        <v>2.9399999999999803E-11</v>
+      </c>
+      <c r="D1126" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1126" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1126" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1126" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1127" spans="1:8">
+      <c r="A1127" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1127" s="13">
+        <v>9.7019999999999606E-6</v>
+      </c>
+      <c r="D1127" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1127" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1127" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1127" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1128" spans="1:8">
+      <c r="A1128" t="s">
+        <v>528</v>
+      </c>
+      <c r="C1128" s="13">
+        <v>9.7999999999999604E-9</v>
+      </c>
+      <c r="D1128" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1128" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1128" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1128" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1129" spans="1:8">
+      <c r="A1129" t="s">
+        <v>529</v>
+      </c>
+      <c r="C1129" s="13">
+        <v>9.7999999999999594E-8</v>
+      </c>
+      <c r="D1129" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1129" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1129" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1129" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1130" spans="1:8">
+      <c r="A1130" t="s">
+        <v>530</v>
+      </c>
+      <c r="C1130" s="13">
+        <v>1.1759999999999901E-6</v>
+      </c>
+      <c r="D1130" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1130" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1130" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1130" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1131" spans="1:8">
+      <c r="A1131" t="s">
+        <v>88</v>
+      </c>
+      <c r="C1131" s="13">
+        <v>1.95999999999999E-7</v>
+      </c>
+      <c r="D1131" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1131" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1131" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1131" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1132" spans="1:8">
+      <c r="A1132" t="s">
+        <v>531</v>
+      </c>
+      <c r="C1132" s="13">
+        <v>1.9599999999999901E-8</v>
+      </c>
+      <c r="D1132" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1132" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1132" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1132" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1133" spans="1:8">
+      <c r="A1133" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1133" s="13">
+        <v>4.8999999999999796E-7</v>
+      </c>
+      <c r="D1133" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1133" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1133" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1133" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1134" spans="1:8">
+      <c r="A1134" t="s">
+        <v>532</v>
+      </c>
+      <c r="C1134" s="13">
+        <v>1.95999999999999E-7</v>
+      </c>
+      <c r="D1134" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1134" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1134" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1134" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1135" spans="1:8">
+      <c r="A1135" t="s">
+        <v>166</v>
+      </c>
+      <c r="C1135" s="13">
+        <v>1.2739999999999901E-7</v>
+      </c>
+      <c r="D1135" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1135" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1135" t="s">
+        <v>208</v>
+      </c>
+      <c r="H1135" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1136" spans="1:8">
+      <c r="A1136" t="s">
+        <v>533</v>
+      </c>
+      <c r="C1136" s="13">
+        <v>2.9399999999999799E-9</v>
+      </c>
+      <c r="D1136" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1136" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1136" t="s">
+        <v>208</v>
+      </c>
+      <c r="H1136" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1137" spans="1:8">
+      <c r="A1137" t="s">
+        <v>534</v>
+      </c>
+      <c r="C1137" s="13">
+        <v>4.8999999999999797E-8</v>
+      </c>
+      <c r="D1137" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1137" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1137" t="s">
+        <v>208</v>
+      </c>
+      <c r="H1137" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1138" spans="1:8">
+      <c r="A1138" t="s">
+        <v>535</v>
+      </c>
+      <c r="C1138" s="13">
+        <v>4.8999999999999797E-8</v>
+      </c>
+      <c r="D1138" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1138" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1138" t="s">
+        <v>208</v>
+      </c>
+      <c r="H1138" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added heat production in boiler for NG. Corrected error in biogas upgrading using PSA
</commit_message>
<xml_diff>
--- a/inventories/lci-Tr2050.xlsx
+++ b/inventories/lci-Tr2050.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engie-my.sharepoint.com/personal/db6421_engie_com/Documents/Documents/Local_repo/ADEME_scenarios_premise_gas/inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="244" documentId="13_ncr:1_{D0F9393E-493D-4D41-96B2-57E4008F0D51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2EDCD6C-09BE-4CDF-BF6D-716DA194E047}"/>
+  <xr:revisionPtr revIDLastSave="269" documentId="13_ncr:1_{D0F9393E-493D-4D41-96B2-57E4008F0D51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7794C347-6631-4EE7-A82C-DE756D6D539B}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="lci" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4742" uniqueCount="536">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4904" uniqueCount="539">
   <si>
     <t>Database</t>
   </si>
@@ -1644,6 +1644,15 @@
   </si>
   <si>
     <t>Sulfite</t>
+  </si>
+  <si>
+    <t>heat production, natural gas, at boiler condensing modulating &lt;100kW</t>
+  </si>
+  <si>
+    <t>heat, natural gas</t>
+  </si>
+  <si>
+    <t>market for natural gas, high pressure</t>
   </si>
 </sst>
 </file>
@@ -2180,18 +2189,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AH1138"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <dimension ref="A1:AH1176"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="73.140625" customWidth="1"/>
-    <col min="2" max="2" width="18.5703125" style="13" customWidth="1"/>
-    <col min="3" max="3" width="17.140625" customWidth="1"/>
-    <col min="4" max="4" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.42578125" customWidth="1"/>
-    <col min="6" max="6" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="109.7109375" customWidth="1"/>
+    <col min="1" max="1" width="73.109375" customWidth="1"/>
+    <col min="2" max="2" width="18.5546875" style="13" customWidth="1"/>
+    <col min="3" max="3" width="17.109375" customWidth="1"/>
+    <col min="4" max="4" width="24.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.44140625" customWidth="1"/>
+    <col min="6" max="6" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="109.6640625" customWidth="1"/>
     <col min="10" max="10" width="31" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2243,7 +2252,7 @@
       <c r="I4" s="6"/>
       <c r="K4" s="5"/>
     </row>
-    <row r="5" spans="1:14" ht="15.75">
+    <row r="5" spans="1:14" ht="15.6">
       <c r="A5" s="18" t="s">
         <v>1</v>
       </c>
@@ -2325,7 +2334,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="15.75">
+    <row r="13" spans="1:14" ht="15.6">
       <c r="A13" s="18" t="s">
         <v>7</v>
       </c>
@@ -2334,7 +2343,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="15.75">
+    <row r="14" spans="1:14" ht="15.6">
       <c r="A14" s="18" t="s">
         <v>8</v>
       </c>
@@ -3047,7 +3056,7 @@
       <c r="AG47" s="47"/>
       <c r="AH47" s="47"/>
     </row>
-    <row r="48" spans="1:34" s="15" customFormat="1" ht="15.75">
+    <row r="48" spans="1:34" s="15" customFormat="1" ht="15.6">
       <c r="A48" s="2" t="s">
         <v>1</v>
       </c>
@@ -3067,7 +3076,7 @@
       <c r="O48" s="16"/>
       <c r="P48" s="16"/>
     </row>
-    <row r="49" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="49" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A49" s="2" t="s">
         <v>3</v>
       </c>
@@ -3087,7 +3096,7 @@
       <c r="O49" s="16"/>
       <c r="P49" s="16"/>
     </row>
-    <row r="50" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="50" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A50" s="2" t="s">
         <v>11</v>
       </c>
@@ -3107,7 +3116,7 @@
       <c r="O50" s="16"/>
       <c r="P50" s="16"/>
     </row>
-    <row r="51" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="51" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A51" s="2" t="s">
         <v>4</v>
       </c>
@@ -3127,7 +3136,7 @@
       <c r="O51" s="16"/>
       <c r="P51" s="16"/>
     </row>
-    <row r="52" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="52" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A52" s="2" t="s">
         <v>2</v>
       </c>
@@ -3147,7 +3156,7 @@
       <c r="O52" s="16"/>
       <c r="P52" s="16"/>
     </row>
-    <row r="53" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="53" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A53" s="2" t="s">
         <v>6</v>
       </c>
@@ -3169,7 +3178,7 @@
       <c r="O53" s="16"/>
       <c r="P53" s="16"/>
     </row>
-    <row r="54" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="54" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A54" s="2" t="s">
         <v>7</v>
       </c>
@@ -3189,7 +3198,7 @@
       <c r="O54" s="16"/>
       <c r="P54" s="16"/>
     </row>
-    <row r="55" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="55" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A55" s="2" t="s">
         <v>8</v>
       </c>
@@ -3227,7 +3236,7 @@
       <c r="S55" s="17"/>
       <c r="T55" s="18"/>
     </row>
-    <row r="56" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="56" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A56" t="s">
         <v>54</v>
       </c>
@@ -3259,7 +3268,7 @@
       <c r="P56" s="16"/>
       <c r="T56"/>
     </row>
-    <row r="57" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="57" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A57" t="s">
         <v>52</v>
       </c>
@@ -3293,7 +3302,7 @@
       <c r="Q57"/>
       <c r="R57"/>
     </row>
-    <row r="58" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="58" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A58" t="s">
         <v>53</v>
       </c>
@@ -3327,7 +3336,7 @@
       <c r="Q58"/>
       <c r="R58"/>
     </row>
-    <row r="59" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="59" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A59" t="s">
         <v>43</v>
       </c>
@@ -3361,7 +3370,7 @@
       <c r="Q59"/>
       <c r="R59"/>
     </row>
-    <row r="60" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="60" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A60" t="s">
         <v>46</v>
       </c>
@@ -3395,7 +3404,7 @@
       <c r="Q60"/>
       <c r="R60"/>
     </row>
-    <row r="61" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="61" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A61" t="s">
         <v>27</v>
       </c>
@@ -3428,7 +3437,7 @@
       <c r="Q61"/>
       <c r="R61"/>
     </row>
-    <row r="62" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="62" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A62" t="s">
         <v>21</v>
       </c>
@@ -3461,7 +3470,7 @@
       <c r="Q62"/>
       <c r="R62"/>
     </row>
-    <row r="63" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="63" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A63" t="s">
         <v>24</v>
       </c>
@@ -3490,7 +3499,7 @@
       <c r="Q63" s="20"/>
       <c r="R63"/>
     </row>
-    <row r="64" spans="1:20" s="15" customFormat="1" ht="15.75">
+    <row r="64" spans="1:20" s="15" customFormat="1" ht="15.6">
       <c r="A64" t="s">
         <v>51</v>
       </c>
@@ -3559,7 +3568,7 @@
       <c r="AG65" s="47"/>
       <c r="AH65" s="47"/>
     </row>
-    <row r="66" spans="1:34" ht="15.75">
+    <row r="66" spans="1:34" ht="15.6">
       <c r="A66" s="18" t="s">
         <v>1</v>
       </c>
@@ -3621,13 +3630,13 @@
         <v>13</v>
       </c>
     </row>
-    <row r="74" spans="1:34" ht="15.75">
+    <row r="74" spans="1:34" ht="15.6">
       <c r="A74" s="18" t="s">
         <v>7</v>
       </c>
       <c r="B74"/>
     </row>
-    <row r="75" spans="1:34" ht="15.75">
+    <row r="75" spans="1:34" ht="15.6">
       <c r="A75" s="18" t="s">
         <v>8</v>
       </c>
@@ -17017,7 +17026,7 @@
       </c>
       <c r="B457"/>
     </row>
-    <row r="458" spans="1:9" ht="15.75">
+    <row r="458" spans="1:9" ht="15.6">
       <c r="A458" s="18" t="s">
         <v>7</v>
       </c>
@@ -17414,7 +17423,7 @@
       </c>
       <c r="B481"/>
     </row>
-    <row r="482" spans="1:9" ht="15.75">
+    <row r="482" spans="1:9" ht="15.6">
       <c r="A482" s="18" t="s">
         <v>7</v>
       </c>
@@ -17991,7 +18000,7 @@
       </c>
       <c r="B513"/>
     </row>
-    <row r="514" spans="1:9" ht="15.75">
+    <row r="514" spans="1:9" ht="15.6">
       <c r="A514" s="18" t="s">
         <v>7</v>
       </c>
@@ -18568,7 +18577,7 @@
       </c>
       <c r="B545"/>
     </row>
-    <row r="546" spans="1:9" ht="15.75">
+    <row r="546" spans="1:9" ht="15.6">
       <c r="A546" s="18" t="s">
         <v>7</v>
       </c>
@@ -18939,7 +18948,7 @@
         <v>185</v>
       </c>
       <c r="C563">
-        <v>2.0799999999999999E-4</v>
+        <v>0</v>
       </c>
       <c r="D563" s="31" t="s">
         <v>13</v>
@@ -18962,7 +18971,7 @@
         <v>187</v>
       </c>
       <c r="C564">
-        <v>0</v>
+        <v>2.0799999999999999E-4</v>
       </c>
       <c r="D564" s="31" t="s">
         <v>13</v>
@@ -18985,7 +18994,7 @@
         <v>189</v>
       </c>
       <c r="C565">
-        <v>3.98E-6</v>
+        <v>0</v>
       </c>
       <c r="D565" s="31" t="s">
         <v>13</v>
@@ -19008,7 +19017,7 @@
         <v>191</v>
       </c>
       <c r="C566">
-        <v>0</v>
+        <v>3.98E-6</v>
       </c>
       <c r="D566" s="31" t="s">
         <v>13</v>
@@ -19145,7 +19154,7 @@
       </c>
       <c r="B577"/>
     </row>
-    <row r="578" spans="1:9" ht="15.75">
+    <row r="578" spans="1:9" ht="15.6">
       <c r="A578" s="18" t="s">
         <v>7</v>
       </c>
@@ -19722,7 +19731,7 @@
       </c>
       <c r="B609"/>
     </row>
-    <row r="610" spans="1:9" ht="15.75">
+    <row r="610" spans="1:9" ht="15.6">
       <c r="A610" s="18" t="s">
         <v>7</v>
       </c>
@@ -20119,7 +20128,7 @@
       </c>
       <c r="B633"/>
     </row>
-    <row r="634" spans="1:9" ht="15.75">
+    <row r="634" spans="1:9" ht="15.6">
       <c r="A634" s="18" t="s">
         <v>7</v>
       </c>
@@ -20696,7 +20705,7 @@
       </c>
       <c r="B665"/>
     </row>
-    <row r="666" spans="1:9" ht="15.75">
+    <row r="666" spans="1:9" ht="15.6">
       <c r="A666" s="18" t="s">
         <v>7</v>
       </c>
@@ -21273,7 +21282,7 @@
       </c>
       <c r="B697"/>
     </row>
-    <row r="698" spans="1:9" ht="15.75">
+    <row r="698" spans="1:9" ht="15.6">
       <c r="A698" s="18" t="s">
         <v>7</v>
       </c>
@@ -21644,7 +21653,7 @@
         <v>185</v>
       </c>
       <c r="C715">
-        <v>2.0799999999999999E-4</v>
+        <v>0</v>
       </c>
       <c r="D715" s="31" t="s">
         <v>13</v>
@@ -21667,7 +21676,7 @@
         <v>187</v>
       </c>
       <c r="C716">
-        <v>0</v>
+        <v>2.0799999999999999E-4</v>
       </c>
       <c r="D716" s="31" t="s">
         <v>13</v>
@@ -21690,7 +21699,7 @@
         <v>189</v>
       </c>
       <c r="C717">
-        <v>3.98E-6</v>
+        <v>0</v>
       </c>
       <c r="D717" s="31" t="s">
         <v>13</v>
@@ -21713,7 +21722,7 @@
         <v>191</v>
       </c>
       <c r="C718">
-        <v>0</v>
+        <v>3.98E-6</v>
       </c>
       <c r="D718" s="31" t="s">
         <v>13</v>
@@ -21851,7 +21860,7 @@
       </c>
       <c r="B729"/>
     </row>
-    <row r="730" spans="1:9" ht="15.75">
+    <row r="730" spans="1:9" ht="15.6">
       <c r="A730" s="18" t="s">
         <v>7</v>
       </c>
@@ -22430,7 +22439,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="762" spans="1:20" ht="15.75">
+    <row r="762" spans="1:20" ht="15.6">
       <c r="A762" s="18" t="s">
         <v>7</v>
       </c>
@@ -24588,7 +24597,7 @@
       <c r="H886" s="49"/>
       <c r="I886" s="49"/>
     </row>
-    <row r="887" spans="1:10" ht="15.75">
+    <row r="887" spans="1:10" ht="15.6">
       <c r="A887" s="18" t="s">
         <v>1</v>
       </c>
@@ -24650,7 +24659,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="894" spans="1:10" ht="15.75">
+    <row r="894" spans="1:10" ht="15.6">
       <c r="A894" s="18" t="s">
         <v>7</v>
       </c>
@@ -25314,7 +25323,7 @@
       <c r="H923" s="49"/>
       <c r="I923" s="49"/>
     </row>
-    <row r="924" spans="1:10" ht="15.75">
+    <row r="924" spans="1:10" ht="15.6">
       <c r="A924" s="18" t="s">
         <v>1</v>
       </c>
@@ -25376,7 +25385,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="931" spans="1:9" ht="15.75">
+    <row r="931" spans="1:9" ht="15.6">
       <c r="A931" s="18" t="s">
         <v>7</v>
       </c>
@@ -26043,7 +26052,7 @@
       <c r="H960" s="49"/>
       <c r="I960" s="49"/>
     </row>
-    <row r="961" spans="1:10" ht="15.75">
+    <row r="961" spans="1:10" ht="15.6">
       <c r="A961" s="18" t="s">
         <v>1</v>
       </c>
@@ -26105,7 +26114,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="968" spans="1:10" ht="15.75">
+    <row r="968" spans="1:10" ht="15.6">
       <c r="A968" s="18" t="s">
         <v>7</v>
       </c>
@@ -26321,7 +26330,7 @@
       <c r="H978" s="49"/>
       <c r="I978" s="49"/>
     </row>
-    <row r="979" spans="1:10" ht="15.75">
+    <row r="979" spans="1:10" ht="15.6">
       <c r="A979" s="18" t="s">
         <v>1</v>
       </c>
@@ -26383,7 +26392,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="986" spans="1:10" ht="15.75">
+    <row r="986" spans="1:10" ht="15.6">
       <c r="A986" s="18" t="s">
         <v>7</v>
       </c>
@@ -26578,7 +26587,7 @@
       <c r="H995" s="49"/>
       <c r="I995" s="49"/>
     </row>
-    <row r="996" spans="1:10" ht="15.75">
+    <row r="996" spans="1:10" ht="15.6">
       <c r="A996" s="18" t="s">
         <v>1</v>
       </c>
@@ -26640,7 +26649,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="1003" spans="1:10" ht="15.75">
+    <row r="1003" spans="1:10" ht="15.6">
       <c r="A1003" s="18" t="s">
         <v>7</v>
       </c>
@@ -26855,7 +26864,7 @@
       <c r="H1013" s="49"/>
       <c r="I1013" s="49"/>
     </row>
-    <row r="1014" spans="1:10" ht="15.75">
+    <row r="1014" spans="1:10" ht="15.6">
       <c r="A1014" s="18" t="s">
         <v>1</v>
       </c>
@@ -26917,7 +26926,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="1021" spans="1:10" ht="15.75">
+    <row r="1021" spans="1:10" ht="15.6">
       <c r="A1021" s="18" t="s">
         <v>7</v>
       </c>
@@ -27196,7 +27205,7 @@
       <c r="H1034" s="49"/>
       <c r="I1034" s="49"/>
     </row>
-    <row r="1035" spans="1:10" ht="15.75">
+    <row r="1035" spans="1:10" ht="15.6">
       <c r="A1035" s="18" t="s">
         <v>1</v>
       </c>
@@ -27258,7 +27267,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="1042" spans="1:9" ht="15.75">
+    <row r="1042" spans="1:9" ht="15.6">
       <c r="A1042" s="18" t="s">
         <v>7</v>
       </c>
@@ -27498,7 +27507,7 @@
       <c r="H1053" s="49"/>
       <c r="I1053" s="49"/>
     </row>
-    <row r="1054" spans="1:9" ht="15.75">
+    <row r="1054" spans="1:9" ht="15.6">
       <c r="A1054" s="18" t="s">
         <v>1</v>
       </c>
@@ -27560,7 +27569,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="1061" spans="1:10" ht="15.75">
+    <row r="1061" spans="1:10" ht="15.6">
       <c r="A1061" s="18" t="s">
         <v>7</v>
       </c>
@@ -27813,7 +27822,7 @@
       <c r="H1073" s="49"/>
       <c r="I1073" s="49"/>
     </row>
-    <row r="1074" spans="1:10" ht="15.75">
+    <row r="1074" spans="1:10" ht="15.6">
       <c r="A1074" s="18" t="s">
         <v>1</v>
       </c>
@@ -27873,7 +27882,7 @@
       </c>
       <c r="B1080"/>
     </row>
-    <row r="1081" spans="1:10" ht="15.75">
+    <row r="1081" spans="1:10" ht="15.6">
       <c r="A1081" s="18" t="s">
         <v>7</v>
       </c>
@@ -27966,7 +27975,7 @@
       <c r="H1085" s="49"/>
       <c r="I1085" s="49"/>
     </row>
-    <row r="1086" spans="1:10" ht="15.75">
+    <row r="1086" spans="1:10" ht="15.6">
       <c r="A1086" s="18" t="s">
         <v>1</v>
       </c>
@@ -28028,7 +28037,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="1093" spans="1:10" ht="15.75">
+    <row r="1093" spans="1:10" ht="15.6">
       <c r="A1093" s="18" t="s">
         <v>7</v>
       </c>
@@ -28201,7 +28210,7 @@
       <c r="H1101" s="49"/>
       <c r="I1101" s="49"/>
     </row>
-    <row r="1102" spans="1:10" ht="15.75">
+    <row r="1102" spans="1:10" ht="15.6">
       <c r="A1102" s="18" t="s">
         <v>1</v>
       </c>
@@ -28260,7 +28269,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="1109" spans="1:10" ht="15.75">
+    <row r="1109" spans="1:10" ht="15.6">
       <c r="A1109" s="18" t="s">
         <v>7</v>
       </c>
@@ -28821,7 +28830,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="1137" spans="1:8">
+    <row r="1137" spans="1:10">
       <c r="A1137" t="s">
         <v>534</v>
       </c>
@@ -28841,7 +28850,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="1138" spans="1:8">
+    <row r="1138" spans="1:10">
       <c r="A1138" t="s">
         <v>535</v>
       </c>
@@ -28858,6 +28867,677 @@
         <v>208</v>
       </c>
       <c r="H1138" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1139" spans="1:10">
+      <c r="A1139" s="49"/>
+      <c r="B1139" s="50"/>
+      <c r="C1139" s="49"/>
+      <c r="D1139" s="49"/>
+      <c r="E1139" s="49"/>
+      <c r="F1139" s="49"/>
+      <c r="G1139" s="49"/>
+      <c r="H1139" s="49"/>
+      <c r="I1139" s="49"/>
+    </row>
+    <row r="1140" spans="1:10" ht="15.6">
+      <c r="A1140" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1140" s="23" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="1141" spans="1:10">
+      <c r="A1141" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1141" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1141" s="55"/>
+    </row>
+    <row r="1142" spans="1:10">
+      <c r="A1142" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1142" s="13">
+        <v>1</v>
+      </c>
+      <c r="F1142" s="13"/>
+      <c r="H1142" s="13"/>
+    </row>
+    <row r="1143" spans="1:10">
+      <c r="A1143" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1143" s="13" t="s">
+        <v>537</v>
+      </c>
+      <c r="F1143" s="13"/>
+      <c r="J1143" s="56"/>
+    </row>
+    <row r="1144" spans="1:10">
+      <c r="A1144" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1144" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1144" s="20"/>
+    </row>
+    <row r="1145" spans="1:10">
+      <c r="A1145" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1145" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="1146" spans="1:10">
+      <c r="A1146" s="24" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="1147" spans="1:10" ht="15.6">
+      <c r="A1147" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1147" s="25"/>
+      <c r="D1147" s="26"/>
+      <c r="E1147" s="26"/>
+      <c r="F1147" s="26"/>
+      <c r="G1147" s="26"/>
+      <c r="H1147" s="26"/>
+      <c r="I1147" s="26"/>
+    </row>
+    <row r="1148" spans="1:10">
+      <c r="A1148" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1148" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1148" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1148" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1148" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="F1148" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1148" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1148" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1148" s="24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1149" spans="1:10">
+      <c r="A1149" s="13" t="s">
+        <v>536</v>
+      </c>
+      <c r="B1149" s="13" t="s">
+        <v>537</v>
+      </c>
+      <c r="C1149">
+        <v>1</v>
+      </c>
+      <c r="D1149" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1149" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1149" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="1150" spans="1:10">
+      <c r="A1150" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1150" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="C1150" s="13">
+        <v>6.4679999999999999E-7</v>
+      </c>
+      <c r="D1150" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1150" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1150" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1151" spans="1:10">
+      <c r="A1151" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1151" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1151">
+        <v>2.7243999999999801E-3</v>
+      </c>
+      <c r="D1151" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1151" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1151" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1152" spans="1:10">
+      <c r="A1152" t="s">
+        <v>538</v>
+      </c>
+      <c r="B1152" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1152">
+        <v>2.8796896151254369E-2</v>
+      </c>
+      <c r="D1152" t="s">
+        <v>91</v>
+      </c>
+      <c r="G1152" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1152" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1153" spans="1:8">
+      <c r="A1153" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1153">
+        <v>5.6796586669920886E-2</v>
+      </c>
+      <c r="D1153" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1153" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1153" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1153" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1154" spans="1:8">
+      <c r="A1154" t="s">
+        <v>86</v>
+      </c>
+      <c r="C1154">
+        <v>2.0027932960891646E-6</v>
+      </c>
+      <c r="D1154" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1154" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1154" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1154" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1155" spans="1:8">
+      <c r="A1155" t="s">
+        <v>82</v>
+      </c>
+      <c r="C1155" s="13">
+        <v>9.79999999999996E-10</v>
+      </c>
+      <c r="D1155" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1155" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1155" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1155" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1156" spans="1:8">
+      <c r="A1156" t="s">
+        <v>522</v>
+      </c>
+      <c r="C1156" s="13">
+        <v>1.46999999999999E-7</v>
+      </c>
+      <c r="D1156" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1156" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1156" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1156" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1157" spans="1:8">
+      <c r="A1157" t="s">
+        <v>523</v>
+      </c>
+      <c r="C1157" s="13">
+        <v>3.91999999999998E-7</v>
+      </c>
+      <c r="D1157" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1157" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1157" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1157" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1158" spans="1:8">
+      <c r="A1158" t="s">
+        <v>524</v>
+      </c>
+      <c r="C1158" s="13">
+        <v>9.7999999999999607E-12</v>
+      </c>
+      <c r="D1158" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1158" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1158" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1158" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1159" spans="1:8">
+      <c r="A1159" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1159" s="13">
+        <v>6.8599999999999701E-7</v>
+      </c>
+      <c r="D1159" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1159" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1159" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1159" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1160" spans="1:8">
+      <c r="A1160" t="s">
+        <v>140</v>
+      </c>
+      <c r="C1160" s="13">
+        <v>5.7819999999999702E-6</v>
+      </c>
+      <c r="D1160" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1160" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1160" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1160" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1161" spans="1:8">
+      <c r="A1161" t="s">
+        <v>85</v>
+      </c>
+      <c r="C1161" s="13">
+        <v>4.8999999999999796E-7</v>
+      </c>
+      <c r="D1161" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1161" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1161" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1161" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1162" spans="1:8">
+      <c r="A1162" t="s">
+        <v>525</v>
+      </c>
+      <c r="C1162" s="13">
+        <v>2.9399999999999797E-17</v>
+      </c>
+      <c r="D1162" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1162" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1162" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1162" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1163" spans="1:8">
+      <c r="A1163" t="s">
+        <v>526</v>
+      </c>
+      <c r="C1163" s="13">
+        <v>9.7999999999999594E-8</v>
+      </c>
+      <c r="D1163" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1163" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1163" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1163" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1164" spans="1:8">
+      <c r="A1164" t="s">
+        <v>527</v>
+      </c>
+      <c r="C1164" s="13">
+        <v>2.9399999999999803E-11</v>
+      </c>
+      <c r="D1164" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1164" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1164" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1164" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1165" spans="1:8">
+      <c r="A1165" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1165" s="13">
+        <v>9.7019999999999606E-6</v>
+      </c>
+      <c r="D1165" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1165" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1165" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1165" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1166" spans="1:8">
+      <c r="A1166" t="s">
+        <v>528</v>
+      </c>
+      <c r="C1166" s="13">
+        <v>9.7999999999999604E-9</v>
+      </c>
+      <c r="D1166" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1166" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1166" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1166" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1167" spans="1:8">
+      <c r="A1167" t="s">
+        <v>529</v>
+      </c>
+      <c r="C1167" s="13">
+        <v>9.7999999999999594E-8</v>
+      </c>
+      <c r="D1167" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1167" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1167" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1167" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1168" spans="1:8">
+      <c r="A1168" t="s">
+        <v>530</v>
+      </c>
+      <c r="C1168" s="13">
+        <v>1.1759999999999901E-6</v>
+      </c>
+      <c r="D1168" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1168" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1168" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1168" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1169" spans="1:8">
+      <c r="A1169" t="s">
+        <v>88</v>
+      </c>
+      <c r="C1169" s="13">
+        <v>1.95999999999999E-7</v>
+      </c>
+      <c r="D1169" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1169" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1169" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1169" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1170" spans="1:8">
+      <c r="A1170" t="s">
+        <v>531</v>
+      </c>
+      <c r="C1170" s="13">
+        <v>1.9599999999999901E-8</v>
+      </c>
+      <c r="D1170" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1170" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1170" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1170" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1171" spans="1:8">
+      <c r="A1171" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1171" s="13">
+        <v>4.8999999999999796E-7</v>
+      </c>
+      <c r="D1171" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1171" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1171" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1171" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1172" spans="1:8">
+      <c r="A1172" t="s">
+        <v>532</v>
+      </c>
+      <c r="C1172" s="13">
+        <v>1.95999999999999E-7</v>
+      </c>
+      <c r="D1172" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1172" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1172" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1172" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1173" spans="1:8">
+      <c r="A1173" t="s">
+        <v>166</v>
+      </c>
+      <c r="C1173" s="13">
+        <v>1.2739999999999901E-7</v>
+      </c>
+      <c r="D1173" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1173" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1173" t="s">
+        <v>208</v>
+      </c>
+      <c r="H1173" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1174" spans="1:8">
+      <c r="A1174" t="s">
+        <v>533</v>
+      </c>
+      <c r="C1174" s="13">
+        <v>2.9399999999999799E-9</v>
+      </c>
+      <c r="D1174" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1174" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1174" t="s">
+        <v>208</v>
+      </c>
+      <c r="H1174" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1175" spans="1:8">
+      <c r="A1175" t="s">
+        <v>534</v>
+      </c>
+      <c r="C1175" s="13">
+        <v>4.8999999999999797E-8</v>
+      </c>
+      <c r="D1175" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1175" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1175" t="s">
+        <v>208</v>
+      </c>
+      <c r="H1175" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="1176" spans="1:8">
+      <c r="A1176" t="s">
+        <v>535</v>
+      </c>
+      <c r="C1176" s="13">
+        <v>4.8999999999999797E-8</v>
+      </c>
+      <c r="D1176" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1176" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1176" t="s">
+        <v>208</v>
+      </c>
+      <c r="H1176" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
- Changed pkm in market for mobility to person kilometer for consistency. - Updated market for mobility to avoid the unlinked activity message when generating the database.
</commit_message>
<xml_diff>
--- a/inventories/lci-Tr2050.xlsx
+++ b/inventories/lci-Tr2050.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engie-my.sharepoint.com/personal/db6421_engie_com/Documents/Documents/Local_repo/ADEME_scenarios_premise_gas/inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1044" documentId="13_ncr:1_{D0F9393E-493D-4D41-96B2-57E4008F0D51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B354B266-886E-4B26-9EA0-C26E74A3C1B9}"/>
+  <xr:revisionPtr revIDLastSave="1052" documentId="13_ncr:1_{D0F9393E-493D-4D41-96B2-57E4008F0D51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA45AAD1-F78C-4B10-A8EA-D86CA8AAC0B5}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6030" uniqueCount="760">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6031" uniqueCount="759">
   <si>
     <t>Database</t>
   </si>
@@ -2306,16 +2306,13 @@
     <t>mobility</t>
   </si>
   <si>
-    <t>transport, passenger</t>
-  </si>
-  <si>
-    <t>pkm</t>
-  </si>
-  <si>
-    <t>market for passenger mobility, Tr2050</t>
-  </si>
-  <si>
     <t>Scaled to 1 pkm from "GENESIS_2030_conventional_Base" (Thonemann et al., 2024) considering kerosene consumption and infrastructure in ecoinvent 391</t>
+  </si>
+  <si>
+    <t>Replaced by transport market from ADEME scenarios once the database generated</t>
+  </si>
+  <si>
+    <t>transport, passenger train</t>
   </si>
 </sst>
 </file>
@@ -28236,7 +28233,7 @@
         <v>57</v>
       </c>
       <c r="B1060" t="s">
-        <v>759</v>
+        <v>756</v>
       </c>
     </row>
     <row r="1061" spans="1:10" ht="15.6">
@@ -34975,19 +34972,22 @@
         <v>758</v>
       </c>
       <c r="B1464" s="13" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="C1464" s="65">
         <v>5025.4162915136185</v>
       </c>
       <c r="D1464" t="s">
-        <v>757</v>
+        <v>486</v>
       </c>
       <c r="G1464" t="s">
         <v>28</v>
       </c>
       <c r="H1464" t="s">
         <v>12</v>
+      </c>
+      <c r="I1464" t="s">
+        <v>757</v>
       </c>
     </row>
     <row r="1465" spans="1:9">

</xml_diff>

<commit_message>
- Removed unlinked activities warning (heat shelter, heat non-residential, and EoL) by replacing activities by generated markets
</commit_message>
<xml_diff>
--- a/inventories/lci-Tr2050.xlsx
+++ b/inventories/lci-Tr2050.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engie-my.sharepoint.com/personal/db6421_engie_com/Documents/Documents/Local_repo/ADEME_scenarios_premise_gas/inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1052" documentId="13_ncr:1_{D0F9393E-493D-4D41-96B2-57E4008F0D51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA45AAD1-F78C-4B10-A8EA-D86CA8AAC0B5}"/>
+  <xr:revisionPtr revIDLastSave="1115" documentId="13_ncr:1_{D0F9393E-493D-4D41-96B2-57E4008F0D51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02C36435-0722-4858-8B9B-C68B70933DB5}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6031" uniqueCount="759">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6060" uniqueCount="760">
   <si>
     <t>Database</t>
   </si>
@@ -2108,15 +2108,9 @@
     <t>market for shelter DLS, Tr2050</t>
   </si>
   <si>
-    <t>market for heat shelter, Tr2050</t>
-  </si>
-  <si>
     <t>Illumination</t>
   </si>
   <si>
-    <t>Space heating and cooling</t>
-  </si>
-  <si>
     <t>market for compact fluorescent lamp</t>
   </si>
   <si>
@@ -2228,9 +2222,6 @@
     <t>collective services</t>
   </si>
   <si>
-    <t>market for heat non-residential, Tr2050</t>
-  </si>
-  <si>
     <t>market for clay brick</t>
   </si>
   <si>
@@ -2264,12 +2255,6 @@
     <t>market for wastewater, average</t>
   </si>
   <si>
-    <t>market for EoL, Tr2050</t>
-  </si>
-  <si>
-    <t>waste treatment</t>
-  </si>
-  <si>
     <t>EoL composition based on ADEME Transition2050</t>
   </si>
   <si>
@@ -2313,6 +2298,24 @@
   </si>
   <si>
     <t>transport, passenger train</t>
+  </si>
+  <si>
+    <t>Space heating and cooling. Activity replaced by the new market for heat shelter in the generated database</t>
+  </si>
+  <si>
+    <t>municipal solid waste</t>
+  </si>
+  <si>
+    <t>treatment of municipal solid waste, sanitary landfill</t>
+  </si>
+  <si>
+    <t>Replaced by the new market in the generated database</t>
+  </si>
+  <si>
+    <t>empty market, proxy for market for heat non-shelter</t>
+  </si>
+  <si>
+    <t>Empty activity. Replaced by the market for non-residential shelter databases are generated</t>
   </si>
 </sst>
 </file>
@@ -2856,7 +2859,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AH1467"/>
+  <dimension ref="A1:AH1478"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="73.109375" customWidth="1"/>
@@ -28233,7 +28236,7 @@
         <v>57</v>
       </c>
       <c r="B1060" t="s">
-        <v>756</v>
+        <v>751</v>
       </c>
     </row>
     <row r="1061" spans="1:10" ht="15.6">
@@ -31687,7 +31690,7 @@
         <v>9.5016861504842378</v>
       </c>
       <c r="D1259" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="G1259" t="s">
         <v>96</v>
@@ -32897,7 +32900,7 @@
         <v>1</v>
       </c>
       <c r="B1329" s="23" t="s">
-        <v>689</v>
+        <v>758</v>
       </c>
     </row>
     <row r="1330" spans="1:9">
@@ -32907,7 +32910,6 @@
       <c r="B1330" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="H1330" s="55"/>
     </row>
     <row r="1331" spans="1:9">
       <c r="A1331" s="24" t="s">
@@ -32916,17 +32918,14 @@
       <c r="B1331" s="13">
         <v>1</v>
       </c>
-      <c r="F1331" s="13"/>
-      <c r="H1331" s="13"/>
     </row>
     <row r="1332" spans="1:9">
       <c r="A1332" s="24" t="s">
         <v>4</v>
       </c>
       <c r="B1332" s="13" t="s">
-        <v>688</v>
-      </c>
-      <c r="F1332" s="13"/>
+        <v>758</v>
+      </c>
     </row>
     <row r="1333" spans="1:9">
       <c r="A1333" s="24" t="s">
@@ -32935,14 +32934,13 @@
       <c r="B1333" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="F1333" s="20"/>
     </row>
     <row r="1334" spans="1:9">
       <c r="A1334" s="24" t="s">
         <v>6</v>
       </c>
       <c r="B1334" s="13" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="1335" spans="1:9">
@@ -32992,17 +32990,17 @@
       </c>
     </row>
     <row r="1338" spans="1:9">
-      <c r="A1338" s="13" t="s">
-        <v>689</v>
+      <c r="A1338" s="24" t="s">
+        <v>758</v>
       </c>
       <c r="B1338" s="13" t="s">
-        <v>688</v>
+        <v>758</v>
       </c>
       <c r="C1338">
         <v>1</v>
       </c>
-      <c r="D1338" t="s">
-        <v>6</v>
+      <c r="D1338" s="13" t="s">
+        <v>35</v>
       </c>
       <c r="G1338" t="s">
         <v>28</v>
@@ -33010,1994 +33008,2130 @@
       <c r="H1338" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="1339" spans="1:9" s="13" customFormat="1">
-      <c r="A1339" s="13" t="s">
+      <c r="I1338" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="1339" spans="1:9">
+      <c r="A1339" s="49"/>
+      <c r="B1339" s="50"/>
+      <c r="C1339" s="49"/>
+      <c r="D1339" s="49"/>
+      <c r="E1339" s="49"/>
+      <c r="F1339" s="49"/>
+      <c r="G1339" s="49"/>
+      <c r="H1339" s="49"/>
+      <c r="I1339" s="49"/>
+    </row>
+    <row r="1340" spans="1:9" ht="15.6">
+      <c r="A1340" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1340" s="23" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="1341" spans="1:9">
+      <c r="A1341" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1341" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1341" s="55"/>
+    </row>
+    <row r="1342" spans="1:9">
+      <c r="A1342" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1342" s="13">
+        <v>1</v>
+      </c>
+      <c r="F1342" s="13"/>
+      <c r="H1342" s="13"/>
+    </row>
+    <row r="1343" spans="1:9">
+      <c r="A1343" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1343" s="13" t="s">
+        <v>688</v>
+      </c>
+      <c r="F1343" s="13"/>
+    </row>
+    <row r="1344" spans="1:9">
+      <c r="A1344" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1344" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1344" s="20"/>
+    </row>
+    <row r="1345" spans="1:9">
+      <c r="A1345" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1345" s="13" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1346" spans="1:9">
+      <c r="A1346" s="24" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="1347" spans="1:9" ht="15.6">
+      <c r="A1347" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1347" s="25"/>
+      <c r="D1347" s="26"/>
+      <c r="E1347" s="26"/>
+      <c r="F1347" s="26"/>
+      <c r="G1347" s="26"/>
+      <c r="H1347" s="26"/>
+      <c r="I1347" s="26"/>
+    </row>
+    <row r="1348" spans="1:9">
+      <c r="A1348" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1348" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1348" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1348" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1348" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="F1348" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1348" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1348" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1348" s="24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1349" spans="1:9">
+      <c r="A1349" s="13" t="s">
+        <v>689</v>
+      </c>
+      <c r="B1349" s="13" t="s">
+        <v>688</v>
+      </c>
+      <c r="C1349">
+        <v>1</v>
+      </c>
+      <c r="D1349" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1349" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1349" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="1350" spans="1:9" s="13" customFormat="1">
+      <c r="A1350" s="13" t="s">
+        <v>535</v>
+      </c>
+      <c r="B1350" s="13" t="s">
+        <v>536</v>
+      </c>
+      <c r="C1350" s="20">
+        <v>2228.7496354420773</v>
+      </c>
+      <c r="D1350" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1350" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1350" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1350" s="13" t="s">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="1351" spans="1:9">
+      <c r="A1351" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1351" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1351" s="65">
+        <v>11.624825581395351</v>
+      </c>
+      <c r="D1351" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1351" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1351" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1351" t="s">
         <v>690</v>
       </c>
-      <c r="B1339" s="13" t="s">
-        <v>488</v>
-      </c>
-      <c r="C1339" s="20">
-        <v>2228.7496354420773</v>
-      </c>
-      <c r="D1339" t="s">
-        <v>35</v>
-      </c>
-      <c r="G1339" s="13" t="s">
+    </row>
+    <row r="1352" spans="1:9">
+      <c r="A1352" t="s">
+        <v>691</v>
+      </c>
+      <c r="B1352" t="s">
+        <v>692</v>
+      </c>
+      <c r="C1352" s="41">
+        <v>1</v>
+      </c>
+      <c r="D1352" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1352" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1352" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1353" spans="1:9">
+      <c r="A1353" t="s">
+        <v>693</v>
+      </c>
+      <c r="B1353" t="s">
+        <v>694</v>
+      </c>
+      <c r="C1353" s="41">
+        <v>9.7226201036316464</v>
+      </c>
+      <c r="D1353" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1353" t="s">
+        <v>134</v>
+      </c>
+      <c r="H1353" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1354" spans="1:9">
+      <c r="A1354" t="s">
+        <v>695</v>
+      </c>
+      <c r="B1354" t="s">
+        <v>696</v>
+      </c>
+      <c r="C1354" s="41">
+        <v>1.4885317466709565E-2</v>
+      </c>
+      <c r="D1354" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1354" t="s">
+        <v>134</v>
+      </c>
+      <c r="H1354" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1355" spans="1:9">
+      <c r="A1355" t="s">
+        <v>697</v>
+      </c>
+      <c r="B1355" t="s">
+        <v>698</v>
+      </c>
+      <c r="C1355" s="41">
+        <v>2.9533786710786259E-2</v>
+      </c>
+      <c r="D1355" t="s">
+        <v>91</v>
+      </c>
+      <c r="G1355" t="s">
+        <v>134</v>
+      </c>
+      <c r="H1355" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1356" spans="1:9">
+      <c r="A1356" t="s">
+        <v>699</v>
+      </c>
+      <c r="B1356" t="s">
+        <v>700</v>
+      </c>
+      <c r="C1356" s="41">
+        <v>0.12822525947672769</v>
+      </c>
+      <c r="D1356" t="s">
+        <v>91</v>
+      </c>
+      <c r="G1356" t="s">
+        <v>134</v>
+      </c>
+      <c r="H1356" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1357" spans="1:9">
+      <c r="A1357" t="s">
+        <v>701</v>
+      </c>
+      <c r="B1357" t="s">
+        <v>702</v>
+      </c>
+      <c r="C1357" s="41">
+        <v>17.155020006048819</v>
+      </c>
+      <c r="D1357" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1357" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1357" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1358" spans="1:9">
+      <c r="A1358" s="49"/>
+      <c r="B1358" s="50"/>
+      <c r="C1358" s="49"/>
+      <c r="D1358" s="49"/>
+      <c r="E1358" s="49"/>
+      <c r="F1358" s="49"/>
+      <c r="G1358" s="49"/>
+      <c r="H1358" s="49"/>
+      <c r="I1358" s="49"/>
+    </row>
+    <row r="1359" spans="1:9" ht="15.6">
+      <c r="A1359" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1359" s="23" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="1360" spans="1:9">
+      <c r="A1360" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1360" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="H1339" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1339" s="13" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="1340" spans="1:9">
-      <c r="A1340" t="s">
-        <v>27</v>
-      </c>
-      <c r="B1340" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="C1340" s="65">
-        <v>11.624825581395351</v>
-      </c>
-      <c r="D1340" t="s">
-        <v>19</v>
-      </c>
-      <c r="G1340" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1340" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1340" t="s">
-        <v>691</v>
-      </c>
-    </row>
-    <row r="1341" spans="1:9">
-      <c r="A1341" t="s">
-        <v>693</v>
-      </c>
-      <c r="B1341" t="s">
-        <v>694</v>
-      </c>
-      <c r="C1341" s="41">
+      <c r="H1360" s="55"/>
+    </row>
+    <row r="1361" spans="1:9">
+      <c r="A1361" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1361" s="13">
         <v>1</v>
       </c>
-      <c r="D1341" t="s">
+      <c r="F1361" s="13"/>
+      <c r="H1361" s="13"/>
+    </row>
+    <row r="1362" spans="1:9">
+      <c r="A1362" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1362" s="13" t="s">
+        <v>705</v>
+      </c>
+      <c r="F1362" s="13"/>
+    </row>
+    <row r="1363" spans="1:9">
+      <c r="A1363" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1363" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1363" s="20"/>
+    </row>
+    <row r="1364" spans="1:9">
+      <c r="A1364" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="G1341" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1341" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="1342" spans="1:9">
-      <c r="A1342" t="s">
-        <v>695</v>
-      </c>
-      <c r="B1342" t="s">
-        <v>696</v>
-      </c>
-      <c r="C1342" s="41">
-        <v>9.7226201036316464</v>
-      </c>
-      <c r="D1342" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1342" t="s">
-        <v>134</v>
-      </c>
-      <c r="H1342" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="1343" spans="1:9">
-      <c r="A1343" t="s">
-        <v>697</v>
-      </c>
-      <c r="B1343" t="s">
-        <v>698</v>
-      </c>
-      <c r="C1343" s="41">
-        <v>1.4885317466709565E-2</v>
-      </c>
-      <c r="D1343" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1343" t="s">
-        <v>134</v>
-      </c>
-      <c r="H1343" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="1344" spans="1:9">
-      <c r="A1344" t="s">
-        <v>699</v>
-      </c>
-      <c r="B1344" t="s">
-        <v>700</v>
-      </c>
-      <c r="C1344" s="41">
-        <v>2.9533786710786259E-2</v>
-      </c>
-      <c r="D1344" t="s">
-        <v>91</v>
-      </c>
-      <c r="G1344" t="s">
-        <v>134</v>
-      </c>
-      <c r="H1344" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="1345" spans="1:9">
-      <c r="A1345" t="s">
-        <v>701</v>
-      </c>
-      <c r="B1345" t="s">
-        <v>702</v>
-      </c>
-      <c r="C1345" s="41">
-        <v>0.12822525947672769</v>
-      </c>
-      <c r="D1345" t="s">
-        <v>91</v>
-      </c>
-      <c r="G1345" t="s">
-        <v>134</v>
-      </c>
-      <c r="H1345" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="1346" spans="1:9">
-      <c r="A1346" t="s">
-        <v>703</v>
-      </c>
-      <c r="B1346" t="s">
+      <c r="B1364" s="13" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1365" spans="1:9">
+      <c r="A1365" s="24" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="1366" spans="1:9" ht="15.6">
+      <c r="A1366" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1366" s="25"/>
+      <c r="D1366" s="26"/>
+      <c r="E1366" s="26"/>
+      <c r="F1366" s="26"/>
+      <c r="G1366" s="26"/>
+      <c r="H1366" s="26"/>
+      <c r="I1366" s="26"/>
+    </row>
+    <row r="1367" spans="1:9">
+      <c r="A1367" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1367" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1367" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1367" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1367" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="F1367" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1367" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1367" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1367" s="24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1368" spans="1:9">
+      <c r="A1368" s="13" t="s">
         <v>704</v>
       </c>
-      <c r="C1346" s="41">
-        <v>17.155020006048819</v>
-      </c>
-      <c r="D1346" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1346" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1346" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="1347" spans="1:9">
-      <c r="A1347" s="49"/>
-      <c r="B1347" s="50"/>
-      <c r="C1347" s="49"/>
-      <c r="D1347" s="49"/>
-      <c r="E1347" s="49"/>
-      <c r="F1347" s="49"/>
-      <c r="G1347" s="49"/>
-      <c r="H1347" s="49"/>
-      <c r="I1347" s="49"/>
-    </row>
-    <row r="1348" spans="1:9" ht="15.6">
-      <c r="A1348" s="18" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1348" s="23" t="s">
-        <v>706</v>
-      </c>
-    </row>
-    <row r="1349" spans="1:9">
-      <c r="A1349" s="24" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1349" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1349" s="55"/>
-    </row>
-    <row r="1350" spans="1:9">
-      <c r="A1350" s="24" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1350" s="13">
-        <v>1</v>
-      </c>
-      <c r="F1350" s="13"/>
-      <c r="H1350" s="13"/>
-    </row>
-    <row r="1351" spans="1:9">
-      <c r="A1351" s="24" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1351" s="13" t="s">
-        <v>707</v>
-      </c>
-      <c r="F1351" s="13"/>
-    </row>
-    <row r="1352" spans="1:9">
-      <c r="A1352" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="B1352" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="F1352" s="20"/>
-    </row>
-    <row r="1353" spans="1:9">
-      <c r="A1353" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1353" s="13" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="1354" spans="1:9">
-      <c r="A1354" s="24" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="1355" spans="1:9" ht="15.6">
-      <c r="A1355" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1355" s="25"/>
-      <c r="D1355" s="26"/>
-      <c r="E1355" s="26"/>
-      <c r="F1355" s="26"/>
-      <c r="G1355" s="26"/>
-      <c r="H1355" s="26"/>
-      <c r="I1355" s="26"/>
-    </row>
-    <row r="1356" spans="1:9">
-      <c r="A1356" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1356" s="23" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1356" s="30" t="s">
-        <v>9</v>
-      </c>
-      <c r="D1356" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1356" s="24" t="s">
-        <v>81</v>
-      </c>
-      <c r="F1356" s="24" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1356" s="24" t="s">
-        <v>2</v>
-      </c>
-      <c r="H1356" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1356" s="24" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="1357" spans="1:9">
-      <c r="A1357" s="13" t="s">
-        <v>706</v>
-      </c>
-      <c r="B1357" s="13" t="s">
-        <v>707</v>
-      </c>
-      <c r="C1357">
-        <v>1</v>
-      </c>
-      <c r="D1357" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1357" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1357" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="1358" spans="1:9">
-      <c r="A1358" t="s">
-        <v>27</v>
-      </c>
-      <c r="B1358" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="C1358" s="65">
-        <v>68.516800000000003</v>
-      </c>
-      <c r="D1358" t="s">
-        <v>19</v>
-      </c>
-      <c r="G1358" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1358" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="1359" spans="1:9">
-      <c r="A1359" t="s">
-        <v>708</v>
-      </c>
-      <c r="B1359" t="s">
-        <v>718</v>
-      </c>
-      <c r="C1359" s="41">
-        <v>0.1</v>
-      </c>
-      <c r="D1359" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1359" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1359" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="1360" spans="1:9">
-      <c r="A1360" t="s">
-        <v>709</v>
-      </c>
-      <c r="B1360" t="s">
-        <v>719</v>
-      </c>
-      <c r="C1360" s="41">
-        <v>0.4</v>
-      </c>
-      <c r="D1360" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1360" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1360" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="1361" spans="1:9">
-      <c r="A1361" t="s">
-        <v>710</v>
-      </c>
-      <c r="B1361" t="s">
-        <v>720</v>
-      </c>
-      <c r="C1361" s="41">
-        <v>0.4</v>
-      </c>
-      <c r="D1361" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1361" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1361" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="1362" spans="1:9">
-      <c r="A1362" t="s">
-        <v>711</v>
-      </c>
-      <c r="B1362" t="s">
-        <v>721</v>
-      </c>
-      <c r="C1362" s="41">
-        <v>0</v>
-      </c>
-      <c r="D1362" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1362" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1362" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="1363" spans="1:9">
-      <c r="A1363" t="s">
-        <v>712</v>
-      </c>
-      <c r="B1363" t="s">
-        <v>722</v>
-      </c>
-      <c r="C1363" s="41">
-        <v>0</v>
-      </c>
-      <c r="D1363" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1363" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1363" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="1364" spans="1:9">
-      <c r="A1364" t="s">
-        <v>713</v>
-      </c>
-      <c r="B1364" t="s">
-        <v>723</v>
-      </c>
-      <c r="C1364" s="41">
-        <v>0</v>
-      </c>
-      <c r="D1364" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1364" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1364" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="1365" spans="1:9">
-      <c r="A1365" t="s">
-        <v>714</v>
-      </c>
-      <c r="B1365" t="s">
-        <v>724</v>
-      </c>
-      <c r="C1365">
-        <v>0</v>
-      </c>
-      <c r="D1365" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1365" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1365" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="1366" spans="1:9">
-      <c r="A1366" t="s">
-        <v>715</v>
-      </c>
-      <c r="B1366" t="s">
-        <v>725</v>
-      </c>
-      <c r="C1366">
-        <v>0</v>
-      </c>
-      <c r="D1366" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1366" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1366" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="1367" spans="1:9">
-      <c r="A1367" t="s">
-        <v>716</v>
-      </c>
-      <c r="B1367" t="s">
-        <v>726</v>
-      </c>
-      <c r="C1367">
-        <v>0.6</v>
-      </c>
-      <c r="D1367" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1367" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1367" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="1368" spans="1:9">
-      <c r="A1368" t="s">
-        <v>717</v>
-      </c>
-      <c r="B1368" t="s">
-        <v>727</v>
+      <c r="B1368" s="13" t="s">
+        <v>705</v>
       </c>
       <c r="C1368">
         <v>1</v>
       </c>
       <c r="D1368" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="G1368" t="s">
-        <v>134</v>
+        <v>28</v>
       </c>
       <c r="H1368" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
     </row>
     <row r="1369" spans="1:9">
-      <c r="A1369" s="49"/>
-      <c r="B1369" s="50"/>
-      <c r="C1369" s="49"/>
-      <c r="D1369" s="49"/>
-      <c r="E1369" s="49"/>
-      <c r="F1369" s="49"/>
-      <c r="G1369" s="49"/>
-      <c r="H1369" s="49"/>
-      <c r="I1369" s="49"/>
-    </row>
-    <row r="1370" spans="1:9" ht="15.6">
-      <c r="A1370" s="18" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1370" s="23" t="s">
-        <v>728</v>
+      <c r="A1369" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1369" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1369" s="65">
+        <v>68.516800000000003</v>
+      </c>
+      <c r="D1369" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1369" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1369" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1370" spans="1:9">
+      <c r="A1370" t="s">
+        <v>706</v>
+      </c>
+      <c r="B1370" t="s">
+        <v>716</v>
+      </c>
+      <c r="C1370" s="41">
+        <v>0.1</v>
+      </c>
+      <c r="D1370" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1370" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1370" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="1371" spans="1:9">
-      <c r="A1371" s="24" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1371" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1371" s="55"/>
+      <c r="A1371" t="s">
+        <v>707</v>
+      </c>
+      <c r="B1371" t="s">
+        <v>717</v>
+      </c>
+      <c r="C1371" s="41">
+        <v>0.4</v>
+      </c>
+      <c r="D1371" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1371" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1371" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="1372" spans="1:9">
-      <c r="A1372" s="24" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1372" s="13">
-        <v>1</v>
-      </c>
-      <c r="F1372" s="13"/>
-      <c r="H1372" s="13"/>
+      <c r="A1372" t="s">
+        <v>708</v>
+      </c>
+      <c r="B1372" t="s">
+        <v>718</v>
+      </c>
+      <c r="C1372" s="41">
+        <v>0.4</v>
+      </c>
+      <c r="D1372" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1372" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1372" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="1373" spans="1:9">
-      <c r="A1373" s="24" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1373" s="13" t="s">
-        <v>729</v>
-      </c>
-      <c r="F1373" s="13"/>
+      <c r="A1373" t="s">
+        <v>709</v>
+      </c>
+      <c r="B1373" t="s">
+        <v>719</v>
+      </c>
+      <c r="C1373" s="41">
+        <v>0</v>
+      </c>
+      <c r="D1373" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1373" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1373" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="1374" spans="1:9">
-      <c r="A1374" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="B1374" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="F1374" s="20"/>
+      <c r="A1374" t="s">
+        <v>710</v>
+      </c>
+      <c r="B1374" t="s">
+        <v>720</v>
+      </c>
+      <c r="C1374" s="41">
+        <v>0</v>
+      </c>
+      <c r="D1374" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1374" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1374" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="1375" spans="1:9">
-      <c r="A1375" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1375" s="13" t="s">
-        <v>6</v>
+      <c r="A1375" t="s">
+        <v>711</v>
+      </c>
+      <c r="B1375" t="s">
+        <v>721</v>
+      </c>
+      <c r="C1375" s="41">
+        <v>0</v>
+      </c>
+      <c r="D1375" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1375" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1375" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="1376" spans="1:9">
-      <c r="A1376" s="24" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="1377" spans="1:9" ht="15.6">
-      <c r="A1377" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1377" s="25"/>
-      <c r="D1377" s="26"/>
-      <c r="E1377" s="26"/>
-      <c r="F1377" s="26"/>
-      <c r="G1377" s="26"/>
-      <c r="H1377" s="26"/>
-      <c r="I1377" s="26"/>
+      <c r="A1376" t="s">
+        <v>712</v>
+      </c>
+      <c r="B1376" t="s">
+        <v>722</v>
+      </c>
+      <c r="C1376">
+        <v>0</v>
+      </c>
+      <c r="D1376" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1376" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1376" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1377" spans="1:9">
+      <c r="A1377" t="s">
+        <v>713</v>
+      </c>
+      <c r="B1377" t="s">
+        <v>723</v>
+      </c>
+      <c r="C1377">
+        <v>0</v>
+      </c>
+      <c r="D1377" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1377" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1377" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="1378" spans="1:9">
-      <c r="A1378" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1378" s="23" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1378" s="30" t="s">
-        <v>9</v>
-      </c>
-      <c r="D1378" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1378" s="24" t="s">
-        <v>81</v>
-      </c>
-      <c r="F1378" s="24" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1378" s="24" t="s">
-        <v>2</v>
-      </c>
-      <c r="H1378" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1378" s="24" t="s">
-        <v>11</v>
+      <c r="A1378" t="s">
+        <v>714</v>
+      </c>
+      <c r="B1378" t="s">
+        <v>724</v>
+      </c>
+      <c r="C1378">
+        <v>0.6</v>
+      </c>
+      <c r="D1378" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1378" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1378" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="1379" spans="1:9">
-      <c r="A1379" s="13" t="s">
-        <v>728</v>
-      </c>
-      <c r="B1379" s="13" t="s">
-        <v>729</v>
+      <c r="A1379" t="s">
+        <v>715</v>
+      </c>
+      <c r="B1379" t="s">
+        <v>725</v>
       </c>
       <c r="C1379">
         <v>1</v>
       </c>
       <c r="D1379" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1379" t="s">
+        <v>134</v>
+      </c>
+      <c r="H1379" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1380" spans="1:9">
+      <c r="A1380" s="49"/>
+      <c r="B1380" s="50"/>
+      <c r="C1380" s="49"/>
+      <c r="D1380" s="49"/>
+      <c r="E1380" s="49"/>
+      <c r="F1380" s="49"/>
+      <c r="G1380" s="49"/>
+      <c r="H1380" s="49"/>
+      <c r="I1380" s="49"/>
+    </row>
+    <row r="1381" spans="1:9" ht="15.6">
+      <c r="A1381" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1381" s="23" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="1382" spans="1:9">
+      <c r="A1382" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1382" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1382" s="55"/>
+    </row>
+    <row r="1383" spans="1:9">
+      <c r="A1383" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1383" s="13">
+        <v>1</v>
+      </c>
+      <c r="F1383" s="13"/>
+      <c r="H1383" s="13"/>
+    </row>
+    <row r="1384" spans="1:9">
+      <c r="A1384" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1384" s="13" t="s">
+        <v>727</v>
+      </c>
+      <c r="F1384" s="13"/>
+    </row>
+    <row r="1385" spans="1:9">
+      <c r="A1385" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1385" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1385" s="20"/>
+    </row>
+    <row r="1386" spans="1:9">
+      <c r="A1386" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="G1379" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1379" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="1380" spans="1:9">
-      <c r="A1380" s="13" t="s">
-        <v>730</v>
-      </c>
-      <c r="B1380" s="13" t="s">
-        <v>488</v>
-      </c>
-      <c r="C1380" s="20">
-        <v>1410.5830808917863</v>
-      </c>
-      <c r="D1380" t="s">
-        <v>35</v>
-      </c>
-      <c r="E1380" s="13"/>
-      <c r="F1380" s="13"/>
-      <c r="G1380" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1380" s="13" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="1381" spans="1:9">
-      <c r="A1381" t="s">
-        <v>27</v>
-      </c>
-      <c r="B1381" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="C1381" s="65">
-        <v>58.887640000000005</v>
-      </c>
-      <c r="D1381" t="s">
-        <v>19</v>
-      </c>
-      <c r="G1381" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1381" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1381" t="s">
-        <v>691</v>
-      </c>
-    </row>
-    <row r="1382" spans="1:9">
-      <c r="A1382" t="s">
-        <v>699</v>
-      </c>
-      <c r="B1382" t="s">
-        <v>700</v>
-      </c>
-      <c r="C1382" s="41">
-        <v>2.2536817079020791E-2</v>
-      </c>
-      <c r="D1382" t="s">
-        <v>91</v>
-      </c>
-      <c r="G1382" t="s">
-        <v>134</v>
-      </c>
-      <c r="H1382" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1382" t="s">
-        <v>733</v>
-      </c>
-    </row>
-    <row r="1383" spans="1:9">
-      <c r="A1383" t="s">
-        <v>701</v>
-      </c>
-      <c r="B1383" t="s">
-        <v>702</v>
-      </c>
-      <c r="C1383" s="41">
-        <v>2.2463377515747087E-2</v>
-      </c>
-      <c r="D1383" t="s">
-        <v>91</v>
-      </c>
-      <c r="G1383" t="s">
-        <v>134</v>
-      </c>
-      <c r="H1383" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1383" t="s">
-        <v>733</v>
-      </c>
-    </row>
-    <row r="1384" spans="1:9">
-      <c r="A1384" t="s">
-        <v>703</v>
-      </c>
-      <c r="B1384" t="s">
-        <v>704</v>
-      </c>
-      <c r="C1384" s="41">
-        <v>2.5508072892144331</v>
-      </c>
-      <c r="D1384" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1384" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1384" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1384" t="s">
-        <v>733</v>
-      </c>
-    </row>
-    <row r="1385" spans="1:9">
-      <c r="A1385" t="s">
-        <v>731</v>
-      </c>
-      <c r="B1385" t="s">
-        <v>732</v>
-      </c>
-      <c r="C1385" s="41">
-        <v>4.7112989220033237</v>
-      </c>
-      <c r="D1385" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1385" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1385" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1385" t="s">
-        <v>733</v>
-      </c>
-    </row>
-    <row r="1386" spans="1:9">
-      <c r="A1386" t="s">
-        <v>693</v>
-      </c>
-      <c r="B1386" t="s">
-        <v>694</v>
-      </c>
-      <c r="C1386" s="41">
-        <v>4</v>
-      </c>
-      <c r="D1386" t="s">
+      <c r="B1386" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="G1386" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1386" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1386" t="s">
-        <v>733</v>
-      </c>
     </row>
     <row r="1387" spans="1:9">
-      <c r="A1387" s="49"/>
-      <c r="B1387" s="50"/>
-      <c r="C1387" s="49"/>
-      <c r="D1387" s="49"/>
-      <c r="E1387" s="49"/>
-      <c r="F1387" s="49"/>
-      <c r="G1387" s="49"/>
-      <c r="H1387" s="49"/>
-      <c r="I1387" s="49"/>
+      <c r="A1387" s="24" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="1388" spans="1:9" ht="15.6">
       <c r="A1388" s="18" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1388" s="23" t="s">
-        <v>734</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="C1388" s="25"/>
+      <c r="D1388" s="26"/>
+      <c r="E1388" s="26"/>
+      <c r="F1388" s="26"/>
+      <c r="G1388" s="26"/>
+      <c r="H1388" s="26"/>
+      <c r="I1388" s="26"/>
     </row>
     <row r="1389" spans="1:9">
       <c r="A1389" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1389" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1389" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1389" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1389" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="F1389" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1389" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="B1389" s="13" t="s">
+      <c r="H1389" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1389" s="24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1390" spans="1:9">
+      <c r="A1390" s="13" t="s">
+        <v>726</v>
+      </c>
+      <c r="B1390" s="13" t="s">
+        <v>727</v>
+      </c>
+      <c r="C1390">
+        <v>1</v>
+      </c>
+      <c r="D1390" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1390" t="s">
         <v>28</v>
       </c>
-      <c r="H1389" s="55"/>
-    </row>
-    <row r="1390" spans="1:9">
-      <c r="A1390" s="24" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1390" s="13">
-        <v>1</v>
-      </c>
-      <c r="F1390" s="13"/>
-      <c r="H1390" s="13"/>
+      <c r="H1390" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="1391" spans="1:9">
-      <c r="A1391" s="24" t="s">
+      <c r="A1391" s="13" t="s">
+        <v>758</v>
+      </c>
+      <c r="B1391" s="13" t="s">
+        <v>758</v>
+      </c>
+      <c r="C1391" s="20">
+        <v>1410.5830808917863</v>
+      </c>
+      <c r="D1391" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1391" s="13"/>
+      <c r="F1391" s="13"/>
+      <c r="G1391" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1391" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1391" s="13" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="1392" spans="1:9">
+      <c r="A1392" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1392" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1392" s="65">
+        <v>58.887640000000005</v>
+      </c>
+      <c r="D1392" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1392" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1392" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1392" t="s">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="1393" spans="1:9">
+      <c r="A1393" t="s">
+        <v>697</v>
+      </c>
+      <c r="B1393" t="s">
+        <v>698</v>
+      </c>
+      <c r="C1393" s="41">
+        <v>2.2536817079020791E-2</v>
+      </c>
+      <c r="D1393" t="s">
+        <v>91</v>
+      </c>
+      <c r="G1393" t="s">
+        <v>134</v>
+      </c>
+      <c r="H1393" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1393" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="1394" spans="1:9">
+      <c r="A1394" t="s">
+        <v>699</v>
+      </c>
+      <c r="B1394" t="s">
+        <v>700</v>
+      </c>
+      <c r="C1394" s="41">
+        <v>2.2463377515747087E-2</v>
+      </c>
+      <c r="D1394" t="s">
+        <v>91</v>
+      </c>
+      <c r="G1394" t="s">
+        <v>134</v>
+      </c>
+      <c r="H1394" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1394" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="1395" spans="1:9">
+      <c r="A1395" t="s">
+        <v>701</v>
+      </c>
+      <c r="B1395" t="s">
+        <v>702</v>
+      </c>
+      <c r="C1395" s="41">
+        <v>2.5508072892144331</v>
+      </c>
+      <c r="D1395" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1395" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1395" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1395" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="1396" spans="1:9">
+      <c r="A1396" t="s">
+        <v>728</v>
+      </c>
+      <c r="B1396" t="s">
+        <v>729</v>
+      </c>
+      <c r="C1396" s="41">
+        <v>4.7112989220033237</v>
+      </c>
+      <c r="D1396" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1396" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1396" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1396" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="1397" spans="1:9">
+      <c r="A1397" t="s">
+        <v>691</v>
+      </c>
+      <c r="B1397" t="s">
+        <v>692</v>
+      </c>
+      <c r="C1397" s="41">
         <v>4</v>
-      </c>
-      <c r="B1391" s="13" t="s">
-        <v>735</v>
-      </c>
-      <c r="F1391" s="13"/>
-    </row>
-    <row r="1392" spans="1:9">
-      <c r="A1392" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="B1392" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="F1392" s="20"/>
-    </row>
-    <row r="1393" spans="1:9">
-      <c r="A1393" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1393" s="13" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="1394" spans="1:9">
-      <c r="A1394" s="24" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="1395" spans="1:9" ht="15.6">
-      <c r="A1395" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1395" s="25"/>
-      <c r="D1395" s="26"/>
-      <c r="E1395" s="26"/>
-      <c r="F1395" s="26"/>
-      <c r="G1395" s="26"/>
-      <c r="H1395" s="26"/>
-      <c r="I1395" s="26"/>
-    </row>
-    <row r="1396" spans="1:9">
-      <c r="A1396" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1396" s="23" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1396" s="30" t="s">
-        <v>9</v>
-      </c>
-      <c r="D1396" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1396" s="24" t="s">
-        <v>81</v>
-      </c>
-      <c r="F1396" s="24" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1396" s="24" t="s">
-        <v>2</v>
-      </c>
-      <c r="H1396" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1396" s="24" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="1397" spans="1:9">
-      <c r="A1397" s="13" t="s">
-        <v>734</v>
-      </c>
-      <c r="B1397" s="13" t="s">
-        <v>735</v>
-      </c>
-      <c r="C1397">
-        <v>1</v>
       </c>
       <c r="D1397" t="s">
         <v>6</v>
       </c>
       <c r="G1397" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1397" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1397" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="1398" spans="1:9">
+      <c r="A1398" s="49"/>
+      <c r="B1398" s="50"/>
+      <c r="C1398" s="49"/>
+      <c r="D1398" s="49"/>
+      <c r="E1398" s="49"/>
+      <c r="F1398" s="49"/>
+      <c r="G1398" s="49"/>
+      <c r="H1398" s="49"/>
+      <c r="I1398" s="49"/>
+    </row>
+    <row r="1399" spans="1:9" ht="15.6">
+      <c r="A1399" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1399" s="23" t="s">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="1400" spans="1:9">
+      <c r="A1400" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1400" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="H1397" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="1398" spans="1:9">
-      <c r="A1398" s="13" t="s">
-        <v>730</v>
-      </c>
-      <c r="B1398" s="13" t="s">
-        <v>488</v>
-      </c>
-      <c r="C1398" s="20">
-        <v>894.81948850800109</v>
-      </c>
-      <c r="D1398" t="s">
-        <v>35</v>
-      </c>
-      <c r="E1398" s="13"/>
-      <c r="F1398" s="13"/>
-      <c r="G1398" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1398" s="13" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="1399" spans="1:9">
-      <c r="A1399" t="s">
-        <v>27</v>
-      </c>
-      <c r="B1399" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="C1399" s="65">
-        <v>36.161279999999998</v>
-      </c>
-      <c r="D1399" t="s">
-        <v>19</v>
-      </c>
-      <c r="G1399" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1399" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1399" t="s">
-        <v>691</v>
-      </c>
-    </row>
-    <row r="1400" spans="1:9">
-      <c r="A1400" t="s">
-        <v>699</v>
-      </c>
-      <c r="B1400" t="s">
-        <v>700</v>
-      </c>
-      <c r="C1400" s="41">
-        <v>9.588780239886489E-3</v>
-      </c>
-      <c r="D1400" t="s">
-        <v>91</v>
-      </c>
-      <c r="G1400" t="s">
-        <v>134</v>
-      </c>
-      <c r="H1400" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1400" t="s">
-        <v>733</v>
-      </c>
+      <c r="H1400" s="55"/>
     </row>
     <row r="1401" spans="1:9">
-      <c r="A1401" t="s">
-        <v>701</v>
-      </c>
-      <c r="B1401" t="s">
-        <v>702</v>
-      </c>
-      <c r="C1401" s="41">
-        <v>6.5376650045297548E-3</v>
-      </c>
-      <c r="D1401" t="s">
-        <v>91</v>
-      </c>
-      <c r="G1401" t="s">
-        <v>134</v>
-      </c>
-      <c r="H1401" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1401" t="s">
-        <v>733</v>
-      </c>
+      <c r="A1401" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1401" s="13">
+        <v>1</v>
+      </c>
+      <c r="F1401" s="13"/>
+      <c r="H1401" s="13"/>
     </row>
     <row r="1402" spans="1:9">
-      <c r="A1402" t="s">
-        <v>703</v>
-      </c>
-      <c r="B1402" t="s">
-        <v>704</v>
-      </c>
-      <c r="C1402" s="41">
-        <v>0.91385899274745341</v>
-      </c>
-      <c r="D1402" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1402" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1402" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1402" t="s">
-        <v>733</v>
-      </c>
+      <c r="A1402" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1402" s="13" t="s">
+        <v>732</v>
+      </c>
+      <c r="F1402" s="13"/>
     </row>
     <row r="1403" spans="1:9">
-      <c r="A1403" t="s">
-        <v>731</v>
-      </c>
-      <c r="B1403" t="s">
-        <v>732</v>
-      </c>
-      <c r="C1403" s="41">
-        <v>2.6329079093854051</v>
-      </c>
-      <c r="D1403" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1403" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1403" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1403" t="s">
-        <v>733</v>
-      </c>
+      <c r="A1403" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1403" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1403" s="20"/>
     </row>
     <row r="1404" spans="1:9">
-      <c r="A1404" t="s">
-        <v>693</v>
-      </c>
-      <c r="B1404" t="s">
-        <v>694</v>
-      </c>
-      <c r="C1404" s="41">
-        <v>4</v>
-      </c>
-      <c r="D1404" t="s">
+      <c r="A1404" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="G1404" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1404" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1404" t="s">
-        <v>733</v>
+      <c r="B1404" s="13" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="1405" spans="1:9">
-      <c r="A1405" s="49"/>
-      <c r="B1405" s="50"/>
-      <c r="C1405" s="49"/>
-      <c r="D1405" s="49"/>
-      <c r="E1405" s="49"/>
-      <c r="F1405" s="49"/>
-      <c r="G1405" s="49"/>
-      <c r="H1405" s="49"/>
-      <c r="I1405" s="49"/>
+      <c r="A1405" s="24" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="1406" spans="1:9" ht="15.6">
       <c r="A1406" s="18" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1406" s="23" t="s">
-        <v>736</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="C1406" s="25"/>
+      <c r="D1406" s="26"/>
+      <c r="E1406" s="26"/>
+      <c r="F1406" s="26"/>
+      <c r="G1406" s="26"/>
+      <c r="H1406" s="26"/>
+      <c r="I1406" s="26"/>
     </row>
     <row r="1407" spans="1:9">
       <c r="A1407" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1407" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1407" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1407" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1407" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="F1407" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1407" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="B1407" s="13" t="s">
+      <c r="H1407" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1407" s="24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1408" spans="1:9">
+      <c r="A1408" s="13" t="s">
+        <v>731</v>
+      </c>
+      <c r="B1408" s="13" t="s">
+        <v>732</v>
+      </c>
+      <c r="C1408">
+        <v>1</v>
+      </c>
+      <c r="D1408" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1408" t="s">
         <v>28</v>
       </c>
-      <c r="H1407" s="55"/>
-    </row>
-    <row r="1408" spans="1:9">
-      <c r="A1408" s="24" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1408" s="13">
-        <v>1</v>
-      </c>
-      <c r="F1408" s="13"/>
-      <c r="H1408" s="13"/>
+      <c r="H1408" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="1409" spans="1:9">
-      <c r="A1409" s="24" t="s">
+      <c r="A1409" s="13" t="s">
+        <v>758</v>
+      </c>
+      <c r="B1409" s="13" t="s">
+        <v>758</v>
+      </c>
+      <c r="C1409" s="20">
+        <v>894.81948850800109</v>
+      </c>
+      <c r="D1409" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1409" s="13"/>
+      <c r="F1409" s="13"/>
+      <c r="G1409" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1409" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1410" spans="1:9">
+      <c r="A1410" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1410" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1410" s="65">
+        <v>36.161279999999998</v>
+      </c>
+      <c r="D1410" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1410" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1410" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1410" t="s">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="1411" spans="1:9">
+      <c r="A1411" t="s">
+        <v>697</v>
+      </c>
+      <c r="B1411" t="s">
+        <v>698</v>
+      </c>
+      <c r="C1411" s="41">
+        <v>9.588780239886489E-3</v>
+      </c>
+      <c r="D1411" t="s">
+        <v>91</v>
+      </c>
+      <c r="G1411" t="s">
+        <v>134</v>
+      </c>
+      <c r="H1411" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1411" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="1412" spans="1:9">
+      <c r="A1412" t="s">
+        <v>699</v>
+      </c>
+      <c r="B1412" t="s">
+        <v>700</v>
+      </c>
+      <c r="C1412" s="41">
+        <v>6.5376650045297548E-3</v>
+      </c>
+      <c r="D1412" t="s">
+        <v>91</v>
+      </c>
+      <c r="G1412" t="s">
+        <v>134</v>
+      </c>
+      <c r="H1412" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1412" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="1413" spans="1:9">
+      <c r="A1413" t="s">
+        <v>701</v>
+      </c>
+      <c r="B1413" t="s">
+        <v>702</v>
+      </c>
+      <c r="C1413" s="41">
+        <v>0.91385899274745341</v>
+      </c>
+      <c r="D1413" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1413" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1413" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1413" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="1414" spans="1:9">
+      <c r="A1414" t="s">
+        <v>728</v>
+      </c>
+      <c r="B1414" t="s">
+        <v>729</v>
+      </c>
+      <c r="C1414" s="41">
+        <v>2.6329079093854051</v>
+      </c>
+      <c r="D1414" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1414" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1414" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1414" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="1415" spans="1:9">
+      <c r="A1415" t="s">
+        <v>691</v>
+      </c>
+      <c r="B1415" t="s">
+        <v>692</v>
+      </c>
+      <c r="C1415" s="41">
         <v>4</v>
-      </c>
-      <c r="B1409" s="13" t="s">
-        <v>737</v>
-      </c>
-      <c r="F1409" s="13"/>
-    </row>
-    <row r="1410" spans="1:9">
-      <c r="A1410" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="B1410" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="F1410" s="20"/>
-    </row>
-    <row r="1411" spans="1:9">
-      <c r="A1411" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1411" s="13" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="1412" spans="1:9">
-      <c r="A1412" s="24" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="1413" spans="1:9" ht="15.6">
-      <c r="A1413" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1413" s="25"/>
-      <c r="D1413" s="26"/>
-      <c r="E1413" s="26"/>
-      <c r="F1413" s="26"/>
-      <c r="G1413" s="26"/>
-      <c r="H1413" s="26"/>
-      <c r="I1413" s="26"/>
-    </row>
-    <row r="1414" spans="1:9">
-      <c r="A1414" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1414" s="23" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1414" s="30" t="s">
-        <v>9</v>
-      </c>
-      <c r="D1414" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1414" s="24" t="s">
-        <v>81</v>
-      </c>
-      <c r="F1414" s="24" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1414" s="24" t="s">
-        <v>2</v>
-      </c>
-      <c r="H1414" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1414" s="24" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="1415" spans="1:9">
-      <c r="A1415" s="13" t="s">
-        <v>736</v>
-      </c>
-      <c r="B1415" s="13" t="s">
-        <v>737</v>
-      </c>
-      <c r="C1415">
-        <v>1</v>
       </c>
       <c r="D1415" t="s">
         <v>6</v>
       </c>
       <c r="G1415" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1415" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1415" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="1416" spans="1:9">
+      <c r="A1416" s="49"/>
+      <c r="B1416" s="50"/>
+      <c r="C1416" s="49"/>
+      <c r="D1416" s="49"/>
+      <c r="E1416" s="49"/>
+      <c r="F1416" s="49"/>
+      <c r="G1416" s="49"/>
+      <c r="H1416" s="49"/>
+      <c r="I1416" s="49"/>
+    </row>
+    <row r="1417" spans="1:9" ht="15.6">
+      <c r="A1417" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1417" s="23" t="s">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="1418" spans="1:9">
+      <c r="A1418" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1418" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="H1415" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="1416" spans="1:9">
-      <c r="A1416" s="13" t="s">
-        <v>730</v>
-      </c>
-      <c r="B1416" s="13" t="s">
-        <v>488</v>
-      </c>
-      <c r="C1416" s="20">
-        <v>1489.4729522387051</v>
-      </c>
-      <c r="D1416" t="s">
-        <v>35</v>
-      </c>
-      <c r="E1416" s="13"/>
-      <c r="F1416" s="13"/>
-      <c r="G1416" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1416" s="13" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="1417" spans="1:9">
-      <c r="A1417" t="s">
-        <v>27</v>
-      </c>
-      <c r="B1417" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="C1417" s="65">
-        <v>24.169328609229943</v>
-      </c>
-      <c r="D1417" t="s">
-        <v>19</v>
-      </c>
-      <c r="G1417" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1417" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1417" t="s">
-        <v>691</v>
-      </c>
-    </row>
-    <row r="1418" spans="1:9">
-      <c r="A1418" t="s">
-        <v>699</v>
-      </c>
-      <c r="B1418" t="s">
-        <v>700</v>
-      </c>
-      <c r="C1418" s="41">
-        <v>9.1578497118428651E-3</v>
-      </c>
-      <c r="D1418" t="s">
-        <v>91</v>
-      </c>
-      <c r="G1418" t="s">
-        <v>134</v>
-      </c>
-      <c r="H1418" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1418" t="s">
-        <v>733</v>
-      </c>
+      <c r="H1418" s="55"/>
     </row>
     <row r="1419" spans="1:9">
-      <c r="A1419" t="s">
-        <v>701</v>
-      </c>
-      <c r="B1419" t="s">
-        <v>702</v>
-      </c>
-      <c r="C1419" s="41">
-        <v>8.1936173025088151E-3</v>
-      </c>
-      <c r="D1419" t="s">
-        <v>91</v>
-      </c>
-      <c r="G1419" t="s">
-        <v>134</v>
-      </c>
-      <c r="H1419" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1419" t="s">
-        <v>733</v>
-      </c>
+      <c r="A1419" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1419" s="13">
+        <v>1</v>
+      </c>
+      <c r="F1419" s="13"/>
+      <c r="H1419" s="13"/>
     </row>
     <row r="1420" spans="1:9">
-      <c r="A1420" t="s">
-        <v>703</v>
-      </c>
-      <c r="B1420" t="s">
-        <v>704</v>
-      </c>
-      <c r="C1420" s="41">
-        <v>1.0519495105134982</v>
-      </c>
-      <c r="D1420" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1420" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1420" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1420" t="s">
-        <v>733</v>
-      </c>
+      <c r="A1420" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1420" s="13" t="s">
+        <v>734</v>
+      </c>
+      <c r="F1420" s="13"/>
     </row>
     <row r="1421" spans="1:9">
-      <c r="A1421" t="s">
-        <v>731</v>
-      </c>
-      <c r="B1421" t="s">
-        <v>732</v>
-      </c>
-      <c r="C1421" s="41">
-        <v>1.9865136400462349</v>
-      </c>
-      <c r="D1421" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1421" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1421" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1421" t="s">
-        <v>733</v>
-      </c>
+      <c r="A1421" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1421" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1421" s="20"/>
     </row>
     <row r="1422" spans="1:9">
-      <c r="A1422" t="s">
-        <v>693</v>
-      </c>
-      <c r="B1422" t="s">
-        <v>694</v>
-      </c>
-      <c r="C1422" s="41">
-        <v>4</v>
-      </c>
-      <c r="D1422" t="s">
+      <c r="A1422" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="G1422" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1422" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1422" t="s">
-        <v>733</v>
+      <c r="B1422" s="13" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="1423" spans="1:9">
-      <c r="A1423" s="49"/>
-      <c r="B1423" s="50"/>
-      <c r="C1423" s="49"/>
-      <c r="D1423" s="49"/>
-      <c r="E1423" s="49"/>
-      <c r="F1423" s="49"/>
-      <c r="G1423" s="49"/>
-      <c r="H1423" s="49"/>
-      <c r="I1423" s="49"/>
+      <c r="A1423" s="24" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="1424" spans="1:9" ht="15.6">
       <c r="A1424" s="18" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1424" s="23" t="s">
-        <v>738</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="C1424" s="25"/>
+      <c r="D1424" s="26"/>
+      <c r="E1424" s="26"/>
+      <c r="F1424" s="26"/>
+      <c r="G1424" s="26"/>
+      <c r="H1424" s="26"/>
+      <c r="I1424" s="26"/>
     </row>
     <row r="1425" spans="1:9">
       <c r="A1425" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1425" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1425" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1425" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1425" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="F1425" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1425" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="B1425" s="13" t="s">
+      <c r="H1425" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1425" s="24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1426" spans="1:9">
+      <c r="A1426" s="13" t="s">
+        <v>733</v>
+      </c>
+      <c r="B1426" s="13" t="s">
+        <v>734</v>
+      </c>
+      <c r="C1426">
+        <v>1</v>
+      </c>
+      <c r="D1426" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1426" t="s">
         <v>28</v>
       </c>
-      <c r="H1425" s="55"/>
-    </row>
-    <row r="1426" spans="1:9">
-      <c r="A1426" s="24" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1426" s="13">
-        <v>1</v>
-      </c>
-      <c r="F1426" s="13"/>
-      <c r="H1426" s="13"/>
+      <c r="H1426" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="1427" spans="1:9">
-      <c r="A1427" s="24" t="s">
+      <c r="A1427" s="13" t="s">
+        <v>758</v>
+      </c>
+      <c r="B1427" s="13" t="s">
+        <v>758</v>
+      </c>
+      <c r="C1427" s="20">
+        <v>1489.4729522387051</v>
+      </c>
+      <c r="D1427" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1427" s="13"/>
+      <c r="F1427" s="13"/>
+      <c r="G1427" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1427" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1428" spans="1:9">
+      <c r="A1428" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1428" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1428" s="65">
+        <v>24.169328609229943</v>
+      </c>
+      <c r="D1428" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1428" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1428" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1428" t="s">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="1429" spans="1:9">
+      <c r="A1429" t="s">
+        <v>697</v>
+      </c>
+      <c r="B1429" t="s">
+        <v>698</v>
+      </c>
+      <c r="C1429" s="41">
+        <v>9.1578497118428651E-3</v>
+      </c>
+      <c r="D1429" t="s">
+        <v>91</v>
+      </c>
+      <c r="G1429" t="s">
+        <v>134</v>
+      </c>
+      <c r="H1429" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1429" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="1430" spans="1:9">
+      <c r="A1430" t="s">
+        <v>699</v>
+      </c>
+      <c r="B1430" t="s">
+        <v>700</v>
+      </c>
+      <c r="C1430" s="41">
+        <v>8.1936173025088151E-3</v>
+      </c>
+      <c r="D1430" t="s">
+        <v>91</v>
+      </c>
+      <c r="G1430" t="s">
+        <v>134</v>
+      </c>
+      <c r="H1430" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1430" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="1431" spans="1:9">
+      <c r="A1431" t="s">
+        <v>701</v>
+      </c>
+      <c r="B1431" t="s">
+        <v>702</v>
+      </c>
+      <c r="C1431" s="41">
+        <v>1.0519495105134982</v>
+      </c>
+      <c r="D1431" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1431" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1431" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1431" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="1432" spans="1:9">
+      <c r="A1432" t="s">
+        <v>728</v>
+      </c>
+      <c r="B1432" t="s">
+        <v>729</v>
+      </c>
+      <c r="C1432" s="41">
+        <v>1.9865136400462349</v>
+      </c>
+      <c r="D1432" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1432" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1432" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1432" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="1433" spans="1:9">
+      <c r="A1433" t="s">
+        <v>691</v>
+      </c>
+      <c r="B1433" t="s">
+        <v>692</v>
+      </c>
+      <c r="C1433" s="41">
         <v>4</v>
-      </c>
-      <c r="B1427" s="13" t="s">
-        <v>739</v>
-      </c>
-      <c r="F1427" s="13"/>
-    </row>
-    <row r="1428" spans="1:9">
-      <c r="A1428" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="B1428" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="F1428" s="20"/>
-    </row>
-    <row r="1429" spans="1:9">
-      <c r="A1429" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1429" s="13" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="1430" spans="1:9">
-      <c r="A1430" s="24" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="1431" spans="1:9" ht="15.6">
-      <c r="A1431" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1431" s="25"/>
-      <c r="D1431" s="26"/>
-      <c r="E1431" s="26"/>
-      <c r="F1431" s="26"/>
-      <c r="G1431" s="26"/>
-      <c r="H1431" s="26"/>
-      <c r="I1431" s="26"/>
-    </row>
-    <row r="1432" spans="1:9">
-      <c r="A1432" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1432" s="23" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1432" s="30" t="s">
-        <v>9</v>
-      </c>
-      <c r="D1432" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1432" s="24" t="s">
-        <v>81</v>
-      </c>
-      <c r="F1432" s="24" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1432" s="24" t="s">
-        <v>2</v>
-      </c>
-      <c r="H1432" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1432" s="24" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="1433" spans="1:9">
-      <c r="A1433" s="13" t="s">
-        <v>738</v>
-      </c>
-      <c r="B1433" s="13" t="s">
-        <v>739</v>
-      </c>
-      <c r="C1433">
-        <v>1</v>
       </c>
       <c r="D1433" t="s">
         <v>6</v>
       </c>
       <c r="G1433" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1433" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1433" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="1434" spans="1:9">
+      <c r="A1434" s="49"/>
+      <c r="B1434" s="50"/>
+      <c r="C1434" s="49"/>
+      <c r="D1434" s="49"/>
+      <c r="E1434" s="49"/>
+      <c r="F1434" s="49"/>
+      <c r="G1434" s="49"/>
+      <c r="H1434" s="49"/>
+      <c r="I1434" s="49"/>
+    </row>
+    <row r="1435" spans="1:9" ht="15.6">
+      <c r="A1435" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1435" s="23" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="1436" spans="1:9">
+      <c r="A1436" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1436" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="H1433" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="1434" spans="1:9">
-      <c r="A1434" s="13" t="s">
-        <v>730</v>
-      </c>
-      <c r="B1434" s="13" t="s">
-        <v>488</v>
-      </c>
-      <c r="C1434" s="20">
-        <v>1263.1449007073684</v>
-      </c>
-      <c r="D1434" t="s">
-        <v>35</v>
-      </c>
-      <c r="E1434" s="13"/>
-      <c r="F1434" s="13"/>
-      <c r="G1434" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1434" s="13" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="1435" spans="1:9">
-      <c r="A1435" t="s">
-        <v>740</v>
-      </c>
-      <c r="B1435" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1435" s="36">
-        <v>18250</v>
-      </c>
-      <c r="D1435" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1435" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1435" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1435" t="s">
-        <v>733</v>
-      </c>
-    </row>
-    <row r="1436" spans="1:9">
-      <c r="A1436" t="s">
-        <v>742</v>
-      </c>
-      <c r="B1436" t="s">
-        <v>743</v>
-      </c>
-      <c r="C1436" s="20">
-        <v>-529.99999999999989</v>
-      </c>
-      <c r="D1436" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1436" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1436" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1436" t="s">
-        <v>744</v>
-      </c>
+      <c r="H1436" s="55"/>
     </row>
     <row r="1437" spans="1:9">
-      <c r="A1437" t="s">
-        <v>741</v>
-      </c>
-      <c r="B1437" t="s">
-        <v>461</v>
-      </c>
-      <c r="C1437" s="20">
-        <v>-18.25</v>
-      </c>
-      <c r="D1437" t="s">
-        <v>91</v>
-      </c>
-      <c r="G1437" t="s">
-        <v>134</v>
-      </c>
-      <c r="H1437" t="s">
-        <v>12</v>
-      </c>
+      <c r="A1437" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1437" s="13">
+        <v>1</v>
+      </c>
+      <c r="F1437" s="13"/>
+      <c r="H1437" s="13"/>
     </row>
     <row r="1438" spans="1:9">
-      <c r="A1438" s="49"/>
-      <c r="B1438" s="50"/>
-      <c r="C1438" s="49"/>
-      <c r="D1438" s="49"/>
-      <c r="E1438" s="49"/>
-      <c r="F1438" s="49"/>
-      <c r="G1438" s="49"/>
-      <c r="H1438" s="49"/>
-      <c r="I1438" s="49"/>
-    </row>
-    <row r="1439" spans="1:9" ht="15.6">
-      <c r="A1439" s="18" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1439" s="23" t="s">
-        <v>745</v>
-      </c>
+      <c r="A1438" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1438" s="13" t="s">
+        <v>736</v>
+      </c>
+      <c r="F1438" s="13"/>
+    </row>
+    <row r="1439" spans="1:9">
+      <c r="A1439" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1439" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1439" s="20"/>
     </row>
     <row r="1440" spans="1:9">
       <c r="A1440" s="24" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B1440" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1440" s="55"/>
+        <v>6</v>
+      </c>
     </row>
     <row r="1441" spans="1:9">
       <c r="A1441" s="24" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1441" s="13">
-        <v>1</v>
-      </c>
-      <c r="F1441" s="13"/>
-      <c r="H1441" s="13"/>
-    </row>
-    <row r="1442" spans="1:9">
-      <c r="A1442" s="24" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1442" s="13" t="s">
-        <v>746</v>
-      </c>
-      <c r="F1442" s="13"/>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="1442" spans="1:9" ht="15.6">
+      <c r="A1442" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1442" s="25"/>
+      <c r="D1442" s="26"/>
+      <c r="E1442" s="26"/>
+      <c r="F1442" s="26"/>
+      <c r="G1442" s="26"/>
+      <c r="H1442" s="26"/>
+      <c r="I1442" s="26"/>
     </row>
     <row r="1443" spans="1:9">
       <c r="A1443" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1443" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1443" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1443" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1443" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="F1443" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1443" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1443" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="B1443" s="13" t="s">
+      <c r="I1443" s="24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1444" spans="1:9">
+      <c r="A1444" s="13" t="s">
+        <v>735</v>
+      </c>
+      <c r="B1444" s="13" t="s">
+        <v>736</v>
+      </c>
+      <c r="C1444">
+        <v>1</v>
+      </c>
+      <c r="D1444" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1444" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1444" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="1445" spans="1:9">
+      <c r="A1445" s="13" t="s">
+        <v>758</v>
+      </c>
+      <c r="B1445" s="13" t="s">
+        <v>758</v>
+      </c>
+      <c r="C1445" s="20">
+        <v>1263.1449007073684</v>
+      </c>
+      <c r="D1445" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1445" s="13"/>
+      <c r="F1445" s="13"/>
+      <c r="G1445" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1445" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1446" spans="1:9">
+      <c r="A1446" t="s">
+        <v>737</v>
+      </c>
+      <c r="B1446" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1446" s="36">
+        <v>18250</v>
+      </c>
+      <c r="D1446" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1446" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1446" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1446" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="1447" spans="1:9">
+      <c r="A1447" t="s">
+        <v>756</v>
+      </c>
+      <c r="B1447" t="s">
+        <v>755</v>
+      </c>
+      <c r="C1447" s="20">
+        <v>-529.99999999999989</v>
+      </c>
+      <c r="D1447" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1447" t="s">
+        <v>134</v>
+      </c>
+      <c r="H1447" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1447" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="1448" spans="1:9">
+      <c r="A1448" t="s">
+        <v>738</v>
+      </c>
+      <c r="B1448" t="s">
+        <v>461</v>
+      </c>
+      <c r="C1448" s="20">
+        <v>-18.25</v>
+      </c>
+      <c r="D1448" t="s">
+        <v>91</v>
+      </c>
+      <c r="G1448" t="s">
+        <v>134</v>
+      </c>
+      <c r="H1448" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="1449" spans="1:9">
+      <c r="A1449" s="49"/>
+      <c r="B1449" s="50"/>
+      <c r="C1449" s="49"/>
+      <c r="D1449" s="49"/>
+      <c r="E1449" s="49"/>
+      <c r="F1449" s="49"/>
+      <c r="G1449" s="49"/>
+      <c r="H1449" s="49"/>
+      <c r="I1449" s="49"/>
+    </row>
+    <row r="1450" spans="1:9" ht="15.6">
+      <c r="A1450" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1450" s="23" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="1451" spans="1:9">
+      <c r="A1451" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1451" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1451" s="55"/>
+    </row>
+    <row r="1452" spans="1:9">
+      <c r="A1452" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1452" s="13">
+        <v>1</v>
+      </c>
+      <c r="F1452" s="13"/>
+      <c r="H1452" s="13"/>
+    </row>
+    <row r="1453" spans="1:9">
+      <c r="A1453" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1453" s="13" t="s">
+        <v>741</v>
+      </c>
+      <c r="F1453" s="13"/>
+    </row>
+    <row r="1454" spans="1:9">
+      <c r="A1454" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1454" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="F1443" s="20"/>
-    </row>
-    <row r="1444" spans="1:9">
-      <c r="A1444" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1444" s="13" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="1445" spans="1:9">
-      <c r="A1445" s="24" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="1446" spans="1:9" ht="15.6">
-      <c r="A1446" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1446" s="25"/>
-      <c r="D1446" s="26"/>
-      <c r="E1446" s="26"/>
-      <c r="F1446" s="26"/>
-      <c r="G1446" s="26"/>
-      <c r="H1446" s="26"/>
-      <c r="I1446" s="26"/>
-    </row>
-    <row r="1447" spans="1:9">
-      <c r="A1447" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1447" s="23" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1447" s="30" t="s">
-        <v>9</v>
-      </c>
-      <c r="D1447" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1447" s="24" t="s">
-        <v>81</v>
-      </c>
-      <c r="F1447" s="24" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1447" s="24" t="s">
-        <v>2</v>
-      </c>
-      <c r="H1447" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1447" s="24" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="1448" spans="1:9">
-      <c r="A1448" s="13" t="s">
-        <v>745</v>
-      </c>
-      <c r="B1448" s="13" t="s">
-        <v>746</v>
-      </c>
-      <c r="C1448">
-        <v>1</v>
-      </c>
-      <c r="D1448" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1448" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1448" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="1449" spans="1:9">
-      <c r="A1449" t="s">
-        <v>27</v>
-      </c>
-      <c r="B1449" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="C1449" s="65">
-        <v>191.99835548282837</v>
-      </c>
-      <c r="D1449" t="s">
-        <v>19</v>
-      </c>
-      <c r="G1449" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1449" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1449" t="s">
-        <v>753</v>
-      </c>
-    </row>
-    <row r="1450" spans="1:9">
-      <c r="A1450" t="s">
-        <v>747</v>
-      </c>
-      <c r="B1450" t="s">
-        <v>748</v>
-      </c>
-      <c r="C1450">
-        <v>0.34714397042969852</v>
-      </c>
-      <c r="D1450" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1450" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1450" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1450" t="s">
-        <v>753</v>
-      </c>
-    </row>
-    <row r="1451" spans="1:9">
-      <c r="A1451" t="s">
-        <v>749</v>
-      </c>
-      <c r="B1451" t="s">
-        <v>750</v>
-      </c>
-      <c r="C1451">
-        <v>0.10335917312661498</v>
-      </c>
-      <c r="D1451" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1451" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1451" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1451" t="s">
-        <v>753</v>
-      </c>
-    </row>
-    <row r="1452" spans="1:9">
-      <c r="A1452" t="s">
-        <v>751</v>
-      </c>
-      <c r="B1452" t="s">
-        <v>752</v>
-      </c>
-      <c r="C1452">
-        <v>7.7519379844961239E-2</v>
-      </c>
-      <c r="D1452" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1452" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1452" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1452" t="s">
-        <v>753</v>
-      </c>
-    </row>
-    <row r="1453" spans="1:9">
-      <c r="A1453" s="49"/>
-      <c r="B1453" s="50"/>
-      <c r="C1453" s="49"/>
-      <c r="D1453" s="49"/>
-      <c r="E1453" s="49"/>
-      <c r="F1453" s="49"/>
-      <c r="G1453" s="49"/>
-      <c r="H1453" s="49"/>
-      <c r="I1453" s="49"/>
-    </row>
-    <row r="1454" spans="1:9" ht="15.6">
-      <c r="A1454" s="18" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1454" s="23" t="s">
-        <v>754</v>
-      </c>
+      <c r="F1454" s="20"/>
     </row>
     <row r="1455" spans="1:9">
       <c r="A1455" s="24" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B1455" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1455" s="55"/>
+        <v>6</v>
+      </c>
     </row>
     <row r="1456" spans="1:9">
       <c r="A1456" s="24" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1456" s="13">
-        <v>1</v>
-      </c>
-      <c r="F1456" s="13"/>
-      <c r="H1456" s="13"/>
-    </row>
-    <row r="1457" spans="1:9">
-      <c r="A1457" s="24" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1457" s="13" t="s">
-        <v>755</v>
-      </c>
-      <c r="F1457" s="13"/>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="1457" spans="1:9" ht="15.6">
+      <c r="A1457" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1457" s="25"/>
+      <c r="D1457" s="26"/>
+      <c r="E1457" s="26"/>
+      <c r="F1457" s="26"/>
+      <c r="G1457" s="26"/>
+      <c r="H1457" s="26"/>
+      <c r="I1457" s="26"/>
     </row>
     <row r="1458" spans="1:9">
       <c r="A1458" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1458" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1458" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1458" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1458" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="F1458" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1458" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1458" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="B1458" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="F1458" s="20"/>
+      <c r="I1458" s="24" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="1459" spans="1:9">
-      <c r="A1459" s="24" t="s">
+      <c r="A1459" s="13" t="s">
+        <v>740</v>
+      </c>
+      <c r="B1459" s="13" t="s">
+        <v>741</v>
+      </c>
+      <c r="C1459">
+        <v>1</v>
+      </c>
+      <c r="D1459" t="s">
         <v>6</v>
       </c>
-      <c r="B1459" s="13" t="s">
+      <c r="G1459" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1459" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="1460" spans="1:9">
+      <c r="A1460" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1460" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1460" s="65">
+        <v>191.99835548282837</v>
+      </c>
+      <c r="D1460" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1460" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1460" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1460" t="s">
+        <v>748</v>
+      </c>
+    </row>
+    <row r="1461" spans="1:9">
+      <c r="A1461" t="s">
+        <v>742</v>
+      </c>
+      <c r="B1461" t="s">
+        <v>743</v>
+      </c>
+      <c r="C1461">
+        <v>0.34714397042969852</v>
+      </c>
+      <c r="D1461" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="1460" spans="1:9">
-      <c r="A1460" s="24" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="1461" spans="1:9" ht="15.6">
-      <c r="A1461" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1461" s="25"/>
-      <c r="D1461" s="26"/>
-      <c r="E1461" s="26"/>
-      <c r="F1461" s="26"/>
-      <c r="G1461" s="26"/>
-      <c r="H1461" s="26"/>
-      <c r="I1461" s="26"/>
+      <c r="G1461" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1461" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1461" t="s">
+        <v>748</v>
+      </c>
     </row>
     <row r="1462" spans="1:9">
-      <c r="A1462" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1462" s="23" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1462" s="30" t="s">
-        <v>9</v>
-      </c>
-      <c r="D1462" s="24" t="s">
+      <c r="A1462" t="s">
+        <v>744</v>
+      </c>
+      <c r="B1462" t="s">
+        <v>745</v>
+      </c>
+      <c r="C1462">
+        <v>0.10335917312661498</v>
+      </c>
+      <c r="D1462" t="s">
         <v>6</v>
       </c>
-      <c r="E1462" s="24" t="s">
-        <v>81</v>
-      </c>
-      <c r="F1462" s="24" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1462" s="24" t="s">
-        <v>2</v>
-      </c>
-      <c r="H1462" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1462" s="24" t="s">
-        <v>11</v>
+      <c r="G1462" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1462" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1462" t="s">
+        <v>748</v>
       </c>
     </row>
     <row r="1463" spans="1:9">
-      <c r="A1463" s="13" t="s">
-        <v>754</v>
-      </c>
-      <c r="B1463" s="13" t="s">
-        <v>755</v>
+      <c r="A1463" t="s">
+        <v>746</v>
+      </c>
+      <c r="B1463" t="s">
+        <v>747</v>
       </c>
       <c r="C1463">
-        <v>1</v>
+        <v>7.7519379844961239E-2</v>
       </c>
       <c r="D1463" t="s">
         <v>6</v>
       </c>
       <c r="G1463" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1463" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1463" t="s">
+        <v>748</v>
+      </c>
+    </row>
+    <row r="1464" spans="1:9">
+      <c r="A1464" s="49"/>
+      <c r="B1464" s="50"/>
+      <c r="C1464" s="49"/>
+      <c r="D1464" s="49"/>
+      <c r="E1464" s="49"/>
+      <c r="F1464" s="49"/>
+      <c r="G1464" s="49"/>
+      <c r="H1464" s="49"/>
+      <c r="I1464" s="49"/>
+    </row>
+    <row r="1465" spans="1:9" ht="15.6">
+      <c r="A1465" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1465" s="23" t="s">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="1466" spans="1:9">
+      <c r="A1466" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1466" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="H1463" t="s">
+      <c r="H1466" s="55"/>
+    </row>
+    <row r="1467" spans="1:9">
+      <c r="A1467" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1467" s="13">
+        <v>1</v>
+      </c>
+      <c r="F1467" s="13"/>
+      <c r="H1467" s="13"/>
+    </row>
+    <row r="1468" spans="1:9">
+      <c r="A1468" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1468" s="13" t="s">
+        <v>750</v>
+      </c>
+      <c r="F1468" s="13"/>
+    </row>
+    <row r="1469" spans="1:9">
+      <c r="A1469" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1469" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1469" s="20"/>
+    </row>
+    <row r="1470" spans="1:9">
+      <c r="A1470" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1470" s="13" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="1471" spans="1:9">
+      <c r="A1471" s="24" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="1472" spans="1:9" ht="15.6">
+      <c r="A1472" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1472" s="25"/>
+      <c r="D1472" s="26"/>
+      <c r="E1472" s="26"/>
+      <c r="F1472" s="26"/>
+      <c r="G1472" s="26"/>
+      <c r="H1472" s="26"/>
+      <c r="I1472" s="26"/>
+    </row>
+    <row r="1473" spans="1:9">
+      <c r="A1473" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1473" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1473" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1473" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1473" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="F1473" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1473" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1473" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1473" s="24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1474" spans="1:9">
+      <c r="A1474" s="13" t="s">
+        <v>749</v>
+      </c>
+      <c r="B1474" s="13" t="s">
+        <v>750</v>
+      </c>
+      <c r="C1474">
+        <v>1</v>
+      </c>
+      <c r="D1474" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1474" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1474" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="1464" spans="1:9">
-      <c r="A1464" s="13" t="s">
-        <v>758</v>
-      </c>
-      <c r="B1464" s="13" t="s">
-        <v>758</v>
-      </c>
-      <c r="C1464" s="65">
+    <row r="1475" spans="1:9">
+      <c r="A1475" s="13" t="s">
+        <v>753</v>
+      </c>
+      <c r="B1475" s="13" t="s">
+        <v>753</v>
+      </c>
+      <c r="C1475" s="65">
         <v>5025.4162915136185</v>
       </c>
-      <c r="D1464" t="s">
+      <c r="D1475" t="s">
         <v>486</v>
       </c>
-      <c r="G1464" t="s">
+      <c r="G1475" t="s">
         <v>28</v>
       </c>
-      <c r="H1464" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1464" t="s">
-        <v>757</v>
-      </c>
-    </row>
-    <row r="1465" spans="1:9">
-      <c r="B1465"/>
-    </row>
-    <row r="1466" spans="1:9">
-      <c r="B1466"/>
-    </row>
-    <row r="1467" spans="1:9">
-      <c r="B1467"/>
+      <c r="H1475" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1475" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="1476" spans="1:9">
+      <c r="B1476"/>
+    </row>
+    <row r="1477" spans="1:9">
+      <c r="B1477"/>
+    </row>
+    <row r="1478" spans="1:9">
+      <c r="B1478"/>
     </row>
   </sheetData>
   <phoneticPr fontId="14" type="noConversion"/>

</xml_diff>